<commit_message>
add user tests 13 passing, update docs and README
</commit_message>
<xml_diff>
--- a/test_cases/test_cases_phase1.xlsx
+++ b/test_cases/test_cases_phase1.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant Test Cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -58,7 +59,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -138,11 +139,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -170,6 +190,14 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -624,8 +652,8 @@
       <c r="C2" s="8" t="n"/>
       <c r="D2" s="8" t="n"/>
       <c r="E2" s="8" t="n"/>
-      <c r="F2" s="9" t="n"/>
-      <c r="G2" s="9" t="n"/>
+      <c r="F2" s="8" t="n"/>
+      <c r="G2" s="8" t="n"/>
       <c r="H2" s="8" t="n"/>
       <c r="I2" s="8" t="n"/>
       <c r="J2" s="8" t="n"/>
@@ -642,8 +670,8 @@
       <c r="C3" s="8" t="n"/>
       <c r="D3" s="8" t="n"/>
       <c r="E3" s="8" t="n"/>
-      <c r="F3" s="9" t="n"/>
-      <c r="G3" s="9" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="8" t="n"/>
       <c r="H3" s="8" t="n"/>
       <c r="I3" s="8" t="n"/>
       <c r="J3" s="8" t="n"/>
@@ -910,8 +938,8 @@
       <c r="C9" s="8" t="n"/>
       <c r="D9" s="8" t="n"/>
       <c r="E9" s="8" t="n"/>
-      <c r="F9" s="9" t="n"/>
-      <c r="G9" s="9" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="8" t="n"/>
       <c r="H9" s="8" t="n"/>
       <c r="I9" s="8" t="n"/>
       <c r="J9" s="8" t="n"/>
@@ -928,8 +956,8 @@
       <c r="C10" s="8" t="n"/>
       <c r="D10" s="8" t="n"/>
       <c r="E10" s="8" t="n"/>
-      <c r="F10" s="9" t="n"/>
-      <c r="G10" s="9" t="n"/>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="8" t="n"/>
       <c r="H10" s="8" t="n"/>
       <c r="I10" s="8" t="n"/>
       <c r="J10" s="8" t="n"/>
@@ -1146,8 +1174,8 @@
       <c r="C15" s="8" t="n"/>
       <c r="D15" s="8" t="n"/>
       <c r="E15" s="8" t="n"/>
-      <c r="F15" s="9" t="n"/>
-      <c r="G15" s="9" t="n"/>
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="8" t="n"/>
       <c r="H15" s="8" t="n"/>
       <c r="I15" s="8" t="n"/>
       <c r="J15" s="8" t="n"/>
@@ -1164,8 +1192,8 @@
       <c r="C16" s="8" t="n"/>
       <c r="D16" s="8" t="n"/>
       <c r="E16" s="8" t="n"/>
-      <c r="F16" s="9" t="n"/>
-      <c r="G16" s="9" t="n"/>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="8" t="n"/>
       <c r="H16" s="8" t="n"/>
       <c r="I16" s="8" t="n"/>
       <c r="J16" s="8" t="n"/>
@@ -1432,8 +1460,8 @@
       <c r="C22" s="8" t="n"/>
       <c r="D22" s="8" t="n"/>
       <c r="E22" s="8" t="n"/>
-      <c r="F22" s="9" t="n"/>
-      <c r="G22" s="9" t="n"/>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="8" t="n"/>
       <c r="H22" s="8" t="n"/>
       <c r="I22" s="8" t="n"/>
       <c r="J22" s="8" t="n"/>
@@ -1450,8 +1478,8 @@
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="8" t="n"/>
       <c r="E23" s="8" t="n"/>
-      <c r="F23" s="9" t="n"/>
-      <c r="G23" s="9" t="n"/>
+      <c r="F23" s="8" t="n"/>
+      <c r="G23" s="8" t="n"/>
       <c r="H23" s="8" t="n"/>
       <c r="I23" s="8" t="n"/>
       <c r="J23" s="8" t="n"/>
@@ -1618,8 +1646,8 @@
       <c r="C27" s="8" t="n"/>
       <c r="D27" s="8" t="n"/>
       <c r="E27" s="8" t="n"/>
-      <c r="F27" s="9" t="n"/>
-      <c r="G27" s="9" t="n"/>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="8" t="n"/>
       <c r="H27" s="8" t="n"/>
       <c r="I27" s="8" t="n"/>
       <c r="J27" s="8" t="n"/>
@@ -1636,8 +1664,8 @@
       <c r="C28" s="8" t="n"/>
       <c r="D28" s="8" t="n"/>
       <c r="E28" s="8" t="n"/>
-      <c r="F28" s="9" t="n"/>
-      <c r="G28" s="9" t="n"/>
+      <c r="F28" s="8" t="n"/>
+      <c r="G28" s="8" t="n"/>
       <c r="H28" s="8" t="n"/>
       <c r="I28" s="8" t="n"/>
       <c r="J28" s="8" t="n"/>
@@ -1854,8 +1882,8 @@
       <c r="C33" s="8" t="n"/>
       <c r="D33" s="8" t="n"/>
       <c r="E33" s="8" t="n"/>
-      <c r="F33" s="9" t="n"/>
-      <c r="G33" s="9" t="n"/>
+      <c r="F33" s="8" t="n"/>
+      <c r="G33" s="8" t="n"/>
       <c r="H33" s="8" t="n"/>
       <c r="I33" s="8" t="n"/>
       <c r="J33" s="8" t="n"/>
@@ -1872,8 +1900,8 @@
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="8" t="n"/>
       <c r="E34" s="8" t="n"/>
-      <c r="F34" s="9" t="n"/>
-      <c r="G34" s="9" t="n"/>
+      <c r="F34" s="8" t="n"/>
+      <c r="G34" s="8" t="n"/>
       <c r="H34" s="8" t="n"/>
       <c r="I34" s="8" t="n"/>
       <c r="J34" s="8" t="n"/>
@@ -2190,8 +2218,8 @@
       <c r="C41" s="8" t="n"/>
       <c r="D41" s="8" t="n"/>
       <c r="E41" s="8" t="n"/>
-      <c r="F41" s="9" t="n"/>
-      <c r="G41" s="9" t="n"/>
+      <c r="F41" s="8" t="n"/>
+      <c r="G41" s="8" t="n"/>
       <c r="H41" s="8" t="n"/>
       <c r="I41" s="8" t="n"/>
       <c r="J41" s="8" t="n"/>
@@ -2208,8 +2236,8 @@
       <c r="C42" s="8" t="n"/>
       <c r="D42" s="8" t="n"/>
       <c r="E42" s="8" t="n"/>
-      <c r="F42" s="9" t="n"/>
-      <c r="G42" s="9" t="n"/>
+      <c r="F42" s="8" t="n"/>
+      <c r="G42" s="8" t="n"/>
       <c r="H42" s="8" t="n"/>
       <c r="I42" s="8" t="n"/>
       <c r="J42" s="8" t="n"/>
@@ -2426,8 +2454,8 @@
       <c r="C47" s="8" t="n"/>
       <c r="D47" s="8" t="n"/>
       <c r="E47" s="8" t="n"/>
-      <c r="F47" s="9" t="n"/>
-      <c r="G47" s="9" t="n"/>
+      <c r="F47" s="8" t="n"/>
+      <c r="G47" s="8" t="n"/>
       <c r="H47" s="8" t="n"/>
       <c r="I47" s="8" t="n"/>
       <c r="J47" s="8" t="n"/>
@@ -2444,8 +2472,8 @@
       <c r="C48" s="8" t="n"/>
       <c r="D48" s="8" t="n"/>
       <c r="E48" s="8" t="n"/>
-      <c r="F48" s="9" t="n"/>
-      <c r="G48" s="9" t="n"/>
+      <c r="F48" s="8" t="n"/>
+      <c r="G48" s="8" t="n"/>
       <c r="H48" s="8" t="n"/>
       <c r="I48" s="8" t="n"/>
       <c r="J48" s="8" t="n"/>
@@ -2662,8 +2690,8 @@
       <c r="C53" s="8" t="n"/>
       <c r="D53" s="8" t="n"/>
       <c r="E53" s="8" t="n"/>
-      <c r="F53" s="9" t="n"/>
-      <c r="G53" s="9" t="n"/>
+      <c r="F53" s="8" t="n"/>
+      <c r="G53" s="8" t="n"/>
       <c r="H53" s="8" t="n"/>
       <c r="I53" s="8" t="n"/>
       <c r="J53" s="8" t="n"/>
@@ -2680,8 +2708,8 @@
       <c r="C54" s="8" t="n"/>
       <c r="D54" s="8" t="n"/>
       <c r="E54" s="8" t="n"/>
-      <c r="F54" s="9" t="n"/>
-      <c r="G54" s="9" t="n"/>
+      <c r="F54" s="8" t="n"/>
+      <c r="G54" s="8" t="n"/>
       <c r="H54" s="8" t="n"/>
       <c r="I54" s="8" t="n"/>
       <c r="J54" s="8" t="n"/>
@@ -2998,8 +3026,8 @@
       <c r="C61" s="8" t="n"/>
       <c r="D61" s="8" t="n"/>
       <c r="E61" s="8" t="n"/>
-      <c r="F61" s="9" t="n"/>
-      <c r="G61" s="9" t="n"/>
+      <c r="F61" s="8" t="n"/>
+      <c r="G61" s="8" t="n"/>
       <c r="H61" s="8" t="n"/>
       <c r="I61" s="8" t="n"/>
       <c r="J61" s="8" t="n"/>
@@ -3016,8 +3044,8 @@
       <c r="C62" s="8" t="n"/>
       <c r="D62" s="8" t="n"/>
       <c r="E62" s="8" t="n"/>
-      <c r="F62" s="9" t="n"/>
-      <c r="G62" s="9" t="n"/>
+      <c r="F62" s="8" t="n"/>
+      <c r="G62" s="8" t="n"/>
       <c r="H62" s="8" t="n"/>
       <c r="I62" s="8" t="n"/>
       <c r="J62" s="8" t="n"/>
@@ -3284,8 +3312,8 @@
       <c r="C68" s="8" t="n"/>
       <c r="D68" s="8" t="n"/>
       <c r="E68" s="8" t="n"/>
-      <c r="F68" s="9" t="n"/>
-      <c r="G68" s="9" t="n"/>
+      <c r="F68" s="8" t="n"/>
+      <c r="G68" s="8" t="n"/>
       <c r="H68" s="8" t="n"/>
       <c r="I68" s="8" t="n"/>
       <c r="J68" s="8" t="n"/>
@@ -3302,8 +3330,8 @@
       <c r="C69" s="8" t="n"/>
       <c r="D69" s="8" t="n"/>
       <c r="E69" s="8" t="n"/>
-      <c r="F69" s="9" t="n"/>
-      <c r="G69" s="9" t="n"/>
+      <c r="F69" s="8" t="n"/>
+      <c r="G69" s="8" t="n"/>
       <c r="H69" s="8" t="n"/>
       <c r="I69" s="8" t="n"/>
       <c r="J69" s="8" t="n"/>
@@ -3520,8 +3548,8 @@
       <c r="C74" s="8" t="n"/>
       <c r="D74" s="8" t="n"/>
       <c r="E74" s="8" t="n"/>
-      <c r="F74" s="9" t="n"/>
-      <c r="G74" s="9" t="n"/>
+      <c r="F74" s="8" t="n"/>
+      <c r="G74" s="8" t="n"/>
       <c r="H74" s="8" t="n"/>
       <c r="I74" s="8" t="n"/>
       <c r="J74" s="8" t="n"/>
@@ -3538,8 +3566,8 @@
       <c r="C75" s="8" t="n"/>
       <c r="D75" s="8" t="n"/>
       <c r="E75" s="8" t="n"/>
-      <c r="F75" s="9" t="n"/>
-      <c r="G75" s="9" t="n"/>
+      <c r="F75" s="8" t="n"/>
+      <c r="G75" s="8" t="n"/>
       <c r="H75" s="8" t="n"/>
       <c r="I75" s="8" t="n"/>
       <c r="J75" s="8" t="n"/>
@@ -3775,4 +3803,3340 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L82"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16.8" customWidth="1" min="1" max="1"/>
+    <col width="20.4" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="9.6" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="15.6" customWidth="1" min="10" max="10"/>
+    <col width="10.8" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Requirement Group</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>REQ_ID</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Step Description</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Layer</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Regulatory Reference</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Pass/Fail</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TC-2.1 - Positive User Creation by Program_administrator | User</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="n"/>
+      <c r="C2" s="11" t="n"/>
+      <c r="D2" s="11" t="n"/>
+      <c r="E2" s="11" t="n"/>
+      <c r="F2" s="11" t="n"/>
+      <c r="G2" s="11" t="n"/>
+      <c r="H2" s="11" t="n"/>
+      <c r="I2" s="11" t="n"/>
+      <c r="J2" s="11" t="n"/>
+      <c r="K2" s="12" t="n"/>
+      <c r="L2" s="13" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: No user with the chosen email exists in tenant-aaa-001. program_administrator role is authenticated with MFA enabled.</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
+      <c r="L3" s="13" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.1 Step 1</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Prepare a POST /users payload with tenant_id, first_name, last_name, email, and role.</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created. Response body contains user_id, email, role, and status="active". user_id is a non-null UUID assigned by the system.</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J4" s="16" t="n"/>
+      <c r="K4" s="16" t="n"/>
+      <c r="L4" s="16" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.1 Step 2</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /users using program_administrator headers.</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created. Response body contains user_id, email, role, and status="active". user_id is a non-null UUID assigned by the system.</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="n"/>
+      <c r="K5" s="16" t="n"/>
+      <c r="L5" s="16" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.1 Step 3</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Assert response status is 201 Created.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created. Response body contains user_id, email, role, and status="active". user_id is a non-null UUID assigned by the system.</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I6" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J6" s="16" t="n"/>
+      <c r="K6" s="16" t="n"/>
+      <c r="L6" s="16" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.1 Step 4</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body contains user_id, email, role, and status="active".</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created. Response body contains user_id, email, role, and status="active". user_id is a non-null UUID assigned by the system.</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="n"/>
+      <c r="K7" s="16" t="n"/>
+      <c r="L7" s="16" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.1 Step 5</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Assert user_id is a non-null UUID assigned by the system.</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created. Response body contains user_id, email, role, and status="active". user_id is a non-null UUID assigned by the system.</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J8" s="16" t="n"/>
+      <c r="K8" s="16" t="n"/>
+      <c r="L8" s="16" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TC-2.2 - Negative User Creation by Unauthorized Role Returns 403 | User</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="11" t="n"/>
+      <c r="I9" s="11" t="n"/>
+      <c r="J9" s="11" t="n"/>
+      <c r="K9" s="12" t="n"/>
+      <c r="L9" s="13" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: A user with role care_coordinator is authenticated. program_administrator role is not used.</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n"/>
+      <c r="C10" s="14" t="n"/>
+      <c r="D10" s="14" t="n"/>
+      <c r="E10" s="14" t="n"/>
+      <c r="F10" s="14" t="n"/>
+      <c r="G10" s="14" t="n"/>
+      <c r="H10" s="14" t="n"/>
+      <c r="I10" s="14" t="n"/>
+      <c r="J10" s="14" t="n"/>
+      <c r="K10" s="15" t="n"/>
+      <c r="L10" s="13" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.2 Step 1</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Prepare a POST /users payload with valid user fields (tenant_id, first_name, last_name, email, role).</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. Response body contains error_code="RBAC_DENIED". No record is created.</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="n"/>
+      <c r="K11" s="16" t="n"/>
+      <c r="L11" s="16" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.2 Step 2</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /users using care_coordinator headers.</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. Response body contains error_code="RBAC_DENIED". No record is created.</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="n"/>
+      <c r="K12" s="16" t="n"/>
+      <c r="L12" s="16" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.2 Step 3</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Assert response status is 403 Forbidden.</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. Response body contains error_code="RBAC_DENIED". No record is created.</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="n"/>
+      <c r="K13" s="16" t="n"/>
+      <c r="L13" s="16" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.2 Step 4</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body contains error_code="RBAC_DENIED".</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. Response body contains error_code="RBAC_DENIED". No record is created.</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H14" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J14" s="16" t="n"/>
+      <c r="K14" s="16" t="n"/>
+      <c r="L14" s="16" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TC-2.3 - Positive Login with Valid Credentials Returns 200 | User</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
+      <c r="H15" s="11" t="n"/>
+      <c r="I15" s="11" t="n"/>
+      <c r="J15" s="11" t="n"/>
+      <c r="K15" s="12" t="n"/>
+      <c r="L15" s="13" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: A user account exists with a known user_id and stored password_hash. The account is active.</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="n"/>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="14" t="n"/>
+      <c r="E16" s="14" t="n"/>
+      <c r="F16" s="14" t="n"/>
+      <c r="G16" s="14" t="n"/>
+      <c r="H16" s="14" t="n"/>
+      <c r="I16" s="14" t="n"/>
+      <c r="J16" s="14" t="n"/>
+      <c r="K16" s="15" t="n"/>
+      <c r="L16" s="13" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.3 Step 1</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Prepare a POST /login payload with the valid user_id and the correct password.</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK. Response body contains status="ok". No error is returned.</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="n"/>
+      <c r="K17" s="16" t="n"/>
+      <c r="L17" s="16" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.3 Step 2</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /login.</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK. Response body contains status="ok". No error is returned.</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I18" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J18" s="16" t="n"/>
+      <c r="K18" s="16" t="n"/>
+      <c r="L18" s="16" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.3 Step 3</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Assert response status is 200 OK.</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK. Response body contains status="ok". No error is returned.</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="n"/>
+      <c r="K19" s="16" t="n"/>
+      <c r="L19" s="16" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.3 Step 4</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body contains status="ok" and a success message.</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK. Response body contains status="ok". No error is returned.</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H20" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I20" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J20" s="16" t="n"/>
+      <c r="K20" s="16" t="n"/>
+      <c r="L20" s="16" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>TC-2.4 - Negative Login Wrong Password Returns 401 Error Message Does Not Reveal Which Credential Was Wrong | User</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
+      <c r="F21" s="11" t="n"/>
+      <c r="G21" s="11" t="n"/>
+      <c r="H21" s="11" t="n"/>
+      <c r="I21" s="11" t="n"/>
+      <c r="J21" s="11" t="n"/>
+      <c r="K21" s="12" t="n"/>
+      <c r="L21" s="13" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: A user account exists with a known user_id and stored password_hash. An incorrect non-empty password is used for the attempt.</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="n"/>
+      <c r="C22" s="14" t="n"/>
+      <c r="D22" s="14" t="n"/>
+      <c r="E22" s="14" t="n"/>
+      <c r="F22" s="14" t="n"/>
+      <c r="G22" s="14" t="n"/>
+      <c r="H22" s="14" t="n"/>
+      <c r="I22" s="14" t="n"/>
+      <c r="J22" s="14" t="n"/>
+      <c r="K22" s="15" t="n"/>
+      <c r="L22" s="13" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.4 Step 1</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Prepare a POST /login payload with a valid user_id and an incorrect non-empty password.</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized. Error message is generic and does not disclose whether the user_id or the password was wrong. No session token is returned.</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J23" s="16" t="n"/>
+      <c r="K23" s="16" t="n"/>
+      <c r="L23" s="16" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.4 Step 2</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /login.</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized. Error message is generic and does not disclose whether the user_id or the password was wrong. No session token is returned.</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H24" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J24" s="16" t="n"/>
+      <c r="K24" s="16" t="n"/>
+      <c r="L24" s="16" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.4 Step 3</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Assert response status is 401 Unauthorized.</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized. Error message is generic and does not disclose whether the user_id or the password was wrong. No session token is returned.</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J25" s="16" t="n"/>
+      <c r="K25" s="16" t="n"/>
+      <c r="L25" s="16" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.4 Step 4</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Assert the error message does not contain the words "email", "user_id", or "password".</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized. Error message is generic and does not disclose whether the user_id or the password was wrong. No session token is returned.</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H26" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J26" s="16" t="n"/>
+      <c r="K26" s="16" t="n"/>
+      <c r="L26" s="16" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.4 Step 5</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Assert no session token is present in the response body.</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized. Error message is generic and does not disclose whether the user_id or the password was wrong. No session token is returned.</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H27" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I27" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J27" s="16" t="n"/>
+      <c r="K27" s="16" t="n"/>
+      <c r="L27" s="16" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TC-2.5 - Duplicate Email Same Tenant Returns 409 USER_DUPLICATE_EMAIL | User</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="n"/>
+      <c r="C28" s="11" t="n"/>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="11" t="n"/>
+      <c r="G28" s="11" t="n"/>
+      <c r="H28" s="11" t="n"/>
+      <c r="I28" s="11" t="n"/>
+      <c r="J28" s="11" t="n"/>
+      <c r="K28" s="12" t="n"/>
+      <c r="L28" s="13" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: A user with email "existing@test.care" already exists in tenant-aaa-001. program_administrator role is authenticated.</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="n"/>
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="14" t="n"/>
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="14" t="n"/>
+      <c r="G29" s="14" t="n"/>
+      <c r="H29" s="14" t="n"/>
+      <c r="I29" s="14" t="n"/>
+      <c r="J29" s="14" t="n"/>
+      <c r="K29" s="15" t="n"/>
+      <c r="L29" s="13" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.5 Step 1</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>3.2.7</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Ensure a user with email "existing@test.care" already exists in tenant-aaa-001.</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 409 Conflict. Response body contains error_code="USER_DUPLICATE_EMAIL". No duplicate record is created.</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H30" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I30" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J30" s="16" t="n"/>
+      <c r="K30" s="16" t="n"/>
+      <c r="L30" s="16" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.5 Step 2</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>3.2.7</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /users with email="existing@test.care" in tenant-aaa-001 using program_administrator headers.</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 409 Conflict. Response body contains error_code="USER_DUPLICATE_EMAIL". No duplicate record is created.</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I31" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J31" s="16" t="n"/>
+      <c r="K31" s="16" t="n"/>
+      <c r="L31" s="16" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.5 Step 3</t>
+        </is>
+      </c>
+      <c r="B32" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>3.2.7</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Assert response status is 409 Conflict.</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 409 Conflict. Response body contains error_code="USER_DUPLICATE_EMAIL". No duplicate record is created.</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H32" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I32" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J32" s="16" t="n"/>
+      <c r="K32" s="16" t="n"/>
+      <c r="L32" s="16" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.5 Step 4</t>
+        </is>
+      </c>
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>3.2.7</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body contains error_code="USER_DUPLICATE_EMAIL".</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 409 Conflict. Response body contains error_code="USER_DUPLICATE_EMAIL". No duplicate record is created.</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H33" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I33" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J33" s="16" t="n"/>
+      <c r="K33" s="16" t="n"/>
+      <c r="L33" s="16" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TC-2.6 - Same Email Different Tenant Returns 201 | User</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="n"/>
+      <c r="C34" s="11" t="n"/>
+      <c r="D34" s="11" t="n"/>
+      <c r="E34" s="11" t="n"/>
+      <c r="F34" s="11" t="n"/>
+      <c r="G34" s="11" t="n"/>
+      <c r="H34" s="11" t="n"/>
+      <c r="I34" s="11" t="n"/>
+      <c r="J34" s="11" t="n"/>
+      <c r="K34" s="12" t="n"/>
+      <c r="L34" s="13" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: A user with email "shared@test.care" exists in tenant-aaa-001. program_administrator role is authenticated in tenant-bbb-002.</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="n"/>
+      <c r="C35" s="14" t="n"/>
+      <c r="D35" s="14" t="n"/>
+      <c r="E35" s="14" t="n"/>
+      <c r="F35" s="14" t="n"/>
+      <c r="G35" s="14" t="n"/>
+      <c r="H35" s="14" t="n"/>
+      <c r="I35" s="14" t="n"/>
+      <c r="J35" s="14" t="n"/>
+      <c r="K35" s="15" t="n"/>
+      <c r="L35" s="13" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.6 Step 1</t>
+        </is>
+      </c>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>3.2.7</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Create a user with email="shared@test.care" in tenant-aaa-001 via POST /users.</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created. Each user receives a distinct user_id. The same email may exist in different tenants without conflict.</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H36" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I36" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J36" s="16" t="n"/>
+      <c r="K36" s="16" t="n"/>
+      <c r="L36" s="16" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.6 Step 2</t>
+        </is>
+      </c>
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>3.2.7</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /users with the same email="shared@test.care" in tenant-bbb-002.</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created. Each user receives a distinct user_id. The same email may exist in different tenants without conflict.</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H37" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I37" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J37" s="16" t="n"/>
+      <c r="K37" s="16" t="n"/>
+      <c r="L37" s="16" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.6 Step 3</t>
+        </is>
+      </c>
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>3.2.7</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Assert response status is 201 Created.</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created. Each user receives a distinct user_id. The same email may exist in different tenants without conflict.</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H38" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I38" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J38" s="16" t="n"/>
+      <c r="K38" s="16" t="n"/>
+      <c r="L38" s="16" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.6 Step 4</t>
+        </is>
+      </c>
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C39" s="16" t="inlineStr">
+        <is>
+          <t>3.2.7</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Assert the returned user_id is distinct from the user_id created in tenant-aaa-001.</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created. Each user receives a distinct user_id. The same email may exist in different tenants without conflict.</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H39" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I39" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J39" s="16" t="n"/>
+      <c r="K39" s="16" t="n"/>
+      <c r="L39" s="16" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>TC-2.7 - Account Lockout After 5 Consecutive Failed Logins | User</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="n"/>
+      <c r="C40" s="11" t="n"/>
+      <c r="D40" s="11" t="n"/>
+      <c r="E40" s="11" t="n"/>
+      <c r="F40" s="11" t="n"/>
+      <c r="G40" s="11" t="n"/>
+      <c r="H40" s="11" t="n"/>
+      <c r="I40" s="11" t="n"/>
+      <c r="J40" s="11" t="n"/>
+      <c r="K40" s="12" t="n"/>
+      <c r="L40" s="13" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: An active user account exists with a known user_id and password_hash. The account has failed_login_count=0.</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="n"/>
+      <c r="C41" s="14" t="n"/>
+      <c r="D41" s="14" t="n"/>
+      <c r="E41" s="14" t="n"/>
+      <c r="F41" s="14" t="n"/>
+      <c r="G41" s="14" t="n"/>
+      <c r="H41" s="14" t="n"/>
+      <c r="I41" s="14" t="n"/>
+      <c r="J41" s="14" t="n"/>
+      <c r="K41" s="15" t="n"/>
+      <c r="L41" s="13" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.7 Step 1</t>
+        </is>
+      </c>
+      <c r="B42" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /login 5 times with the same user_id and an incorrect password.</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>The account locks after 5 consecutive failures. failed_login_count reaches 5 and locked_until is set to 30 minutes from now.</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H42" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I42" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J42" s="16" t="n"/>
+      <c r="K42" s="16" t="n"/>
+      <c r="L42" s="16" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.7 Step 2</t>
+        </is>
+      </c>
+      <c r="B43" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Assert each of the first 4 attempts returns HTTP 401 with error_code="AUTH_FAILURE".</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>The account locks after 5 consecutive failures. failed_login_count reaches 5 and locked_until is set to 30 minutes from now.</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H43" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I43" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J43" s="16" t="n"/>
+      <c r="K43" s="16" t="n"/>
+      <c r="L43" s="16" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.7 Step 3</t>
+        </is>
+      </c>
+      <c r="B44" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Assert the 5th attempt also returns HTTP 401.</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>The account locks after 5 consecutive failures. failed_login_count reaches 5 and locked_until is set to 30 minutes from now.</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H44" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I44" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J44" s="16" t="n"/>
+      <c r="K44" s="16" t="n"/>
+      <c r="L44" s="16" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.7 Step 4</t>
+        </is>
+      </c>
+      <c r="B45" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Assert locked_until is set to a timestamp approximately 30 minutes in the future.</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>The account locks after 5 consecutive failures. failed_login_count reaches 5 and locked_until is set to 30 minutes from now.</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H45" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I45" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J45" s="16" t="n"/>
+      <c r="K45" s="16" t="n"/>
+      <c r="L45" s="16" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>TC-2.8 - Locked User Login Attempt Returns 401 ACCOUNT_LOCKED | User</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="n"/>
+      <c r="C46" s="11" t="n"/>
+      <c r="D46" s="11" t="n"/>
+      <c r="E46" s="11" t="n"/>
+      <c r="F46" s="11" t="n"/>
+      <c r="G46" s="11" t="n"/>
+      <c r="H46" s="11" t="n"/>
+      <c r="I46" s="11" t="n"/>
+      <c r="J46" s="11" t="n"/>
+      <c r="K46" s="12" t="n"/>
+      <c r="L46" s="13" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: A user account has locked_until set to a future timestamp (account is currently locked).</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="n"/>
+      <c r="C47" s="14" t="n"/>
+      <c r="D47" s="14" t="n"/>
+      <c r="E47" s="14" t="n"/>
+      <c r="F47" s="14" t="n"/>
+      <c r="G47" s="14" t="n"/>
+      <c r="H47" s="14" t="n"/>
+      <c r="I47" s="14" t="n"/>
+      <c r="J47" s="14" t="n"/>
+      <c r="K47" s="15" t="n"/>
+      <c r="L47" s="13" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.8 Step 1</t>
+        </is>
+      </c>
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Confirm the target user account has locked_until in the future.</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized. Response contains error_code="ACCOUNT_LOCKED". No session is issued regardless of the password supplied.</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H48" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I48" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J48" s="16" t="n"/>
+      <c r="K48" s="16" t="n"/>
+      <c r="L48" s="16" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.8 Step 2</t>
+        </is>
+      </c>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /login with the correct password for the locked user.</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized. Response contains error_code="ACCOUNT_LOCKED". No session is issued regardless of the password supplied.</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H49" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I49" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J49" s="16" t="n"/>
+      <c r="K49" s="16" t="n"/>
+      <c r="L49" s="16" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.8 Step 3</t>
+        </is>
+      </c>
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Assert response status is 401 Unauthorized with error_code="ACCOUNT_LOCKED".</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized. Response contains error_code="ACCOUNT_LOCKED". No session is issued regardless of the password supplied.</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H50" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I50" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J50" s="16" t="n"/>
+      <c r="K50" s="16" t="n"/>
+      <c r="L50" s="16" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.8 Step 4</t>
+        </is>
+      </c>
+      <c r="B51" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Assert no session token or access token is returned.</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized. Response contains error_code="ACCOUNT_LOCKED". No session is issued regardless of the password supplied.</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(d)</t>
+        </is>
+      </c>
+      <c r="H51" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I51" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J51" s="16" t="n"/>
+      <c r="K51" s="16" t="n"/>
+      <c r="L51" s="16" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>TC-2.9 - User Deactivation (Soft Delete) Returns 200 and User Is Marked Inactive in DB | User</t>
+        </is>
+      </c>
+      <c r="B52" s="11" t="n"/>
+      <c r="C52" s="11" t="n"/>
+      <c r="D52" s="11" t="n"/>
+      <c r="E52" s="11" t="n"/>
+      <c r="F52" s="11" t="n"/>
+      <c r="G52" s="11" t="n"/>
+      <c r="H52" s="11" t="n"/>
+      <c r="I52" s="11" t="n"/>
+      <c r="J52" s="11" t="n"/>
+      <c r="K52" s="12" t="n"/>
+      <c r="L52" s="13" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: An active user exists. program_administrator role is authenticated. User records cannot be physically deleted per HIPAA retention rules.</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="n"/>
+      <c r="C53" s="14" t="n"/>
+      <c r="D53" s="14" t="n"/>
+      <c r="E53" s="14" t="n"/>
+      <c r="F53" s="14" t="n"/>
+      <c r="G53" s="14" t="n"/>
+      <c r="H53" s="14" t="n"/>
+      <c r="I53" s="14" t="n"/>
+      <c r="J53" s="14" t="n"/>
+      <c r="K53" s="15" t="n"/>
+      <c r="L53" s="13" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.9 Step 1</t>
+        </is>
+      </c>
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Create an active user via POST /users.</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK. User status is "inactive" in the response. The user record persists in the database with status="inactive" (user records are never physically deleted).</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H54" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I54" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J54" s="16" t="n"/>
+      <c r="K54" s="16" t="n"/>
+      <c r="L54" s="16" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.9 Step 2</t>
+        </is>
+      </c>
+      <c r="B55" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C55" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Send PATCH /users/{user_id} with status="inactive" using program_administrator headers.</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK. User status is "inactive" in the response. The user record persists in the database with status="inactive" (user records are never physically deleted).</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H55" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I55" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J55" s="16" t="n"/>
+      <c r="K55" s="16" t="n"/>
+      <c r="L55" s="16" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.9 Step 3</t>
+        </is>
+      </c>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C56" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Assert response status is 200 OK and response body status field equals "inactive".</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK. User status is "inactive" in the response. The user record persists in the database with status="inactive" (user records are never physically deleted).</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H56" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I56" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J56" s="16" t="n"/>
+      <c r="K56" s="16" t="n"/>
+      <c r="L56" s="16" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.9 Step 4</t>
+        </is>
+      </c>
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Assert the user record still exists in the database with status="inactive".</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK. User status is "inactive" in the response. The user record persists in the database with status="inactive" (user records are never physically deleted).</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H57" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I57" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J57" s="16" t="n"/>
+      <c r="K57" s="16" t="n"/>
+      <c r="L57" s="16" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>TC-2.10 - Audit Log on User Creation Has All Mandatory Fields | User</t>
+        </is>
+      </c>
+      <c r="B58" s="11" t="n"/>
+      <c r="C58" s="11" t="n"/>
+      <c r="D58" s="11" t="n"/>
+      <c r="E58" s="11" t="n"/>
+      <c r="F58" s="11" t="n"/>
+      <c r="G58" s="11" t="n"/>
+      <c r="H58" s="11" t="n"/>
+      <c r="I58" s="11" t="n"/>
+      <c r="J58" s="11" t="n"/>
+      <c r="K58" s="12" t="n"/>
+      <c r="L58" s="13" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: program_administrator role is authenticated. compliance_officer role is available to query audit logs.</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="n"/>
+      <c r="C59" s="14" t="n"/>
+      <c r="D59" s="14" t="n"/>
+      <c r="E59" s="14" t="n"/>
+      <c r="F59" s="14" t="n"/>
+      <c r="G59" s="14" t="n"/>
+      <c r="H59" s="14" t="n"/>
+      <c r="I59" s="14" t="n"/>
+      <c r="J59" s="14" t="n"/>
+      <c r="K59" s="15" t="n"/>
+      <c r="L59" s="13" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.10 Step 1</t>
+        </is>
+      </c>
+      <c r="B60" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C60" s="16" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Create a user via POST /users with program_administrator credentials.</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>PHI_WRITE audit event is created. All 11 mandatory fields are non-null. data_affected contains only field names, not PHI values.</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(b); SOC 2 CC7.2</t>
+        </is>
+      </c>
+      <c r="H60" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I60" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J60" s="16" t="n"/>
+      <c r="K60" s="16" t="n"/>
+      <c r="L60" s="16" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.10 Step 2</t>
+        </is>
+      </c>
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C61" s="16" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Query GET /audit-logs with resource_type=User and the newly created user_id, using compliance_officer headers.</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>PHI_WRITE audit event is created. All 11 mandatory fields are non-null. data_affected contains only field names, not PHI values.</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(b); SOC 2 CC7.2</t>
+        </is>
+      </c>
+      <c r="H61" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I61" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J61" s="16" t="n"/>
+      <c r="K61" s="16" t="n"/>
+      <c r="L61" s="16" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.10 Step 3</t>
+        </is>
+      </c>
+      <c r="B62" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C62" s="16" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Assert a PHI_WRITE audit event exists for the user creation.</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>PHI_WRITE audit event is created. All 11 mandatory fields are non-null. data_affected contains only field names, not PHI values.</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(b); SOC 2 CC7.2</t>
+        </is>
+      </c>
+      <c r="H62" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I62" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J62" s="16" t="n"/>
+      <c r="K62" s="16" t="n"/>
+      <c r="L62" s="16" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.10 Step 4</t>
+        </is>
+      </c>
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>Assert all 11 mandatory fields (timestamp, user_id, tenant_id, session_id, action_type, resource_type, resource_id, data_affected, source_ip, outcome, layer) are present and non-null.</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>PHI_WRITE audit event is created. All 11 mandatory fields are non-null. data_affected contains only field names, not PHI values.</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(b); SOC 2 CC7.2</t>
+        </is>
+      </c>
+      <c r="H63" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I63" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J63" s="16" t="n"/>
+      <c r="K63" s="16" t="n"/>
+      <c r="L63" s="16" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.10 Step 5</t>
+        </is>
+      </c>
+      <c r="B64" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C64" s="16" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>Assert data_affected contains only field names and not any personal information values.</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>PHI_WRITE audit event is created. All 11 mandatory fields are non-null. data_affected contains only field names, not PHI values.</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(b); SOC 2 CC7.2</t>
+        </is>
+      </c>
+      <c r="H64" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I64" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J64" s="16" t="n"/>
+      <c r="K64" s="16" t="n"/>
+      <c r="L64" s="16" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>TC-2.11 - Missing Required Field on User Creation Returns 400 with Field Name | User</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="n"/>
+      <c r="C65" s="11" t="n"/>
+      <c r="D65" s="11" t="n"/>
+      <c r="E65" s="11" t="n"/>
+      <c r="F65" s="11" t="n"/>
+      <c r="G65" s="11" t="n"/>
+      <c r="H65" s="11" t="n"/>
+      <c r="I65" s="11" t="n"/>
+      <c r="J65" s="11" t="n"/>
+      <c r="K65" s="12" t="n"/>
+      <c r="L65" s="13" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: program_administrator role is authenticated. The POST /users payload intentionally omits the required email field.</t>
+        </is>
+      </c>
+      <c r="B66" s="14" t="n"/>
+      <c r="C66" s="14" t="n"/>
+      <c r="D66" s="14" t="n"/>
+      <c r="E66" s="14" t="n"/>
+      <c r="F66" s="14" t="n"/>
+      <c r="G66" s="14" t="n"/>
+      <c r="H66" s="14" t="n"/>
+      <c r="I66" s="14" t="n"/>
+      <c r="J66" s="14" t="n"/>
+      <c r="K66" s="15" t="n"/>
+      <c r="L66" s="13" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.11 Step 1</t>
+        </is>
+      </c>
+      <c r="B67" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C67" s="16" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Prepare a POST /users payload omitting the required email field.</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 or 422. The response body explicitly names "email" as the missing or invalid field.</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H67" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I67" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J67" s="16" t="n"/>
+      <c r="K67" s="16" t="n"/>
+      <c r="L67" s="16" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.11 Step 2</t>
+        </is>
+      </c>
+      <c r="B68" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C68" s="16" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /users using program_administrator headers.</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 or 422. The response body explicitly names "email" as the missing or invalid field.</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H68" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I68" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J68" s="16" t="n"/>
+      <c r="K68" s="16" t="n"/>
+      <c r="L68" s="16" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.11 Step 3</t>
+        </is>
+      </c>
+      <c r="B69" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C69" s="16" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Assert response status is 400 or 422.</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 or 422. The response body explicitly names "email" as the missing or invalid field.</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H69" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I69" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J69" s="16" t="n"/>
+      <c r="K69" s="16" t="n"/>
+      <c r="L69" s="16" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.11 Step 4</t>
+        </is>
+      </c>
+      <c r="B70" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C70" s="16" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>Assert the response body contains the string "email" identifying the missing required field.</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 or 422. The response body explicitly names "email" as the missing or invalid field.</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3)</t>
+        </is>
+      </c>
+      <c r="H70" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I70" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J70" s="16" t="n"/>
+      <c r="K70" s="16" t="n"/>
+      <c r="L70" s="16" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>TC-2.12 - billing_specialist Attempts to Create Participant Returns 403 | User</t>
+        </is>
+      </c>
+      <c r="B71" s="11" t="n"/>
+      <c r="C71" s="11" t="n"/>
+      <c r="D71" s="11" t="n"/>
+      <c r="E71" s="11" t="n"/>
+      <c r="F71" s="11" t="n"/>
+      <c r="G71" s="11" t="n"/>
+      <c r="H71" s="11" t="n"/>
+      <c r="I71" s="11" t="n"/>
+      <c r="J71" s="11" t="n"/>
+      <c r="K71" s="12" t="n"/>
+      <c r="L71" s="13" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: billing_specialist role is authenticated. The POST /participants endpoint requires program_administrator, care_coordinator, nurse_medication_aide, billing_specialist, or compliance_officer role with write permission.</t>
+        </is>
+      </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
+      <c r="L72" s="13" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.12 Step 1</t>
+        </is>
+      </c>
+      <c r="B73" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C73" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>Prepare a POST /participants payload with valid tenant_id, first_name, last_name, date_of_birth, and enrollment_date.</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. Response body contains error_code="RBAC_DENIED". No participant record is created.</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(4)</t>
+        </is>
+      </c>
+      <c r="H73" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I73" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J73" s="16" t="n"/>
+      <c r="K73" s="16" t="n"/>
+      <c r="L73" s="16" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.12 Step 2</t>
+        </is>
+      </c>
+      <c r="B74" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C74" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /participants using billing_specialist headers.</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. Response body contains error_code="RBAC_DENIED". No participant record is created.</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(4)</t>
+        </is>
+      </c>
+      <c r="H74" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I74" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J74" s="16" t="n"/>
+      <c r="K74" s="16" t="n"/>
+      <c r="L74" s="16" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.12 Step 3</t>
+        </is>
+      </c>
+      <c r="B75" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C75" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>Assert response status is 403 Forbidden.</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. Response body contains error_code="RBAC_DENIED". No participant record is created.</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(4)</t>
+        </is>
+      </c>
+      <c r="H75" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I75" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J75" s="16" t="n"/>
+      <c r="K75" s="16" t="n"/>
+      <c r="L75" s="16" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.12 Step 4</t>
+        </is>
+      </c>
+      <c r="B76" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C76" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body contains error_code="RBAC_DENIED".</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. Response body contains error_code="RBAC_DENIED". No participant record is created.</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(4)</t>
+        </is>
+      </c>
+      <c r="H76" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I76" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J76" s="16" t="n"/>
+      <c r="K76" s="16" t="n"/>
+      <c r="L76" s="16" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>TC-2.13 - nurse_medication_aide Attempts to Create Claim Returns 403 | User</t>
+        </is>
+      </c>
+      <c r="B77" s="11" t="n"/>
+      <c r="C77" s="11" t="n"/>
+      <c r="D77" s="11" t="n"/>
+      <c r="E77" s="11" t="n"/>
+      <c r="F77" s="11" t="n"/>
+      <c r="G77" s="11" t="n"/>
+      <c r="H77" s="11" t="n"/>
+      <c r="I77" s="11" t="n"/>
+      <c r="J77" s="11" t="n"/>
+      <c r="K77" s="12" t="n"/>
+      <c r="L77" s="13" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: nurse_medication_aide role is authenticated. POST /claims requires billing_specialist or program_administrator role.</t>
+        </is>
+      </c>
+      <c r="B78" s="14" t="n"/>
+      <c r="C78" s="14" t="n"/>
+      <c r="D78" s="14" t="n"/>
+      <c r="E78" s="14" t="n"/>
+      <c r="F78" s="14" t="n"/>
+      <c r="G78" s="14" t="n"/>
+      <c r="H78" s="14" t="n"/>
+      <c r="I78" s="14" t="n"/>
+      <c r="J78" s="14" t="n"/>
+      <c r="K78" s="15" t="n"/>
+      <c r="L78" s="13" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.13 Step 1</t>
+        </is>
+      </c>
+      <c r="B79" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C79" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>Prepare a POST /claims payload with valid participant_id, attendance_ids, payer_type, procedure_code, and date_of_service_start.</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. Response body contains error_code="RBAC_DENIED". No claim record is created.</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(4)</t>
+        </is>
+      </c>
+      <c r="H79" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I79" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J79" s="16" t="n"/>
+      <c r="K79" s="16" t="n"/>
+      <c r="L79" s="16" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.13 Step 2</t>
+        </is>
+      </c>
+      <c r="B80" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C80" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /claims using nurse_medication_aide headers.</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. Response body contains error_code="RBAC_DENIED". No claim record is created.</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(4)</t>
+        </is>
+      </c>
+      <c r="H80" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I80" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J80" s="16" t="n"/>
+      <c r="K80" s="16" t="n"/>
+      <c r="L80" s="16" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.13 Step 3</t>
+        </is>
+      </c>
+      <c r="B81" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C81" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>Assert response status is 403 Forbidden.</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. Response body contains error_code="RBAC_DENIED". No claim record is created.</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(4)</t>
+        </is>
+      </c>
+      <c r="H81" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I81" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J81" s="16" t="n"/>
+      <c r="K81" s="16" t="n"/>
+      <c r="L81" s="16" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="16" t="inlineStr">
+        <is>
+          <t>TC-2.13 Step 4</t>
+        </is>
+      </c>
+      <c r="B82" s="16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C82" s="16" t="inlineStr">
+        <is>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body contains error_code="RBAC_DENIED".</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. Response body contains error_code="RBAC_DENIED". No claim record is created.</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(4)</t>
+        </is>
+      </c>
+      <c r="H82" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I82" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J82" s="16" t="n"/>
+      <c r="K82" s="16" t="n"/>
+      <c r="L82" s="16" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="26">
+    <mergeCell ref="A58:K58"/>
+    <mergeCell ref="A34:K34"/>
+    <mergeCell ref="A77:K77"/>
+    <mergeCell ref="A15:K15"/>
+    <mergeCell ref="A59:K59"/>
+    <mergeCell ref="A78:K78"/>
+    <mergeCell ref="A65:K65"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A46:K46"/>
+    <mergeCell ref="A66:K66"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A21:K21"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A71:K71"/>
+    <mergeCell ref="A47:K47"/>
+    <mergeCell ref="A22:K22"/>
+    <mergeCell ref="A53:K53"/>
+    <mergeCell ref="A35:K35"/>
+    <mergeCell ref="A72:K72"/>
+    <mergeCell ref="A29:K29"/>
+    <mergeCell ref="A52:K52"/>
+    <mergeCell ref="A10:K10"/>
+    <mergeCell ref="A28:K28"/>
+    <mergeCell ref="A40:K40"/>
+    <mergeCell ref="A9:K9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add test_claim.py TC-4.1 through TC-4.15, fix mock backend compliance, update README
</commit_message>
<xml_diff>
--- a/test_cases/test_cases_phase1.xlsx
+++ b/test_cases/test_cases_phase1.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant Test Cases" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claim" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10157,4 +10158,4716 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L112"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16.8" customWidth="1" min="1" max="1"/>
+    <col width="20.4" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="9.6" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="15.6" customWidth="1" min="10" max="10"/>
+    <col width="10.8" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Requirement Group</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>REQ_ID</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Step Description</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Layer</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Regulatory Reference</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Pass/Fail</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TC-4.1 - POST /claims with Duplicate claim_reference_number Returns 409 CLAIM_DUPLICATE_REFERENCE; DB Confirms Exactly One Claim with That Reference | Claim</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="n"/>
+      <c r="C2" s="8" t="n"/>
+      <c r="D2" s="8" t="n"/>
+      <c r="E2" s="8" t="n"/>
+      <c r="F2" s="8" t="n"/>
+      <c r="G2" s="8" t="n"/>
+      <c r="H2" s="8" t="n"/>
+      <c r="I2" s="8" t="n"/>
+      <c r="J2" s="8" t="n"/>
+      <c r="K2" s="10" t="n"/>
+      <c r="L2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: billing_specialist is authenticated in tenant-aaa-001 (X-User-Status: active, X-User-MFA: true). A claim record with claim_reference_number="MCD-20260301-REF001" is pre-seeded directly in the DB for tenant-aaa-001. A confirmed attendance record att-001 exists for participant P1 in tenant-aaa-001.</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="n"/>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="8" t="n"/>
+      <c r="H3" s="8" t="n"/>
+      <c r="I3" s="8" t="n"/>
+      <c r="J3" s="8" t="n"/>
+      <c r="K3" s="10" t="n"/>
+      <c r="L3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.1 Step 1</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Verify pre-condition: SELECT COUNT(*) FROM claim WHERE claim_reference_number='MCD-20260301-REF001' AND tenant_id='tenant-aaa-001'. Assert count = 1.</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Count = 1. Pre-seeded claim with reference number 'MCD-20260301-REF001' confirmed present before the POST attempt.</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J4" s="16" t="n"/>
+      <c r="K4" s="16" t="n"/>
+      <c r="L4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.1 Step 2</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /claims with billing_specialist headers. Body: {"tenant_id":"tenant-aaa-001","participant_id":"&lt;P1_id&gt;","attendance_ids":["&lt;att-001_id&gt;"],"payer_type":"medicaid","procedure_code":"T2029","date_of_service_start":"2026-03-01"}. Use a test fixture to ensure the server generates claim_reference_number='MCD-20260301-REF001' (same as the pre-seeded record).</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 409 Conflict. Server detects the duplicate claim_reference_number. Response body contains error_code="CLAIM_DUPLICATE_REFERENCE".</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="n"/>
+      <c r="K5" s="16" t="n"/>
+      <c r="L5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.1 Step 3</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Assert response HTTP status code equals 409.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 409 Conflict.</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I6" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J6" s="16" t="n"/>
+      <c r="K6" s="16" t="n"/>
+      <c r="L6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.1 Step 4</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body detail.error_code = "CLAIM_DUPLICATE_REFERENCE" and message describes the reference number collision.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>detail.error_code = "CLAIM_DUPLICATE_REFERENCE". Message indicates the reference number could not be made unique.</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="n"/>
+      <c r="K7" s="16" t="n"/>
+      <c r="L7" s="4" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.1 Step 5</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT COUNT(*) FROM claim WHERE claim_reference_number='MCD-20260301-REF001' AND tenant_id='tenant-aaa-001'. Assert count = 1.</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Count = 1. Exactly one claim exists with this reference number. No duplicate record was created by the failed POST attempt.</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J8" s="16" t="n"/>
+      <c r="K8" s="16" t="n"/>
+      <c r="L8" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TC-4.2 - Composite Duplicate participant_id + date_of_service_start + procedure_code + payer_type Returns 409 CLAIM_DUPLICATE | Claim</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="8" t="n"/>
+      <c r="H9" s="8" t="n"/>
+      <c r="I9" s="8" t="n"/>
+      <c r="J9" s="8" t="n"/>
+      <c r="K9" s="10" t="n"/>
+      <c r="L9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: A claim record already exists in tenant-aaa-001 with participant_id=P1, date_of_service_start="2026-03-01", procedure_code="T2029", payer_type="medicaid", claim_status="draft". A second confirmed attendance record att-002 exists for P1 in tenant-aaa-001. billing_specialist is authenticated.</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="8" t="n"/>
+      <c r="H10" s="8" t="n"/>
+      <c r="I10" s="8" t="n"/>
+      <c r="J10" s="8" t="n"/>
+      <c r="K10" s="10" t="n"/>
+      <c r="L10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.2 Step 1</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Confirm via DB query: SELECT COUNT(*) FROM claim WHERE tenant_id="tenant-aaa-001" AND participant_id="&lt;P1_id&gt;" AND date_of_service_start="2026-03-01" AND procedure_code="T2029" AND payer_type="medicaid". Assert count = 1.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Exactly one claim record matching the composite key exists in the DB.</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="n"/>
+      <c r="K11" s="16" t="n"/>
+      <c r="L11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.2 Step 2</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /claims with billing_specialist headers. Body: {"tenant_id":"tenant-aaa-001","participant_id":"&lt;P1_id&gt;","attendance_ids":["&lt;att-002_id&gt;"],"payer_type":"medicaid","procedure_code":"T2029","date_of_service_start":"2026-03-01"}.</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 409 Conflict. error_code="CLAIM_DUPLICATE". No new claim is created.</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="n"/>
+      <c r="K12" s="16" t="n"/>
+      <c r="L12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.2 Step 3</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Assert response status code equals 409.</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 409 Conflict.</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="n"/>
+      <c r="K13" s="16" t="n"/>
+      <c r="L13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.2 Step 4</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body detail.error_code = "CLAIM_DUPLICATE". Assert message references the duplicate combination (participant, date of service, procedure, payer).</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>error_code = "CLAIM_DUPLICATE". Message describes the composite key collision.</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H14" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J14" s="16" t="n"/>
+      <c r="K14" s="16" t="n"/>
+      <c r="L14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.2 Step 5</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT COUNT(*) FROM claim WHERE tenant_id="tenant-aaa-001" AND participant_id="&lt;P1_id&gt;" AND date_of_service_start="2026-03-01" AND procedure_code="T2029" AND payer_type="medicaid". Assert count still equals 1.</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Count = 1. Only the original claim exists. No duplicate record was created.</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="n"/>
+      <c r="K15" s="16" t="n"/>
+      <c r="L15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TC-4.3 - Unauthorized Roles POST /claims Returns 403 RBAC_DENIED; DB Claim Count Unchanged | Claim</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="8" t="n"/>
+      <c r="H16" s="8" t="n"/>
+      <c r="I16" s="8" t="n"/>
+      <c r="J16" s="8" t="n"/>
+      <c r="K16" s="10" t="n"/>
+      <c r="L16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: Four user accounts exist in tenant-aaa-001 with roles care_coordinator, nurse_medication_aide, physician, participant_family. All have X-User-Status: active, X-User-MFA: true. A confirmed attendance record att-003 exists for participant P1. Initial claim count in tenant-aaa-001 is recorded as N.</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="8" t="n"/>
+      <c r="H17" s="8" t="n"/>
+      <c r="I17" s="8" t="n"/>
+      <c r="J17" s="8" t="n"/>
+      <c r="K17" s="10" t="n"/>
+      <c r="L17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.3 Step 1</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /claims with X-User-Role: care_coordinator headers for tenant-aaa-001. Body: valid claim payload referencing att-003 with required fields. Assert response status equals 403.</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. error_code="RBAC_DENIED". care_coordinator is not permitted to create claims.</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3); CMS Medicaid/Medicare</t>
+        </is>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I18" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J18" s="16" t="n"/>
+      <c r="K18" s="16" t="n"/>
+      <c r="L18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.3 Step 2</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /claims with X-User-Role: nurse_medication_aide headers. Body: same valid payload. Assert response status equals 403.</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. error_code="RBAC_DENIED". nurse_medication_aide is not permitted to create claims.</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3); CMS Medicaid/Medicare</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="n"/>
+      <c r="K19" s="16" t="n"/>
+      <c r="L19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.3 Step 3</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /claims with X-User-Role: physician headers. Body: same valid payload. Assert response status equals 403.</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. error_code="RBAC_DENIED". physician is not permitted to create claims.</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3); CMS Medicaid/Medicare</t>
+        </is>
+      </c>
+      <c r="H20" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I20" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J20" s="16" t="n"/>
+      <c r="K20" s="16" t="n"/>
+      <c r="L20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.3 Step 4</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Send POST /claims with X-User-Role: participant_family headers. Body: same valid payload. Assert response status equals 403.</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden. error_code="RBAC_DENIED". participant_family is not permitted to create claims.</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3); CMS Medicaid/Medicare</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="n"/>
+      <c r="K21" s="16" t="n"/>
+      <c r="L21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.3 Step 5</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Assert all four responses have status 403 and detail.error_code="RBAC_DENIED". Confirm no response returned 201.</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>All 4 unauthorized roles receive HTTP 403 RBAC_DENIED. Zero successful claim creations.</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3); CMS Medicaid/Medicare</t>
+        </is>
+      </c>
+      <c r="H22" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I22" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J22" s="16" t="n"/>
+      <c r="K22" s="16" t="n"/>
+      <c r="L22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.3 Step 6</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT COUNT(*) FROM claim WHERE tenant_id="tenant-aaa-001". Assert count still equals N.</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>DB claim count = N. No new claims created by any unauthorized role attempt.</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.308(a)(3); CMS Medicaid/Medicare</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J23" s="16" t="n"/>
+      <c r="K23" s="16" t="n"/>
+      <c r="L23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TC-4.4 - PATCH Submitted Claim Non-Status Field Returns 422 CLAIM_STATUS_IMMUTABLE; Status Transition Returns 200; PATCH Paid Claim Returns 422; DB Status Unchanged After Rejected Edits | Claim</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="8" t="n"/>
+      <c r="H24" s="8" t="n"/>
+      <c r="I24" s="8" t="n"/>
+      <c r="J24" s="8" t="n"/>
+      <c r="K24" s="10" t="n"/>
+      <c r="L24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: Claim A (C_A) exists in tenant-aaa-001 with claim_status="submitted" and version=1. Claim B (C_B) exists with claim_status="paid" and version=2. billing_specialist is authenticated.</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="8" t="n"/>
+      <c r="G25" s="8" t="n"/>
+      <c r="H25" s="8" t="n"/>
+      <c r="I25" s="8" t="n"/>
+      <c r="J25" s="8" t="n"/>
+      <c r="K25" s="10" t="n"/>
+      <c r="L25" s="3" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.4 Step 1</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>GET /claims/&lt;C_A_id&gt; with billing_specialist headers. Confirm claim_status="submitted" and capture version=1.</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200. claim_status="submitted", version=1.</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H26" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J26" s="16" t="n"/>
+      <c r="K26" s="16" t="n"/>
+      <c r="L26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.4 Step 2</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /claims/&lt;C_A_id&gt; with body {"version":1,"rejection_reason":"Test edit on submitted claim"}. Assert response status equals 422.</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity. error_code="CLAIM_STATUS_IMMUTABLE". Non-status fields cannot be modified on a submitted claim.</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H27" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I27" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J27" s="16" t="n"/>
+      <c r="K27" s="16" t="n"/>
+      <c r="L27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.4 Step 3</t>
+        </is>
+      </c>
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT claim_status, version FROM claim WHERE claim_id="&lt;C_A_id&gt;". Assert claim_status="submitted" and version=1 (unchanged after the rejected PATCH).</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>claim_status="submitted", version=1. No changes applied by the rejected request.</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H28" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I28" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J28" s="16" t="n"/>
+      <c r="K28" s="16" t="n"/>
+      <c r="L28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.4 Step 4</t>
+        </is>
+      </c>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /claims/&lt;C_A_id&gt; with body {"version":1,"claim_status":"accepted"}. Assert response status equals 200. Assert response body claim_status="accepted" and version=2.</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK. claim_status="accepted", version=2. Status transition from submitted to accepted succeeds.</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H29" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I29" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J29" s="16" t="n"/>
+      <c r="K29" s="16" t="n"/>
+      <c r="L29" s="4" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.4 Step 5</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>GET /claims/&lt;C_B_id&gt; to confirm claim_status="paid" and version=2.</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200. claim_status="paid", version=2.</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H30" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I30" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J30" s="16" t="n"/>
+      <c r="K30" s="16" t="n"/>
+      <c r="L30" s="4" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.4 Step 6</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /claims/&lt;C_B_id&gt; with body {"version":2,"rejection_reason":"Attempt to modify paid claim"}. Assert response status equals 422.</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity. error_code="CLAIM_STATUS_IMMUTABLE". Paid claim is fully immutable.</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I31" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J31" s="16" t="n"/>
+      <c r="K31" s="16" t="n"/>
+      <c r="L31" s="4" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.4 Step 7</t>
+        </is>
+      </c>
+      <c r="B32" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT claim_status, version FROM claim WHERE claim_id="&lt;C_B_id&gt;". Assert claim_status="paid" and version=2.</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>claim_status="paid", version=2. No modifications applied to the paid claim.</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H32" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I32" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J32" s="16" t="n"/>
+      <c r="K32" s="16" t="n"/>
+      <c r="L32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TC-4.5 - POST /claims References Non-Confirmed Attendance Returns 422; Cross-Tenant Returns 422 or 404; Confirmed Attendance Returns 201 and Sets Attendance Status Billed | Claim</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="8" t="n"/>
+      <c r="G33" s="8" t="n"/>
+      <c r="H33" s="8" t="n"/>
+      <c r="I33" s="8" t="n"/>
+      <c r="J33" s="8" t="n"/>
+      <c r="K33" s="10" t="n"/>
+      <c r="L33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: Three attendance records exist in tenant-aaa-001: att-pending (status="pending"), att-voided (status="voided"), att-confirmed (status="confirmed"). A fourth record att-other-tenant exists in tenant-bbb-002 (different tenant) with status="confirmed". billing_specialist is authenticated with X-Tenant-Id: tenant-aaa-001.</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="8" t="n"/>
+      <c r="D34" s="8" t="n"/>
+      <c r="E34" s="8" t="n"/>
+      <c r="F34" s="8" t="n"/>
+      <c r="G34" s="8" t="n"/>
+      <c r="H34" s="8" t="n"/>
+      <c r="I34" s="8" t="n"/>
+      <c r="J34" s="8" t="n"/>
+      <c r="K34" s="10" t="n"/>
+      <c r="L34" s="3" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.5 Step 1</t>
+        </is>
+      </c>
+      <c r="B35" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C35" s="16" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims with billing_specialist headers and attendance_ids=[att-pending_id] plus all required fields. Assert response status equals 422.</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity. error_code="ATTENDANCE_NOT_CONFIRMED". Pending attendance cannot be used in a claim.</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H35" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I35" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J35" s="16" t="n"/>
+      <c r="K35" s="16" t="n"/>
+      <c r="L35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.5 Step 2</t>
+        </is>
+      </c>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims with attendance_ids=[att-voided_id] plus all required fields. Assert response status equals 422.</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity. error_code="ATTENDANCE_NOT_CONFIRMED". Voided attendance cannot be used in a claim.</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H36" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I36" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J36" s="16" t="n"/>
+      <c r="K36" s="16" t="n"/>
+      <c r="L36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.5 Step 3</t>
+        </is>
+      </c>
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims with attendance_ids=[att-other-tenant_id] from tenant-bbb-002, using billing_specialist headers for tenant-aaa-001. Assert response status equals 422 or 404.</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 422 or 404. Cross-tenant attendance is not visible to tenant-aaa-001. Request rejected.</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H37" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I37" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J37" s="16" t="n"/>
+      <c r="K37" s="16" t="n"/>
+      <c r="L37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.5 Step 4</t>
+        </is>
+      </c>
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims with attendance_ids=[att-confirmed_id] and all required fields (tenant_id, participant_id, payer_type, procedure_code, date_of_service_start). Assert response status equals 201.</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created. Response body contains claim_id, claim_reference_number, claim_status="draft".</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H38" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I38" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J38" s="16" t="n"/>
+      <c r="K38" s="16" t="n"/>
+      <c r="L38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.5 Step 5</t>
+        </is>
+      </c>
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C39" s="16" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body contains a non-null claim_id, claim_status="draft", and claim_reference_number matching pattern MCD-YYYYMMDD-XXXXXXXX or MCR-YYYYMMDD-XXXXXXXX.</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>claim_id present, claim_status="draft", claim_reference_number in expected format.</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Business Rules</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H39" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I39" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J39" s="16" t="n"/>
+      <c r="K39" s="16" t="n"/>
+      <c r="L39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.5 Step 6</t>
+        </is>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT status FROM attendance WHERE attendance_id="&lt;att-confirmed_id&gt;". Assert status="billed".</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>att-confirmed status = "billed" after successful claim creation. Attendance auto-updated by the POST /claims endpoint.</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H40" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I40" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J40" s="16" t="n"/>
+      <c r="K40" s="16" t="n"/>
+      <c r="L40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>TC-4.6 - POST /claims Multiple Confirmed Attendance Records Returns 201; DB units_billed Sum; Non-Existent Attendance UUID Returns 422 CLAIM_ATTENDANCE_NOT_FOUND | Claim</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="n"/>
+      <c r="C41" s="8" t="n"/>
+      <c r="D41" s="8" t="n"/>
+      <c r="E41" s="8" t="n"/>
+      <c r="F41" s="8" t="n"/>
+      <c r="G41" s="8" t="n"/>
+      <c r="H41" s="8" t="n"/>
+      <c r="I41" s="8" t="n"/>
+      <c r="J41" s="8" t="n"/>
+      <c r="K41" s="10" t="n"/>
+      <c r="L41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: Three confirmed attendance records exist in tenant-aaa-001 for participant P1: att-A (authorized_units_consumed=4.0), att-B (authorized_units_consumed=6.0), att-C (authorized_units_consumed=8.0). billing_specialist is authenticated.</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="n"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="E42" s="8" t="n"/>
+      <c r="F42" s="8" t="n"/>
+      <c r="G42" s="8" t="n"/>
+      <c r="H42" s="8" t="n"/>
+      <c r="I42" s="8" t="n"/>
+      <c r="J42" s="8" t="n"/>
+      <c r="K42" s="10" t="n"/>
+      <c r="L42" s="3" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.6 Step 1</t>
+        </is>
+      </c>
+      <c r="B43" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims with billing_specialist headers. Body: {"tenant_id":"tenant-aaa-001","participant_id":"&lt;P1_id&gt;","attendance_ids":["&lt;att-A_id&gt;","&lt;att-B_id&gt;","&lt;att-C_id&gt;"],"payer_type":"medicaid","procedure_code":"T2029","date_of_service_start":"2026-03-10"}. units_billed is intentionally omitted from the payload. Assert response status equals 201.</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created. Server calculates units_billed = 18.0 as the sum of authorized_units_consumed from all three referenced attendance records (4.0 + 6.0 + 8.0). Claim created with server-calculated value.</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H43" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I43" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J43" s="16" t="n"/>
+      <c r="K43" s="16" t="n"/>
+      <c r="L43" s="4" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.6 Step 2</t>
+        </is>
+      </c>
+      <c r="B44" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body attendance_ids contains att-A_id, att-B_id, and att-C_id. Assert response body units_billed = 18.0 (server-calculated sum, not caller-supplied).</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Response attendance_ids = [att-A_id, att-B_id, att-C_id]. units_billed = 18.0 (4.0 + 6.0 + 8.0). Server-calculated; no caller value required.</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Business Rules</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H44" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I44" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J44" s="16" t="n"/>
+      <c r="K44" s="16" t="n"/>
+      <c r="L44" s="4" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.6 Step 3</t>
+        </is>
+      </c>
+      <c r="B45" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT units_billed FROM claim WHERE claim_id = {returned_claim_id}. Assert units_billed = 18.0.</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>DB units_billed = 18.0. Server-calculated value persisted correctly.</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H45" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I45" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J45" s="16" t="n"/>
+      <c r="K45" s="16" t="n"/>
+      <c r="L45" s="4" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.6 Step 4</t>
+        </is>
+      </c>
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT status FROM attendance WHERE attendance_id IN (att-A_id, att-B_id, att-C_id). Assert all three statuses = "billed".</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>All three referenced attendance records have status = "billed" after claim creation.</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H46" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I46" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J46" s="16" t="n"/>
+      <c r="K46" s="16" t="n"/>
+      <c r="L46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.6 Step 5</t>
+        </is>
+      </c>
+      <c r="B47" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims with attendance_ids=["00000000-0000-0000-0000-000000000000"] (non-existent UUID) and all other required fields. Assert response status equals 422.</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity. error_code="CLAIM_ATTENDANCE_NOT_FOUND". Non-existent attendance UUID rejected.</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H47" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I47" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J47" s="16" t="n"/>
+      <c r="K47" s="16" t="n"/>
+      <c r="L47" s="4" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.6 Step 6</t>
+        </is>
+      </c>
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Assert error_code = "CLAIM_ATTENDANCE_NOT_FOUND" and message contains the invalid UUID "00000000-0000-0000-0000-000000000000" for identification.</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>detail.error_code="CLAIM_ATTENDANCE_NOT_FOUND". Message includes the non-existent UUID.</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H48" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I48" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J48" s="16" t="n"/>
+      <c r="K48" s="16" t="n"/>
+      <c r="L48" s="4" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>TC-4.7 - POST /claims Missing Required Fields participant_id, procedure_code, payer_type Each Return 400 | Claim</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="n"/>
+      <c r="C49" s="8" t="n"/>
+      <c r="D49" s="8" t="n"/>
+      <c r="E49" s="8" t="n"/>
+      <c r="F49" s="8" t="n"/>
+      <c r="G49" s="8" t="n"/>
+      <c r="H49" s="8" t="n"/>
+      <c r="I49" s="8" t="n"/>
+      <c r="J49" s="8" t="n"/>
+      <c r="K49" s="10" t="n"/>
+      <c r="L49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: billing_specialist is authenticated in tenant-aaa-001. A confirmed attendance record att-001 exists. Three separate payloads are prepared each omitting one required field.</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="n"/>
+      <c r="C50" s="8" t="n"/>
+      <c r="D50" s="8" t="n"/>
+      <c r="E50" s="8" t="n"/>
+      <c r="F50" s="8" t="n"/>
+      <c r="G50" s="8" t="n"/>
+      <c r="H50" s="8" t="n"/>
+      <c r="I50" s="8" t="n"/>
+      <c r="J50" s="8" t="n"/>
+      <c r="K50" s="10" t="n"/>
+      <c r="L50" s="3" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.7 Step 1</t>
+        </is>
+      </c>
+      <c r="B51" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims omitting participant_id. Include all other required fields (tenant_id, attendance_ids, payer_type, procedure_code, date_of_service_start). Assert response status is 400 or 422 and response body contains the string "participant_id".</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 or 422. Response text contains "participant_id" identifying the missing field.</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H51" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I51" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J51" s="16" t="n"/>
+      <c r="K51" s="16" t="n"/>
+      <c r="L51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.7 Step 2</t>
+        </is>
+      </c>
+      <c r="B52" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C52" s="16" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims omitting procedure_code. Include all other required fields. Assert response status is 400 or 422 and response body contains the string "procedure_code".</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 or 422. Response text contains "procedure_code".</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H52" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I52" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J52" s="16" t="n"/>
+      <c r="K52" s="16" t="n"/>
+      <c r="L52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.7 Step 3</t>
+        </is>
+      </c>
+      <c r="B53" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C53" s="16" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims omitting payer_type. Include all other required fields. Assert response status is 400 or 422 and response body contains the string "payer_type".</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 or 422. Response text contains "payer_type".</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H53" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I53" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J53" s="16" t="n"/>
+      <c r="K53" s="16" t="n"/>
+      <c r="L53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.7 Step 4</t>
+        </is>
+      </c>
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT COUNT(*) FROM claim WHERE tenant_id="tenant-aaa-001" AND created_at &gt; {test_start_time}. Assert count = 0.</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>No claims created from any of the three invalid requests. DB unchanged.</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H54" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I54" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J54" s="16" t="n"/>
+      <c r="K54" s="16" t="n"/>
+      <c r="L54" s="4" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>TC-4.8 - POST /claims Produces PHI_WRITE Audit Event with All 11 Mandatory Fields; PATCH draft to submitted Produces PHI_DISCLOSE; GET /audit-logs Returns Both Events | Claim</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="n"/>
+      <c r="C55" s="8" t="n"/>
+      <c r="D55" s="8" t="n"/>
+      <c r="E55" s="8" t="n"/>
+      <c r="F55" s="8" t="n"/>
+      <c r="G55" s="8" t="n"/>
+      <c r="H55" s="8" t="n"/>
+      <c r="I55" s="8" t="n"/>
+      <c r="J55" s="8" t="n"/>
+      <c r="K55" s="10" t="n"/>
+      <c r="L55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: billing_specialist (X-User-Id: user-billing-001, X-Session-Id: sess-tc48) is authenticated in tenant-aaa-001. A confirmed attendance record att-audit-001 exists for participant P1. compliance_officer is available for audit log reads.</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="n"/>
+      <c r="C56" s="8" t="n"/>
+      <c r="D56" s="8" t="n"/>
+      <c r="E56" s="8" t="n"/>
+      <c r="F56" s="8" t="n"/>
+      <c r="G56" s="8" t="n"/>
+      <c r="H56" s="8" t="n"/>
+      <c r="I56" s="8" t="n"/>
+      <c r="J56" s="8" t="n"/>
+      <c r="K56" s="10" t="n"/>
+      <c r="L56" s="3" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.8 Step 1</t>
+        </is>
+      </c>
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims with billing_specialist headers (X-User-Id: user-billing-001, X-Session-Id: sess-tc48). Body: valid payload referencing att-audit-001. Assert response status equals 201. Record returned claim_id.</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created. claim_id returned in response.</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(b); CMS Medicaid/Medicare</t>
+        </is>
+      </c>
+      <c r="H57" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I57" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J57" s="16" t="n"/>
+      <c r="K57" s="16" t="n"/>
+      <c r="L57" s="4" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.8 Step 2</t>
+        </is>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>GET /audit-logs?tenant_id=tenant-aaa-001&amp;resource_type=Claim&amp;resource_id={claim_id} using compliance_officer headers. Assert response status equals 200 and body is a non-empty JSON array.</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK. Response is a JSON array with at least one audit entry.</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(b); CMS Medicaid/Medicare</t>
+        </is>
+      </c>
+      <c r="H58" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I58" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J58" s="16" t="n"/>
+      <c r="K58" s="16" t="n"/>
+      <c r="L58" s="4" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.8 Step 3</t>
+        </is>
+      </c>
+      <c r="B59" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C59" s="16" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Assert the audit log array contains an entry with action_type="PHI_WRITE" and resource_id={claim_id}. Assert all 11 mandatory fields are non-null: audit_id, timestamp, user_id, tenant_id, session_id, action_type, resource_type, resource_id, data_affected, source_ip, outcome.</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>PHI_WRITE entry present. All 11 mandatory fields non-null. outcome="SUCCESS".</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Business Rules</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(b); CMS Medicaid/Medicare</t>
+        </is>
+      </c>
+      <c r="H59" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I59" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J59" s="16" t="n"/>
+      <c r="K59" s="16" t="n"/>
+      <c r="L59" s="4" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.8 Step 4</t>
+        </is>
+      </c>
+      <c r="B60" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C60" s="16" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Assert data_affected in the PHI_WRITE entry is an array of field name strings only (e.g. "tenant_id", "procedure_code", "attendance_ids"). Assert no PHI values such as names, SSNs, or DOBs appear anywhere in the audit entry.</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>data_affected contains field names only. No PHI values exposed in audit log.</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>Business Rules</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(b); CMS Medicaid/Medicare</t>
+        </is>
+      </c>
+      <c r="H60" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I60" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J60" s="16" t="n"/>
+      <c r="K60" s="16" t="n"/>
+      <c r="L60" s="4" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.8 Step 5</t>
+        </is>
+      </c>
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C61" s="16" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /claims/{claim_id} with billing_specialist headers. Body: {"version":1,"claim_status":"submitted"}. Assert response status equals 200 and response shows claim_status="submitted".</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK. claim_status = "submitted". draft-to-submitted transition triggers PHI_DISCLOSE audit event.</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(b); CMS Medicaid/Medicare</t>
+        </is>
+      </c>
+      <c r="H61" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I61" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J61" s="16" t="n"/>
+      <c r="K61" s="16" t="n"/>
+      <c r="L61" s="4" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.8 Step 6</t>
+        </is>
+      </c>
+      <c r="B62" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C62" s="16" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>GET /audit-logs?tenant_id=tenant-aaa-001&amp;resource_type=Claim&amp;resource_id={claim_id} using compliance_officer headers. Assert the response list contains an entry with action_type="PHI_DISCLOSE".</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>At least one audit entry with action_type="PHI_DISCLOSE" exists for the claim_id.</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(b); CMS Medicaid/Medicare</t>
+        </is>
+      </c>
+      <c r="H62" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I62" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J62" s="16" t="n"/>
+      <c r="K62" s="16" t="n"/>
+      <c r="L62" s="4" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.8 Step 7</t>
+        </is>
+      </c>
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>Assert PHI_DISCLOSE entry data_affected = ["claim_status","submission_date","claim_reference_number"]. Assert outcome="SUCCESS". Assert no raw PHI values appear in the event.</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>PHI_DISCLOSE data_affected = ["claim_status","submission_date","claim_reference_number"]. outcome="SUCCESS". No PHI values exposed.</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>Business Rules</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(b); CMS Medicaid/Medicare</t>
+        </is>
+      </c>
+      <c r="H63" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I63" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J63" s="16" t="n"/>
+      <c r="K63" s="16" t="n"/>
+      <c r="L63" s="4" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>TC-4.9 - POST /claims with Empty attendance_ids Returns 422 CLAIM_NO_ATTENDANCE_RECORDS; DB No Claim Created; Server Calculates units_billed from Attendance; Caller Value Ignored | Claim</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="n"/>
+      <c r="C64" s="8" t="n"/>
+      <c r="D64" s="8" t="n"/>
+      <c r="E64" s="8" t="n"/>
+      <c r="F64" s="8" t="n"/>
+      <c r="G64" s="8" t="n"/>
+      <c r="H64" s="8" t="n"/>
+      <c r="I64" s="8" t="n"/>
+      <c r="J64" s="8" t="n"/>
+      <c r="K64" s="10" t="n"/>
+      <c r="L64" s="2" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: billing_specialist is authenticated in tenant-aaa-001. A confirmed attendance record att-units-001 (authorized_units_consumed=4.0) exists for participant P1.</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="n"/>
+      <c r="C65" s="8" t="n"/>
+      <c r="D65" s="8" t="n"/>
+      <c r="E65" s="8" t="n"/>
+      <c r="F65" s="8" t="n"/>
+      <c r="G65" s="8" t="n"/>
+      <c r="H65" s="8" t="n"/>
+      <c r="I65" s="8" t="n"/>
+      <c r="J65" s="8" t="n"/>
+      <c r="K65" s="10" t="n"/>
+      <c r="L65" s="3" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.9 Step 1</t>
+        </is>
+      </c>
+      <c r="B66" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C66" s="16" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims with body {"tenant_id":"tenant-aaa-001","participant_id":"&lt;P1_id&gt;","attendance_ids":[],"payer_type":"medicaid","procedure_code":"T2029","date_of_service_start":"2026-03-15"}. Assert response status equals 422.</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity. error_code="CLAIM_NO_ATTENDANCE_RECORDS". Empty attendance list rejected.</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H66" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I66" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J66" s="16" t="n"/>
+      <c r="K66" s="16" t="n"/>
+      <c r="L66" s="4" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.9 Step 2</t>
+        </is>
+      </c>
+      <c r="B67" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C67" s="16" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body detail.error_code = "CLAIM_NO_ATTENDANCE_RECORDS".</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>error_code = "CLAIM_NO_ATTENDANCE_RECORDS".</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H67" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I67" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J67" s="16" t="n"/>
+      <c r="K67" s="16" t="n"/>
+      <c r="L67" s="4" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.9 Step 3</t>
+        </is>
+      </c>
+      <c r="B68" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C68" s="16" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT COUNT(*) FROM claim WHERE tenant_id="tenant-aaa-001" AND date_of_service_start="2026-03-15". Assert count = 0.</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>No claim created. DB unchanged.</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H68" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I68" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J68" s="16" t="n"/>
+      <c r="K68" s="16" t="n"/>
+      <c r="L68" s="4" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.9 Step 4</t>
+        </is>
+      </c>
+      <c r="B69" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C69" s="16" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims with attendance_ids=[att-units-001_id] and units_billed=999.0 (intentionally incorrect caller value; att-units-001 has authorized_units_consumed=4.0) plus all required fields. Assert response status equals 201.</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created. Server ignores caller-supplied units_billed=999.0 and uses server-calculated value = 4.0 (derived from authorized_units_consumed of att-units-001). Response body units_billed = 4.0.</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H69" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I69" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J69" s="16" t="n"/>
+      <c r="K69" s="16" t="n"/>
+      <c r="L69" s="4" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.9 Step 5</t>
+        </is>
+      </c>
+      <c r="B70" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C70" s="16" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body units_billed = 4.0 (server-calculated, not the caller-supplied 999.0). Query DB: SELECT units_billed FROM claim WHERE claim_id = {returned_claim_id}. Assert units_billed = 4.0.</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>Response and DB both show units_billed = 4.0. Caller-supplied value 999.0 was ignored. Server-calculated value from authorized_units_consumed persisted.</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H70" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I70" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J70" s="16" t="n"/>
+      <c r="K70" s="16" t="n"/>
+      <c r="L70" s="4" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>TC-4.10 - POST /claims with Phase 2 Fields secondary_payer_id, mco_id, prior_authorization_number Returns 400; DB No Claim Created in Each Case | Claim</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="n"/>
+      <c r="C71" s="8" t="n"/>
+      <c r="D71" s="8" t="n"/>
+      <c r="E71" s="8" t="n"/>
+      <c r="F71" s="8" t="n"/>
+      <c r="G71" s="8" t="n"/>
+      <c r="H71" s="8" t="n"/>
+      <c r="I71" s="8" t="n"/>
+      <c r="J71" s="8" t="n"/>
+      <c r="K71" s="10" t="n"/>
+      <c r="L71" s="2" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: billing_specialist is authenticated in tenant-aaa-001. A confirmed attendance record att-p2-001 exists. Phase 2 fields (secondary_payer_id, mco_id, prior_authorization_number) are not part of the Phase 1 ClaimCreate schema.</t>
+        </is>
+      </c>
+      <c r="B72" s="8" t="n"/>
+      <c r="C72" s="8" t="n"/>
+      <c r="D72" s="8" t="n"/>
+      <c r="E72" s="8" t="n"/>
+      <c r="F72" s="8" t="n"/>
+      <c r="G72" s="8" t="n"/>
+      <c r="H72" s="8" t="n"/>
+      <c r="I72" s="8" t="n"/>
+      <c r="J72" s="8" t="n"/>
+      <c r="K72" s="10" t="n"/>
+      <c r="L72" s="3" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.10 Step 1</t>
+        </is>
+      </c>
+      <c r="B73" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C73" s="16" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims with all required Phase 1 fields plus secondary_payer_id="payer-999" in the request body. Assert response status equals 400.</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request. secondary_payer_id identified as a disallowed field. No claim created.</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H73" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I73" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J73" s="16" t="n"/>
+      <c r="K73" s="16" t="n"/>
+      <c r="L73" s="4" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.10 Step 2</t>
+        </is>
+      </c>
+      <c r="B74" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C74" s="16" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT COUNT(*) FROM claim WHERE tenant_id="tenant-aaa-001" AND created_at &gt; {test_start_time}. Assert count = 0.</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>No claim created by the secondary_payer_id request.</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H74" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I74" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J74" s="16" t="n"/>
+      <c r="K74" s="16" t="n"/>
+      <c r="L74" s="4" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.10 Step 3</t>
+        </is>
+      </c>
+      <c r="B75" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C75" s="16" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims with all required fields plus mco_id="mco-001". Assert response status equals 400.</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request. mco_id is not an accepted field in Phase 1 claim schema.</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H75" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I75" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J75" s="16" t="n"/>
+      <c r="K75" s="16" t="n"/>
+      <c r="L75" s="4" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.10 Step 4</t>
+        </is>
+      </c>
+      <c r="B76" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C76" s="16" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: assert claim count still unchanged (no new records from step 3 request).</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>No claim created by the mco_id request. Count unchanged.</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H76" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I76" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J76" s="16" t="n"/>
+      <c r="K76" s="16" t="n"/>
+      <c r="L76" s="4" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.10 Step 5</t>
+        </is>
+      </c>
+      <c r="B77" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C77" s="16" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims with all required fields plus prior_authorization_number="PA-12345". Assert response status equals 400.</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request. prior_authorization_number is not accepted in Phase 1.</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H77" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I77" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J77" s="16" t="n"/>
+      <c r="K77" s="16" t="n"/>
+      <c r="L77" s="4" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.10 Step 6</t>
+        </is>
+      </c>
+      <c r="B78" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C78" s="16" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT COUNT(*) FROM claim WHERE tenant_id="tenant-aaa-001" AND created_at &gt; {test_start_time}. Assert count = 0 across all three Phase 2 field requests.</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>No claims created by any of the three rejected requests. DB fully unchanged.</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H78" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I78" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J78" s="16" t="n"/>
+      <c r="K78" s="16" t="n"/>
+      <c r="L78" s="4" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>TC-4.11 - PATCH /claims Stale Version Returns 409 CLAIM_VERSION_CONFLICT; Submitted Claim Returns 422 Before Version Check; Correct Version Returns 200 and DB Version Incremented | Claim</t>
+        </is>
+      </c>
+      <c r="B79" s="8" t="n"/>
+      <c r="C79" s="8" t="n"/>
+      <c r="D79" s="8" t="n"/>
+      <c r="E79" s="8" t="n"/>
+      <c r="F79" s="8" t="n"/>
+      <c r="G79" s="8" t="n"/>
+      <c r="H79" s="8" t="n"/>
+      <c r="I79" s="8" t="n"/>
+      <c r="J79" s="8" t="n"/>
+      <c r="K79" s="10" t="n"/>
+      <c r="L79" s="2" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: Claim A (C_A) exists in tenant-aaa-001 with claim_status="draft" and version=1. Claim B (C_B) exists with claim_status="submitted" and version=1. billing_specialist is authenticated.</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="n"/>
+      <c r="C80" s="8" t="n"/>
+      <c r="D80" s="8" t="n"/>
+      <c r="E80" s="8" t="n"/>
+      <c r="F80" s="8" t="n"/>
+      <c r="G80" s="8" t="n"/>
+      <c r="H80" s="8" t="n"/>
+      <c r="I80" s="8" t="n"/>
+      <c r="J80" s="8" t="n"/>
+      <c r="K80" s="10" t="n"/>
+      <c r="L80" s="3" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.11 Step 1</t>
+        </is>
+      </c>
+      <c r="B81" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C81" s="16" t="inlineStr">
+        <is>
+          <t>4.11</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>GET /claims/&lt;C_A_id&gt; with billing_specialist headers. Confirm claim_status="draft" and version=1.</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200. claim_status="draft", version=1.</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H81" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I81" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J81" s="16" t="n"/>
+      <c r="K81" s="16" t="n"/>
+      <c r="L81" s="4" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.11 Step 2</t>
+        </is>
+      </c>
+      <c r="B82" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C82" s="16" t="inlineStr">
+        <is>
+          <t>4.11</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /claims/&lt;C_A_id&gt; with body {"version":0,"rejection_reason":"stale version test"}. Assert response status equals 409.</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 409 Conflict. error_code="CLAIM_VERSION_CONFLICT". Stale version rejected before any field changes applied.</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H82" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I82" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J82" s="16" t="n"/>
+      <c r="K82" s="16" t="n"/>
+      <c r="L82" s="4" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.11 Step 3</t>
+        </is>
+      </c>
+      <c r="B83" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C83" s="16" t="inlineStr">
+        <is>
+          <t>4.11</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT version, claim_status FROM claim WHERE claim_id="&lt;C_A_id&gt;". Assert version=1 and claim_status="draft" (unchanged).</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>version=1, claim_status="draft". No changes applied by the rejected PATCH.</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H83" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I83" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J83" s="16" t="n"/>
+      <c r="K83" s="16" t="n"/>
+      <c r="L83" s="4" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.11 Step 4</t>
+        </is>
+      </c>
+      <c r="B84" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C84" s="16" t="inlineStr">
+        <is>
+          <t>4.11</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /claims/&lt;C_B_id&gt; (claim_status="submitted") with any body including correct version. Assert response status equals 422 with error_code="CLAIM_STATUS_IMMUTABLE". Confirm 422 is returned before the version check is performed.</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 422 before version check. CLAIM_STATUS_IMMUTABLE returned for submitted claim regardless of version correctness.</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>Business Rules</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H84" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I84" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J84" s="16" t="n"/>
+      <c r="K84" s="16" t="n"/>
+      <c r="L84" s="4" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.11 Step 5</t>
+        </is>
+      </c>
+      <c r="B85" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C85" s="16" t="inlineStr">
+        <is>
+          <t>4.11</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /claims/&lt;C_A_id&gt; with body {"version":1,"rejection_reason":"corrected field value"}. Assert response status equals 200.</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK. Update accepted with correct version. Response body contains updated rejection_reason.</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H85" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I85" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J85" s="16" t="n"/>
+      <c r="K85" s="16" t="n"/>
+      <c r="L85" s="4" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.11 Step 6</t>
+        </is>
+      </c>
+      <c r="B86" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C86" s="16" t="inlineStr">
+        <is>
+          <t>4.11</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body version = 2 (incremented from 1 to 2).</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>version = 2 in response body. Version correctly incremented on successful PATCH.</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>Business Rules</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H86" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I86" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J86" s="16" t="n"/>
+      <c r="K86" s="16" t="n"/>
+      <c r="L86" s="4" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.11 Step 7</t>
+        </is>
+      </c>
+      <c r="B87" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C87" s="16" t="inlineStr">
+        <is>
+          <t>4.11</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT version FROM claim WHERE claim_id="&lt;C_A_id&gt;". Assert version = 2.</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>DB version = 2. Persistent version increment confirmed.</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H87" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I87" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J87" s="16" t="n"/>
+      <c r="K87" s="16" t="n"/>
+      <c r="L87" s="4" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>TC-4.12 - POST /claims Cross-Tenant Attendance Reference Returns 422 or 404; DB No Cross-Tenant Claim Created | Claim</t>
+        </is>
+      </c>
+      <c r="B88" s="8" t="n"/>
+      <c r="C88" s="8" t="n"/>
+      <c r="D88" s="8" t="n"/>
+      <c r="E88" s="8" t="n"/>
+      <c r="F88" s="8" t="n"/>
+      <c r="G88" s="8" t="n"/>
+      <c r="H88" s="8" t="n"/>
+      <c r="I88" s="8" t="n"/>
+      <c r="J88" s="8" t="n"/>
+      <c r="K88" s="10" t="n"/>
+      <c r="L88" s="2" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: Attendance record att-tenant-bbb exists in tenant-bbb-002 with status="confirmed". billing_specialist is authenticated with X-Tenant-Id: tenant-aaa-001.</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="n"/>
+      <c r="C89" s="8" t="n"/>
+      <c r="D89" s="8" t="n"/>
+      <c r="E89" s="8" t="n"/>
+      <c r="F89" s="8" t="n"/>
+      <c r="G89" s="8" t="n"/>
+      <c r="H89" s="8" t="n"/>
+      <c r="I89" s="8" t="n"/>
+      <c r="J89" s="8" t="n"/>
+      <c r="K89" s="10" t="n"/>
+      <c r="L89" s="3" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.12 Step 1</t>
+        </is>
+      </c>
+      <c r="B90" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C90" s="16" t="inlineStr">
+        <is>
+          <t>4.12</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims with billing_specialist headers (X-Tenant-Id: tenant-aaa-001). Body: {"tenant_id":"tenant-aaa-001","participant_id":"&lt;P1_id&gt;","attendance_ids":["&lt;att-tenant-bbb_id&gt;"],"payer_type":"medicaid","procedure_code":"T2029","date_of_service_start":"2026-04-01"}. Assert response status equals 422 or 404.</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 422 or 404. Cross-tenant attendance not found or inaccessible from tenant-aaa-001.</t>
+        </is>
+      </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H90" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I90" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J90" s="16" t="n"/>
+      <c r="K90" s="16" t="n"/>
+      <c r="L90" s="4" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.12 Step 2</t>
+        </is>
+      </c>
+      <c r="B91" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C91" s="16" t="inlineStr">
+        <is>
+          <t>4.12</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body error_code is "ATTENDANCE_NOT_FOUND" or "NOT_FOUND" indicating the cross-tenant attendance was not accessible.</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>error_code = "ATTENDANCE_NOT_FOUND" or "NOT_FOUND". Attendance from another tenant is rejected.</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H91" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I91" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J91" s="16" t="n"/>
+      <c r="K91" s="16" t="n"/>
+      <c r="L91" s="4" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.12 Step 3</t>
+        </is>
+      </c>
+      <c r="B92" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C92" s="16" t="inlineStr">
+        <is>
+          <t>4.12</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT COUNT(*) FROM claim WHERE tenant_id="tenant-aaa-001" AND date_of_service_start="2026-04-01". Assert count = 0.</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr">
+        <is>
+          <t>No claim record created in tenant-aaa-001 referencing the cross-tenant attendance.</t>
+        </is>
+      </c>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H92" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I92" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J92" s="16" t="n"/>
+      <c r="K92" s="16" t="n"/>
+      <c r="L92" s="4" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.12 Step 4</t>
+        </is>
+      </c>
+      <c r="B93" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C93" s="16" t="inlineStr">
+        <is>
+          <t>4.12</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT COUNT(*) FROM claim WHERE attendance_ids LIKE "%&lt;att-tenant-bbb_id&gt;%". Assert count = 0.</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>No claim in any tenant references the cross-tenant attendance in an unauthorized manner.</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H93" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I93" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J93" s="16" t="n"/>
+      <c r="K93" s="16" t="n"/>
+      <c r="L93" s="4" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>TC-4.13 - POST /claims Referencing Attendance Already Linked to Existing Claim Returns 422 ATTENDANCE_NOT_CONFIRMED; DB No Duplicate Claim | Claim</t>
+        </is>
+      </c>
+      <c r="B94" s="8" t="n"/>
+      <c r="C94" s="8" t="n"/>
+      <c r="D94" s="8" t="n"/>
+      <c r="E94" s="8" t="n"/>
+      <c r="F94" s="8" t="n"/>
+      <c r="G94" s="8" t="n"/>
+      <c r="H94" s="8" t="n"/>
+      <c r="I94" s="8" t="n"/>
+      <c r="J94" s="8" t="n"/>
+      <c r="K94" s="10" t="n"/>
+      <c r="L94" s="2" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: Attendance record att-billed-001 exists in tenant-aaa-001 with status="billed", already linked to claim C_existing. billing_specialist is authenticated.</t>
+        </is>
+      </c>
+      <c r="B95" s="8" t="n"/>
+      <c r="C95" s="8" t="n"/>
+      <c r="D95" s="8" t="n"/>
+      <c r="E95" s="8" t="n"/>
+      <c r="F95" s="8" t="n"/>
+      <c r="G95" s="8" t="n"/>
+      <c r="H95" s="8" t="n"/>
+      <c r="I95" s="8" t="n"/>
+      <c r="J95" s="8" t="n"/>
+      <c r="K95" s="10" t="n"/>
+      <c r="L95" s="3" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.13 Step 1</t>
+        </is>
+      </c>
+      <c r="B96" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C96" s="16" t="inlineStr">
+        <is>
+          <t>4.13</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>GET /attendance/&lt;att-billed-001_id&gt; with billing_specialist headers. Assert response status equals 200 and status="billed".</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200. attendance status="billed". Already associated with an existing claim.</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H96" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I96" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J96" s="16" t="n"/>
+      <c r="K96" s="16" t="n"/>
+      <c r="L96" s="4" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.13 Step 2</t>
+        </is>
+      </c>
+      <c r="B97" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C97" s="16" t="inlineStr">
+        <is>
+          <t>4.13</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>POST /claims with body {"tenant_id":"tenant-aaa-001","participant_id":"&lt;P2_id&gt;","attendance_ids":["&lt;att-billed-001_id&gt;"],"payer_type":"medicaid","procedure_code":"T2029","date_of_service_start":"2026-05-01"}. Assert response status equals 422.</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity. error_code="ATTENDANCE_NOT_CONFIRMED". Billed attendance cannot be claimed again.</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H97" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I97" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J97" s="16" t="n"/>
+      <c r="K97" s="16" t="n"/>
+      <c r="L97" s="4" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.13 Step 3</t>
+        </is>
+      </c>
+      <c r="B98" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C98" s="16" t="inlineStr">
+        <is>
+          <t>4.13</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body error_code = "ATTENDANCE_NOT_CONFIRMED" and message indicates att-billed-001 is not in confirmed status.</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t>error_code="ATTENDANCE_NOT_CONFIRMED". Message identifies att-billed-001 as already billed.</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H98" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I98" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J98" s="16" t="n"/>
+      <c r="K98" s="16" t="n"/>
+      <c r="L98" s="4" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.13 Step 4</t>
+        </is>
+      </c>
+      <c r="B99" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C99" s="16" t="inlineStr">
+        <is>
+          <t>4.13</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT COUNT(*) FROM claim WHERE attendance_ids LIKE "%&lt;att-billed-001_id&gt;%" AND claim_id != "&lt;C_existing_id&gt;". Assert count = 0.</t>
+        </is>
+      </c>
+      <c r="E99" s="4" t="inlineStr">
+        <is>
+          <t>Count = 0. att-billed-001 is not linked to any claim other than C_existing.</t>
+        </is>
+      </c>
+      <c r="F99" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H99" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I99" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J99" s="16" t="n"/>
+      <c r="K99" s="16" t="n"/>
+      <c r="L99" s="4" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>TC-4.14 - GET /claims Non-Existent claim_id Returns 404 NOT_FOUND | Claim</t>
+        </is>
+      </c>
+      <c r="B100" s="8" t="n"/>
+      <c r="C100" s="8" t="n"/>
+      <c r="D100" s="8" t="n"/>
+      <c r="E100" s="8" t="n"/>
+      <c r="F100" s="8" t="n"/>
+      <c r="G100" s="8" t="n"/>
+      <c r="H100" s="8" t="n"/>
+      <c r="I100" s="8" t="n"/>
+      <c r="J100" s="8" t="n"/>
+      <c r="K100" s="10" t="n"/>
+      <c r="L100" s="2" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: billing_specialist is authenticated in tenant-aaa-001. The UUID "00000000-0000-0000-0000-999999999999" does not exist in the claim table.</t>
+        </is>
+      </c>
+      <c r="B101" s="8" t="n"/>
+      <c r="C101" s="8" t="n"/>
+      <c r="D101" s="8" t="n"/>
+      <c r="E101" s="8" t="n"/>
+      <c r="F101" s="8" t="n"/>
+      <c r="G101" s="8" t="n"/>
+      <c r="H101" s="8" t="n"/>
+      <c r="I101" s="8" t="n"/>
+      <c r="J101" s="8" t="n"/>
+      <c r="K101" s="10" t="n"/>
+      <c r="L101" s="3" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.14 Step 1</t>
+        </is>
+      </c>
+      <c r="B102" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C102" s="16" t="inlineStr">
+        <is>
+          <t>4.14</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>Send GET /claims/00000000-0000-0000-0000-999999999999 with billing_specialist headers (X-User-Role: billing_specialist, X-User-Status: active, X-Tenant-Id: tenant-aaa-001).</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found. Response body contains error_code="NOT_FOUND".</t>
+        </is>
+      </c>
+      <c r="F102" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G102" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H102" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I102" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J102" s="16" t="n"/>
+      <c r="K102" s="16" t="n"/>
+      <c r="L102" s="4" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.14 Step 2</t>
+        </is>
+      </c>
+      <c r="B103" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C103" s="16" t="inlineStr">
+        <is>
+          <t>4.14</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>Assert response status code equals 404.</t>
+        </is>
+      </c>
+      <c r="E103" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found.</t>
+        </is>
+      </c>
+      <c r="F103" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H103" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I103" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J103" s="16" t="n"/>
+      <c r="K103" s="16" t="n"/>
+      <c r="L103" s="4" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.14 Step 3</t>
+        </is>
+      </c>
+      <c r="B104" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C104" s="16" t="inlineStr">
+        <is>
+          <t>4.14</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body detail.error_code = "NOT_FOUND".</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr">
+        <is>
+          <t>detail.error_code = "NOT_FOUND".</t>
+        </is>
+      </c>
+      <c r="F104" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G104" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H104" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I104" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J104" s="16" t="n"/>
+      <c r="K104" s="16" t="n"/>
+      <c r="L104" s="4" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.14 Step 4</t>
+        </is>
+      </c>
+      <c r="B105" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C105" s="16" t="inlineStr">
+        <is>
+          <t>4.14</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>Assert response body detail.message contains the string "00000000-0000-0000-0000-999999999999" or "Claim" to identify what resource was not found.</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="inlineStr">
+        <is>
+          <t>message contains the requested claim_id or the resource type "Claim" for traceability.</t>
+        </is>
+      </c>
+      <c r="F105" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G105" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H105" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I105" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J105" s="16" t="n"/>
+      <c r="K105" s="16" t="n"/>
+      <c r="L105" s="4" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>TC-4.15 - PATCH /claims Paid Claim Any Non-Status Field Returns 422 CLAIM_STATUS_IMMUTABLE; DB Claim Unchanged | Claim</t>
+        </is>
+      </c>
+      <c r="B106" s="8" t="n"/>
+      <c r="C106" s="8" t="n"/>
+      <c r="D106" s="8" t="n"/>
+      <c r="E106" s="8" t="n"/>
+      <c r="F106" s="8" t="n"/>
+      <c r="G106" s="8" t="n"/>
+      <c r="H106" s="8" t="n"/>
+      <c r="I106" s="8" t="n"/>
+      <c r="J106" s="8" t="n"/>
+      <c r="K106" s="10" t="n"/>
+      <c r="L106" s="2" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions: Claim C_paid exists in tenant-aaa-001 with claim_status="paid" and version=3. billing_specialist is authenticated.</t>
+        </is>
+      </c>
+      <c r="B107" s="8" t="n"/>
+      <c r="C107" s="8" t="n"/>
+      <c r="D107" s="8" t="n"/>
+      <c r="E107" s="8" t="n"/>
+      <c r="F107" s="8" t="n"/>
+      <c r="G107" s="8" t="n"/>
+      <c r="H107" s="8" t="n"/>
+      <c r="I107" s="8" t="n"/>
+      <c r="J107" s="8" t="n"/>
+      <c r="K107" s="10" t="n"/>
+      <c r="L107" s="3" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.15 Step 1</t>
+        </is>
+      </c>
+      <c r="B108" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C108" s="16" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>GET /claims/&lt;C_paid_id&gt; with billing_specialist headers. Confirm claim_status="paid" and capture version=3.</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200. claim_status="paid", version=3.</t>
+        </is>
+      </c>
+      <c r="F108" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G108" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H108" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I108" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J108" s="16" t="n"/>
+      <c r="K108" s="16" t="n"/>
+      <c r="L108" s="4" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.15 Step 2</t>
+        </is>
+      </c>
+      <c r="B109" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C109" s="16" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /claims/&lt;C_paid_id&gt; with body {"version":3,"rejection_reason":"Test non-status field edit"}. Assert response status equals 422.</t>
+        </is>
+      </c>
+      <c r="E109" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity. error_code="CLAIM_STATUS_IMMUTABLE". Paid claim is fully immutable.</t>
+        </is>
+      </c>
+      <c r="F109" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G109" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H109" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I109" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J109" s="16" t="n"/>
+      <c r="K109" s="16" t="n"/>
+      <c r="L109" s="4" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.15 Step 3</t>
+        </is>
+      </c>
+      <c r="B110" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C110" s="16" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /claims/&lt;C_paid_id&gt; with body {"version":3,"claim_status":"draft"}. Assert response status equals 422.</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity. error_code="CLAIM_STATUS_IMMUTABLE". Status cannot be rolled back from "paid".</t>
+        </is>
+      </c>
+      <c r="F110" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G110" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H110" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I110" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J110" s="16" t="n"/>
+      <c r="K110" s="16" t="n"/>
+      <c r="L110" s="4" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.15 Step 4</t>
+        </is>
+      </c>
+      <c r="B111" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C111" s="16" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /claims/&lt;C_paid_id&gt; with body {"version":3,"submission_date":"2026-01-01T00:00:00Z"}. Assert response status equals 422.</t>
+        </is>
+      </c>
+      <c r="E111" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity. error_code="CLAIM_STATUS_IMMUTABLE". All field changes rejected on paid claim.</t>
+        </is>
+      </c>
+      <c r="F111" s="4" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G111" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H111" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I111" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J111" s="16" t="n"/>
+      <c r="K111" s="16" t="n"/>
+      <c r="L111" s="4" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="4" t="inlineStr">
+        <is>
+          <t>TC-4.15 Step 5</t>
+        </is>
+      </c>
+      <c r="B112" s="16" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C112" s="16" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT claim_status, version, rejection_reason FROM claim WHERE claim_id="&lt;C_paid_id&gt;". Assert claim_status="paid", version=3, rejection_reason is null or unchanged.</t>
+        </is>
+      </c>
+      <c r="E112" s="4" t="inlineStr">
+        <is>
+          <t>claim_status="paid", version=3. All fields unchanged. No modifications persisted by any of the three rejected PATCH attempts.</t>
+        </is>
+      </c>
+      <c r="F112" s="4" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G112" s="4" t="inlineStr">
+        <is>
+          <t>CMS Medicaid Billing Integrity; 42 CFR Part 455</t>
+        </is>
+      </c>
+      <c r="H112" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I112" s="16" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J112" s="16" t="n"/>
+      <c r="K112" s="16" t="n"/>
+      <c r="L112" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="30">
+    <mergeCell ref="A34:K34"/>
+    <mergeCell ref="A64:K64"/>
+    <mergeCell ref="A24:K24"/>
+    <mergeCell ref="A49:K49"/>
+    <mergeCell ref="A107:K107"/>
+    <mergeCell ref="A94:K94"/>
+    <mergeCell ref="A79:K79"/>
+    <mergeCell ref="A88:K88"/>
+    <mergeCell ref="A25:K25"/>
+    <mergeCell ref="A65:K65"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A80:K80"/>
+    <mergeCell ref="A56:K56"/>
+    <mergeCell ref="A89:K89"/>
+    <mergeCell ref="A50:K50"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A101:K101"/>
+    <mergeCell ref="A55:K55"/>
+    <mergeCell ref="A95:K95"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A33:K33"/>
+    <mergeCell ref="A71:K71"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="A106:K106"/>
+    <mergeCell ref="A100:K100"/>
+    <mergeCell ref="A72:K72"/>
+    <mergeCell ref="A10:K10"/>
+    <mergeCell ref="A9:K9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add test_mar_record.py TC-5.1-5.21, test_incident.py TC-6.1-6.15, fix hardcoded dates, update test cases xlsx
</commit_message>
<xml_diff>
--- a/test_cases/test_cases_phase1.xlsx
+++ b/test_cases/test_cases_phase1.xlsx
@@ -15322,7 +15322,7 @@
     <row r="9">
       <c r="A9" s="32" t="inlineStr">
         <is>
-          <t>TC-5.2 - POST /mar-records by nurse_medication_aide Returns 201; DB Confirms Correct tenant_id and user_id | MARRecord</t>
+          <t>TC-5.2 - POST /mar-records by nurse_medication_aide Returns 201; DB Confirms Correct tenant_id and user_id; PHI_WRITE Audit Event Logged with All 11 Mandatory Fields | MARRecord</t>
         </is>
       </c>
       <c r="B9" s="36" t="n"/>
@@ -15558,7 +15558,7 @@
     <row r="15">
       <c r="A15" s="32" t="inlineStr">
         <is>
-          <t>TC-5.3 - POST /mar-records from care_coordinator Returns 403 MAR_RBAC_DENIED; POST from billing_specialist Returns 403; DB MAR Count Unchanged After Both Denied Attempts | MARRecord</t>
+          <t>TC-5.3 - POST /mar-records by billing_specialist Returns 403 RBAC_DENIED; DB Confirms No Row Created | MARRecord</t>
         </is>
       </c>
       <c r="B15" s="36" t="n"/>
@@ -16130,7 +16130,7 @@
     <row r="29">
       <c r="A29" s="32" t="inlineStr">
         <is>
-          <t>TC-5.5 - Write to Controlled-Substance MARRecord Produces PHI_WRITE Audit Event; DB Confirms 11 Mandatory Fields Non-Null and No PHI in data_affected; No time.sleep(); DB Query Only | MARRecord</t>
+          <t>TC-5.5 - POST /mar-records with status=administered and null administered_time Returns 422 MAR_MISSING_ADMINISTERED_TIME; DB Confirms No Row Created | MARRecord</t>
         </is>
       </c>
       <c r="B29" s="36" t="n"/>
@@ -16148,7 +16148,7 @@
     <row r="30">
       <c r="A30" s="33" t="inlineStr">
         <is>
-          <t>Preconditions: nurse_medication_aide (X-User-Id: user-nma-001, X-Session-Id: sess-tc55) authenticated in tenant-aaa-001. Participant P1 exists with no existing controlled-substance MAR record for the target time.</t>
+          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Initial MAR count for tenant-aaa-001 captured as N.</t>
         </is>
       </c>
       <c r="B30" s="36" t="n"/>
@@ -16181,12 +16181,12 @@
       </c>
       <c r="D31" s="34" t="inlineStr">
         <is>
-          <t>Send POST /mar-records with is_controlled_substance=true. Body: {"tenant_id":"tenant-aaa-001","participant_id":"&lt;P1&gt;","medication_name":"Oxycodone 5mg","scheduled_time":"fixture_scheduled_time","route":"oral","status":"scheduled","is_controlled_substance":true}.</t>
+          <t>Send POST /mar-records with status=administered and administered_time=null. All other fields valid.</t>
         </is>
       </c>
       <c r="E31" s="34" t="inlineStr">
         <is>
-          <t>HTTP 201 Created. mar_id returned.</t>
+          <t>HTTP 422 Unprocessable Entity. administered_time is required when status=administered.</t>
         </is>
       </c>
       <c r="F31" s="34" t="inlineStr">
@@ -16196,7 +16196,7 @@
       </c>
       <c r="G31" s="34" t="inlineStr">
         <is>
-          <t>HIPAA §164.312(a)(2)(iv); 42 CFR Part 2; CMS Medicaid/Medicare</t>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
         </is>
       </c>
       <c r="H31" s="34" t="inlineStr">
@@ -16231,22 +16231,22 @@
       </c>
       <c r="D32" s="34" t="inlineStr">
         <is>
-          <t>Query DB: SELECT * FROM audit_log WHERE resource_id=&lt;mar_id&gt; AND event_type='PHI_WRITE'. Assert exactly one row exists. No time.sleep() before this query.</t>
+          <t>Assert response HTTP status code equals 422.</t>
         </is>
       </c>
       <c r="E32" s="34" t="inlineStr">
         <is>
-          <t>Exactly one PHI_WRITE audit event row found.</t>
+          <t>HTTP 422.</t>
         </is>
       </c>
       <c r="F32" s="34" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>API</t>
         </is>
       </c>
       <c r="G32" s="34" t="inlineStr">
         <is>
-          <t>HIPAA §164.312(b); 42 CFR Part 2</t>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
         </is>
       </c>
       <c r="H32" s="34" t="inlineStr">
@@ -16281,12 +16281,12 @@
       </c>
       <c r="D33" s="34" t="inlineStr">
         <is>
-          <t>Assert all 11 mandatory fields non-null on the PHI_WRITE event row: event_id, event_type, timestamp, user_id, tenant_id, resource_type, resource_id, action, data_affected, session_id, ip_address.</t>
+          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE tenant_id='tenant-aaa-001'. Assert count = N (unchanged).</t>
         </is>
       </c>
       <c r="E33" s="34" t="inlineStr">
         <is>
-          <t>All 11 mandatory audit fields are non-null.</t>
+          <t>Count = N. No administered MAR row created.</t>
         </is>
       </c>
       <c r="F33" s="34" t="inlineStr">
@@ -16296,7 +16296,7 @@
       </c>
       <c r="G33" s="34" t="inlineStr">
         <is>
-          <t>HIPAA §164.312(b); 42 CFR Part 2</t>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
         </is>
       </c>
       <c r="H33" s="34" t="inlineStr">
@@ -16314,59 +16314,27 @@
       <c r="L33" s="34" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="34" t="inlineStr">
-        <is>
-          <t>TC-5.5 Step 4</t>
-        </is>
-      </c>
-      <c r="B34" s="34" t="inlineStr">
-        <is>
-          <t>MARRecord</t>
-        </is>
-      </c>
-      <c r="C34" s="34" t="inlineStr">
-        <is>
-          <t>5.5</t>
-        </is>
-      </c>
-      <c r="D34" s="34" t="inlineStr">
-        <is>
-          <t>Assert data_affected contains no raw PHI values: no medication_name literal, no participant_id value, no administered_time.</t>
-        </is>
-      </c>
-      <c r="E34" s="34" t="inlineStr">
-        <is>
-          <t>data_affected contains no raw PHI values.</t>
-        </is>
-      </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="G34" s="34" t="inlineStr">
-        <is>
-          <t>HIPAA §164.312(b); 42 CFR Part 2</t>
-        </is>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I34" s="34" t="inlineStr">
-        <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="J34" s="34" t="n"/>
-      <c r="K34" s="34" t="n"/>
-      <c r="L34" s="34" t="n"/>
+      <c r="A34" s="32" t="inlineStr">
+        <is>
+          <t>TC-5.6 - GET Controlled-Substance MARRecord by Privileged Role Returns 200; PHI_READ Audit Event Logged with All 11 Mandatory Fields Non-Null and No PHI in data_affected | MARRecord</t>
+        </is>
+      </c>
+      <c r="B34" s="36" t="n"/>
+      <c r="C34" s="36" t="n"/>
+      <c r="D34" s="36" t="n"/>
+      <c r="E34" s="36" t="n"/>
+      <c r="F34" s="36" t="n"/>
+      <c r="G34" s="36" t="n"/>
+      <c r="H34" s="36" t="n"/>
+      <c r="I34" s="36" t="n"/>
+      <c r="J34" s="36" t="n"/>
+      <c r="K34" s="37" t="n"/>
+      <c r="L34" s="32" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="32" t="inlineStr">
-        <is>
-          <t>TC-5.6 - Unauthorized Read Attempt on Controlled-Substance MARRecord Produces ACCESS_DENIED Audit Event; DB Confirms 11 Mandatory Fields Non-Null; No time.sleep(); DB Query Only | MARRecord</t>
+      <c r="A35" s="33" t="inlineStr">
+        <is>
+          <t>Preconditions: nurse_medication_aide (X-User-Id: user-nma-001, X-Session-Id: sess-tc55) authenticated in tenant-aaa-001. Participant P1 exists with no existing controlled-substance MAR record for the target time.</t>
         </is>
       </c>
       <c r="B35" s="36" t="n"/>
@@ -16379,30 +16347,62 @@
       <c r="I35" s="36" t="n"/>
       <c r="J35" s="36" t="n"/>
       <c r="K35" s="37" t="n"/>
-      <c r="L35" s="32" t="n"/>
+      <c r="L35" s="33" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="33" t="inlineStr">
-        <is>
-          <t>Preconditions: A controlled-substance mar_record exists in tenant-aaa-001 (mar_id known, is_controlled_substance=true). care_coordinator (X-User-Id: user-cc-001, X-Session-Id: sess-tc56) authenticated.</t>
-        </is>
-      </c>
-      <c r="B36" s="36" t="n"/>
-      <c r="C36" s="36" t="n"/>
-      <c r="D36" s="36" t="n"/>
-      <c r="E36" s="36" t="n"/>
-      <c r="F36" s="36" t="n"/>
-      <c r="G36" s="36" t="n"/>
-      <c r="H36" s="36" t="n"/>
-      <c r="I36" s="36" t="n"/>
-      <c r="J36" s="36" t="n"/>
-      <c r="K36" s="37" t="n"/>
-      <c r="L36" s="33" t="n"/>
+      <c r="A36" s="34" t="inlineStr">
+        <is>
+          <t>TC-5.6 Step 1</t>
+        </is>
+      </c>
+      <c r="B36" s="34" t="inlineStr">
+        <is>
+          <t>MARRecord</t>
+        </is>
+      </c>
+      <c r="C36" s="34" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="D36" s="34" t="inlineStr">
+        <is>
+          <t>Send POST /mar-records with is_controlled_substance=true. Body: {"tenant_id":"tenant-aaa-001","participant_id":"&lt;P1&gt;","medication_name":"Oxycodone 5mg","scheduled_time":"fixture_scheduled_time","route":"oral","status":"scheduled","is_controlled_substance":true}.</t>
+        </is>
+      </c>
+      <c r="E36" s="34" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created. mar_id returned.</t>
+        </is>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G36" s="34" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(a)(2)(iv); 42 CFR Part 2; CMS Medicaid/Medicare</t>
+        </is>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I36" s="34" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J36" s="34" t="n"/>
+      <c r="K36" s="34" t="n"/>
+      <c r="L36" s="34" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="34" t="inlineStr">
         <is>
-          <t>TC-5.6 Step 1</t>
+          <t>TC-5.6 Step 2</t>
         </is>
       </c>
       <c r="B37" s="34" t="inlineStr">
@@ -16417,22 +16417,22 @@
       </c>
       <c r="D37" s="34" t="inlineStr">
         <is>
-          <t>Send GET /mar-records/&lt;mar_id&gt; with care_coordinator headers (unauthorized for controlled-substance access).</t>
+          <t>Query DB: SELECT * FROM audit_log WHERE resource_id=&lt;mar_id&gt; AND event_type='PHI_WRITE'. Assert exactly one row exists. No time.sleep() before this query.</t>
         </is>
       </c>
       <c r="E37" s="34" t="inlineStr">
         <is>
-          <t>HTTP 403 Forbidden.</t>
+          <t>Exactly one PHI_WRITE audit event row found.</t>
         </is>
       </c>
       <c r="F37" s="34" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="G37" s="34" t="inlineStr">
         <is>
-          <t>HIPAA §164.312(a)(2)(iv); 42 CFR Part 2; CMS Medicaid/Medicare</t>
+          <t>HIPAA §164.312(b); 42 CFR Part 2</t>
         </is>
       </c>
       <c r="H37" s="34" t="inlineStr">
@@ -16452,7 +16452,7 @@
     <row r="38">
       <c r="A38" s="34" t="inlineStr">
         <is>
-          <t>TC-5.6 Step 2</t>
+          <t>TC-5.6 Step 3</t>
         </is>
       </c>
       <c r="B38" s="34" t="inlineStr">
@@ -16467,12 +16467,12 @@
       </c>
       <c r="D38" s="34" t="inlineStr">
         <is>
-          <t>Query DB: SELECT * FROM audit_log WHERE resource_id=&lt;mar_id&gt; AND event_type='ACCESS_DENIED'. Assert row exists. No time.sleep() before query.</t>
+          <t>Assert all 11 mandatory fields non-null on the PHI_WRITE event row: event_id, event_type, timestamp, user_id, tenant_id, resource_type, resource_id, action, data_affected, session_id, ip_address.</t>
         </is>
       </c>
       <c r="E38" s="34" t="inlineStr">
         <is>
-          <t>ACCESS_DENIED audit event row found for this resource.</t>
+          <t>All 11 mandatory audit fields are non-null.</t>
         </is>
       </c>
       <c r="F38" s="34" t="inlineStr">
@@ -16502,7 +16502,7 @@
     <row r="39">
       <c r="A39" s="34" t="inlineStr">
         <is>
-          <t>TC-5.6 Step 3</t>
+          <t>TC-5.6 Step 4</t>
         </is>
       </c>
       <c r="B39" s="34" t="inlineStr">
@@ -16517,12 +16517,12 @@
       </c>
       <c r="D39" s="34" t="inlineStr">
         <is>
-          <t>Assert all 11 mandatory fields non-null on the ACCESS_DENIED row: event_id, event_type, timestamp, user_id, tenant_id, resource_type, resource_id, action, data_affected, session_id, ip_address.</t>
+          <t>Assert data_affected contains no raw PHI values: no medication_name literal, no participant_id value, no administered_time.</t>
         </is>
       </c>
       <c r="E39" s="34" t="inlineStr">
         <is>
-          <t>All 11 mandatory audit fields are non-null.</t>
+          <t>data_affected contains no raw PHI values.</t>
         </is>
       </c>
       <c r="F39" s="34" t="inlineStr">
@@ -16550,59 +16550,27 @@
       <c r="L39" s="34" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="34" t="inlineStr">
-        <is>
-          <t>TC-5.6 Step 4</t>
-        </is>
-      </c>
-      <c r="B40" s="34" t="inlineStr">
-        <is>
-          <t>MARRecord</t>
-        </is>
-      </c>
-      <c r="C40" s="34" t="inlineStr">
-        <is>
-          <t>5.6</t>
-        </is>
-      </c>
-      <c r="D40" s="34" t="inlineStr">
-        <is>
-          <t>Assert data_affected contains no raw PHI values (no medication_name, participant_id, administered_time literals).</t>
-        </is>
-      </c>
-      <c r="E40" s="34" t="inlineStr">
-        <is>
-          <t>data_affected contains no raw PHI.</t>
-        </is>
-      </c>
-      <c r="F40" s="34" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="G40" s="34" t="inlineStr">
-        <is>
-          <t>HIPAA §164.312(b); 42 CFR Part 2</t>
-        </is>
-      </c>
-      <c r="H40" s="34" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I40" s="34" t="inlineStr">
-        <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="J40" s="34" t="n"/>
-      <c r="K40" s="34" t="n"/>
-      <c r="L40" s="34" t="n"/>
+      <c r="A40" s="32" t="inlineStr">
+        <is>
+          <t>TC-5.7 - POST /mar-records with status=refused and null notes Returns 422 MAR_MISSING_NOTES; DB Confirms No Row Created | MARRecord</t>
+        </is>
+      </c>
+      <c r="B40" s="36" t="n"/>
+      <c r="C40" s="36" t="n"/>
+      <c r="D40" s="36" t="n"/>
+      <c r="E40" s="36" t="n"/>
+      <c r="F40" s="36" t="n"/>
+      <c r="G40" s="36" t="n"/>
+      <c r="H40" s="36" t="n"/>
+      <c r="I40" s="36" t="n"/>
+      <c r="J40" s="36" t="n"/>
+      <c r="K40" s="37" t="n"/>
+      <c r="L40" s="32" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="32" t="inlineStr">
-        <is>
-          <t>TC-5.7 - POST /mar-records with status=administered and Valid administered_time Returns 201; DB Confirms status=administered | MARRecord</t>
+      <c r="A41" s="33" t="inlineStr">
+        <is>
+          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Initial refused MAR count captured as N.</t>
         </is>
       </c>
       <c r="B41" s="36" t="n"/>
@@ -16615,30 +16583,62 @@
       <c r="I41" s="36" t="n"/>
       <c r="J41" s="36" t="n"/>
       <c r="K41" s="37" t="n"/>
-      <c r="L41" s="32" t="n"/>
+      <c r="L41" s="33" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="33" t="inlineStr">
-        <is>
-          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Participant P1 exists. scheduled_time="fixture_scheduled_time".</t>
-        </is>
-      </c>
-      <c r="B42" s="36" t="n"/>
-      <c r="C42" s="36" t="n"/>
-      <c r="D42" s="36" t="n"/>
-      <c r="E42" s="36" t="n"/>
-      <c r="F42" s="36" t="n"/>
-      <c r="G42" s="36" t="n"/>
-      <c r="H42" s="36" t="n"/>
-      <c r="I42" s="36" t="n"/>
-      <c r="J42" s="36" t="n"/>
-      <c r="K42" s="37" t="n"/>
-      <c r="L42" s="33" t="n"/>
+      <c r="A42" s="34" t="inlineStr">
+        <is>
+          <t>TC-5.7 Step 1</t>
+        </is>
+      </c>
+      <c r="B42" s="34" t="inlineStr">
+        <is>
+          <t>MARRecord</t>
+        </is>
+      </c>
+      <c r="C42" s="34" t="inlineStr">
+        <is>
+          <t>5.7</t>
+        </is>
+      </c>
+      <c r="D42" s="34" t="inlineStr">
+        <is>
+          <t>Send POST /mar-records with status=refused and notes=null. All other fields valid.</t>
+        </is>
+      </c>
+      <c r="E42" s="34" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity. notes is required when status=refused.</t>
+        </is>
+      </c>
+      <c r="F42" s="34" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G42" s="34" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H42" s="34" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I42" s="34" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J42" s="34" t="n"/>
+      <c r="K42" s="34" t="n"/>
+      <c r="L42" s="34" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="34" t="inlineStr">
         <is>
-          <t>TC-5.7 Step 1</t>
+          <t>TC-5.7 Step 2</t>
         </is>
       </c>
       <c r="B43" s="34" t="inlineStr">
@@ -16653,12 +16653,12 @@
       </c>
       <c r="D43" s="34" t="inlineStr">
         <is>
-          <t>Send POST /mar-records with status=administered and administered_time=fixture_scheduled_time (equal to scheduled_time, within valid window). Body includes all required fields.</t>
+          <t>Assert response HTTP status code equals 422.</t>
         </is>
       </c>
       <c r="E43" s="34" t="inlineStr">
         <is>
-          <t>HTTP 201 Created. Response contains mar_id.</t>
+          <t>HTTP 422.</t>
         </is>
       </c>
       <c r="F43" s="34" t="inlineStr">
@@ -16688,7 +16688,7 @@
     <row r="44">
       <c r="A44" s="34" t="inlineStr">
         <is>
-          <t>TC-5.7 Step 2</t>
+          <t>TC-5.7 Step 3</t>
         </is>
       </c>
       <c r="B44" s="34" t="inlineStr">
@@ -16703,17 +16703,17 @@
       </c>
       <c r="D44" s="34" t="inlineStr">
         <is>
-          <t>Assert response HTTP status code equals 201.</t>
+          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE tenant_id='tenant-aaa-001' AND status='refused'. Assert count = N (unchanged).</t>
         </is>
       </c>
       <c r="E44" s="34" t="inlineStr">
         <is>
-          <t>HTTP 201 Created.</t>
+          <t>Count = N. No refused MAR row created.</t>
         </is>
       </c>
       <c r="F44" s="34" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="G44" s="34" t="inlineStr">
@@ -16736,59 +16736,27 @@
       <c r="L44" s="34" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="34" t="inlineStr">
-        <is>
-          <t>TC-5.7 Step 3</t>
-        </is>
-      </c>
-      <c r="B45" s="34" t="inlineStr">
-        <is>
-          <t>MARRecord</t>
-        </is>
-      </c>
-      <c r="C45" s="34" t="inlineStr">
-        <is>
-          <t>5.7</t>
-        </is>
-      </c>
-      <c r="D45" s="34" t="inlineStr">
-        <is>
-          <t>Query DB: SELECT status, administered_time FROM mar_record WHERE mar_id=&lt;returned_mar_id&gt;.</t>
-        </is>
-      </c>
-      <c r="E45" s="34" t="inlineStr">
-        <is>
-          <t>status='administered'. administered_time is non-null and matches fixture_scheduled_time.</t>
-        </is>
-      </c>
-      <c r="F45" s="34" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="G45" s="34" t="inlineStr">
-        <is>
-          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
-        </is>
-      </c>
-      <c r="H45" s="34" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I45" s="34" t="inlineStr">
-        <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="J45" s="34" t="n"/>
-      <c r="K45" s="34" t="n"/>
-      <c r="L45" s="34" t="n"/>
+      <c r="A45" s="32" t="inlineStr">
+        <is>
+          <t>TC-5.8 - POST /mar-records with status=held and null notes Returns 422 MAR_MISSING_NOTES; DB Confirms No Row Created | MARRecord</t>
+        </is>
+      </c>
+      <c r="B45" s="36" t="n"/>
+      <c r="C45" s="36" t="n"/>
+      <c r="D45" s="36" t="n"/>
+      <c r="E45" s="36" t="n"/>
+      <c r="F45" s="36" t="n"/>
+      <c r="G45" s="36" t="n"/>
+      <c r="H45" s="36" t="n"/>
+      <c r="I45" s="36" t="n"/>
+      <c r="J45" s="36" t="n"/>
+      <c r="K45" s="37" t="n"/>
+      <c r="L45" s="32" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="32" t="inlineStr">
-        <is>
-          <t>TC-5.8 - POST /mar-records with status=administered and null administered_time Returns 422; DB Confirms No Row Created | MARRecord</t>
+      <c r="A46" s="33" t="inlineStr">
+        <is>
+          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Initial held MAR count captured as N.</t>
         </is>
       </c>
       <c r="B46" s="36" t="n"/>
@@ -16801,30 +16769,62 @@
       <c r="I46" s="36" t="n"/>
       <c r="J46" s="36" t="n"/>
       <c r="K46" s="37" t="n"/>
-      <c r="L46" s="32" t="n"/>
+      <c r="L46" s="33" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="33" t="inlineStr">
-        <is>
-          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Initial MAR count for tenant-aaa-001 captured as N.</t>
-        </is>
-      </c>
-      <c r="B47" s="36" t="n"/>
-      <c r="C47" s="36" t="n"/>
-      <c r="D47" s="36" t="n"/>
-      <c r="E47" s="36" t="n"/>
-      <c r="F47" s="36" t="n"/>
-      <c r="G47" s="36" t="n"/>
-      <c r="H47" s="36" t="n"/>
-      <c r="I47" s="36" t="n"/>
-      <c r="J47" s="36" t="n"/>
-      <c r="K47" s="37" t="n"/>
-      <c r="L47" s="33" t="n"/>
+      <c r="A47" s="34" t="inlineStr">
+        <is>
+          <t>TC-5.8 Step 1</t>
+        </is>
+      </c>
+      <c r="B47" s="34" t="inlineStr">
+        <is>
+          <t>MARRecord</t>
+        </is>
+      </c>
+      <c r="C47" s="34" t="inlineStr">
+        <is>
+          <t>5.8</t>
+        </is>
+      </c>
+      <c r="D47" s="34" t="inlineStr">
+        <is>
+          <t>Send POST /mar-records with status=held and notes=null. All other fields valid.</t>
+        </is>
+      </c>
+      <c r="E47" s="34" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity. notes is required when status=held.</t>
+        </is>
+      </c>
+      <c r="F47" s="34" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G47" s="34" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H47" s="34" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I47" s="34" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J47" s="34" t="n"/>
+      <c r="K47" s="34" t="n"/>
+      <c r="L47" s="34" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="34" t="inlineStr">
         <is>
-          <t>TC-5.8 Step 1</t>
+          <t>TC-5.8 Step 2</t>
         </is>
       </c>
       <c r="B48" s="34" t="inlineStr">
@@ -16839,12 +16839,12 @@
       </c>
       <c r="D48" s="34" t="inlineStr">
         <is>
-          <t>Send POST /mar-records with status=administered and administered_time=null. All other fields valid.</t>
+          <t>Assert response HTTP status code equals 422.</t>
         </is>
       </c>
       <c r="E48" s="34" t="inlineStr">
         <is>
-          <t>HTTP 422 Unprocessable Entity. administered_time is required when status=administered.</t>
+          <t>HTTP 422.</t>
         </is>
       </c>
       <c r="F48" s="34" t="inlineStr">
@@ -16874,7 +16874,7 @@
     <row r="49">
       <c r="A49" s="34" t="inlineStr">
         <is>
-          <t>TC-5.8 Step 2</t>
+          <t>TC-5.8 Step 3</t>
         </is>
       </c>
       <c r="B49" s="34" t="inlineStr">
@@ -16889,17 +16889,17 @@
       </c>
       <c r="D49" s="34" t="inlineStr">
         <is>
-          <t>Assert response HTTP status code equals 422.</t>
+          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE tenant_id='tenant-aaa-001' AND status='held'. Assert count = N (unchanged).</t>
         </is>
       </c>
       <c r="E49" s="34" t="inlineStr">
         <is>
-          <t>HTTP 422.</t>
+          <t>Count = N. No held MAR row created.</t>
         </is>
       </c>
       <c r="F49" s="34" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="G49" s="34" t="inlineStr">
@@ -16922,59 +16922,27 @@
       <c r="L49" s="34" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="34" t="inlineStr">
-        <is>
-          <t>TC-5.8 Step 3</t>
-        </is>
-      </c>
-      <c r="B50" s="34" t="inlineStr">
-        <is>
-          <t>MARRecord</t>
-        </is>
-      </c>
-      <c r="C50" s="34" t="inlineStr">
-        <is>
-          <t>5.8</t>
-        </is>
-      </c>
-      <c r="D50" s="34" t="inlineStr">
-        <is>
-          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE tenant_id='tenant-aaa-001'. Assert count = N (unchanged).</t>
-        </is>
-      </c>
-      <c r="E50" s="34" t="inlineStr">
-        <is>
-          <t>Count = N. No administered MAR row created.</t>
-        </is>
-      </c>
-      <c r="F50" s="34" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="G50" s="34" t="inlineStr">
-        <is>
-          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
-        </is>
-      </c>
-      <c r="H50" s="34" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I50" s="34" t="inlineStr">
-        <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="J50" s="34" t="n"/>
-      <c r="K50" s="34" t="n"/>
-      <c r="L50" s="34" t="n"/>
+      <c r="A50" s="32" t="inlineStr">
+        <is>
+          <t>TC-5.9 - POST /mar-records with Future administered_time Returns 422 ADMIN_TIME_FUTURE; DB Confirms No Row Created | MARRecord</t>
+        </is>
+      </c>
+      <c r="B50" s="36" t="n"/>
+      <c r="C50" s="36" t="n"/>
+      <c r="D50" s="36" t="n"/>
+      <c r="E50" s="36" t="n"/>
+      <c r="F50" s="36" t="n"/>
+      <c r="G50" s="36" t="n"/>
+      <c r="H50" s="36" t="n"/>
+      <c r="I50" s="36" t="n"/>
+      <c r="J50" s="36" t="n"/>
+      <c r="K50" s="37" t="n"/>
+      <c r="L50" s="32" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="32" t="inlineStr">
-        <is>
-          <t>TC-5.9 - POST /mar-records with status=refused and null notes Returns 422; DB Confirms No Row Created | MARRecord</t>
+      <c r="A51" s="33" t="inlineStr">
+        <is>
+          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. All timestamps are fixture-computed at runtime. No hardcoded values. Initial MAR count captured as N.</t>
         </is>
       </c>
       <c r="B51" s="36" t="n"/>
@@ -16987,30 +16955,62 @@
       <c r="I51" s="36" t="n"/>
       <c r="J51" s="36" t="n"/>
       <c r="K51" s="37" t="n"/>
-      <c r="L51" s="32" t="n"/>
+      <c r="L51" s="33" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="33" t="inlineStr">
-        <is>
-          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Initial refused MAR count captured as N.</t>
-        </is>
-      </c>
-      <c r="B52" s="36" t="n"/>
-      <c r="C52" s="36" t="n"/>
-      <c r="D52" s="36" t="n"/>
-      <c r="E52" s="36" t="n"/>
-      <c r="F52" s="36" t="n"/>
-      <c r="G52" s="36" t="n"/>
-      <c r="H52" s="36" t="n"/>
-      <c r="I52" s="36" t="n"/>
-      <c r="J52" s="36" t="n"/>
-      <c r="K52" s="37" t="n"/>
-      <c r="L52" s="33" t="n"/>
+      <c r="A52" s="34" t="inlineStr">
+        <is>
+          <t>TC-5.9 Step 1</t>
+        </is>
+      </c>
+      <c r="B52" s="34" t="inlineStr">
+        <is>
+          <t>MARRecord</t>
+        </is>
+      </c>
+      <c r="C52" s="34" t="inlineStr">
+        <is>
+          <t>5.9</t>
+        </is>
+      </c>
+      <c r="D52" s="34" t="inlineStr">
+        <is>
+          <t>Send POST /mar-records with administered_time set to a future timestamp (fixture_administered_time_future = datetime.now(UTC) + timedelta(hours=1)) and status=administered.</t>
+        </is>
+      </c>
+      <c r="E52" s="34" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity. error_code="ADMIN_TIME_FUTURE".</t>
+        </is>
+      </c>
+      <c r="F52" s="34" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G52" s="34" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H52" s="34" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I52" s="34" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J52" s="34" t="n"/>
+      <c r="K52" s="34" t="n"/>
+      <c r="L52" s="34" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="34" t="inlineStr">
         <is>
-          <t>TC-5.9 Step 1</t>
+          <t>TC-5.9 Step 2</t>
         </is>
       </c>
       <c r="B53" s="34" t="inlineStr">
@@ -17025,12 +17025,12 @@
       </c>
       <c r="D53" s="34" t="inlineStr">
         <is>
-          <t>Send POST /mar-records with status=refused and notes=null. All other fields valid.</t>
+          <t>Assert response HTTP status code equals 422.</t>
         </is>
       </c>
       <c r="E53" s="34" t="inlineStr">
         <is>
-          <t>HTTP 422 Unprocessable Entity. notes is required when status=refused.</t>
+          <t>HTTP 422.</t>
         </is>
       </c>
       <c r="F53" s="34" t="inlineStr">
@@ -17060,7 +17060,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TC-5.9 Step 2</t>
+          <t>TC-5.9 Step 3</t>
         </is>
       </c>
       <c r="B54" s="34" t="inlineStr">
@@ -17075,12 +17075,12 @@
       </c>
       <c r="D54" s="34" t="inlineStr">
         <is>
-          <t>Assert response HTTP status code equals 422.</t>
+          <t>Assert detail.error_code = "ADMIN_TIME_FUTURE".</t>
         </is>
       </c>
       <c r="E54" s="34" t="inlineStr">
         <is>
-          <t>HTTP 422.</t>
+          <t>detail.error_code="ADMIN_TIME_FUTURE".</t>
         </is>
       </c>
       <c r="F54" s="34" t="inlineStr">
@@ -17110,7 +17110,7 @@
     <row r="55">
       <c r="A55" s="34" t="inlineStr">
         <is>
-          <t>TC-5.9 Step 3</t>
+          <t>TC-5.9 Step 4</t>
         </is>
       </c>
       <c r="B55" s="34" t="inlineStr">
@@ -17125,12 +17125,12 @@
       </c>
       <c r="D55" s="34" t="inlineStr">
         <is>
-          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE tenant_id='tenant-aaa-001' AND status='refused'. Assert count = N (unchanged).</t>
+          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE tenant_id='tenant-aaa-001'. Assert count = N (unchanged).</t>
         </is>
       </c>
       <c r="E55" s="34" t="inlineStr">
         <is>
-          <t>Count = N. No refused MAR row created.</t>
+          <t>Count = N. No row created.</t>
         </is>
       </c>
       <c r="F55" s="34" t="inlineStr">
@@ -17160,7 +17160,7 @@
     <row r="56">
       <c r="A56" s="32" t="inlineStr">
         <is>
-          <t>TC-5.10 - POST /mar-records with status=held and null notes Returns 422; DB Confirms No Row Created | MARRecord</t>
+          <t>TC-5.10 - POST /mar-records with administered_time More Than 2 Hours Before scheduled_time Returns 422 ADMIN_TIME_TOO_EARLY; DB Confirms No Row Created | MARRecord</t>
         </is>
       </c>
       <c r="B56" s="36" t="n"/>
@@ -17178,7 +17178,7 @@
     <row r="57">
       <c r="A57" s="33" t="inlineStr">
         <is>
-          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Initial held MAR count captured as N.</t>
+          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. scheduled_time="fixture_scheduled_time". 2h window boundary: fixture_scheduled_time minus timedelta(hours=2). Initial MAR count captured as N.</t>
         </is>
       </c>
       <c r="B57" s="36" t="n"/>
@@ -17211,12 +17211,12 @@
       </c>
       <c r="D58" s="34" t="inlineStr">
         <is>
-          <t>Send POST /mar-records with status=held and notes=null. All other fields valid.</t>
+          <t>Send POST /mar-records with administered_time=fixture_administered_time_too_early (3 hours before scheduled_time, outside 2h window) and status=administered.</t>
         </is>
       </c>
       <c r="E58" s="34" t="inlineStr">
         <is>
-          <t>HTTP 422 Unprocessable Entity. notes is required when status=held.</t>
+          <t>HTTP 422 Unprocessable Entity. error_code="ADMIN_TIME_TOO_EARLY".</t>
         </is>
       </c>
       <c r="F58" s="34" t="inlineStr">
@@ -17311,17 +17311,17 @@
       </c>
       <c r="D60" s="34" t="inlineStr">
         <is>
-          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE tenant_id='tenant-aaa-001' AND status='held'. Assert count = N (unchanged).</t>
+          <t>Assert detail.error_code = "ADMIN_TIME_TOO_EARLY".</t>
         </is>
       </c>
       <c r="E60" s="34" t="inlineStr">
         <is>
-          <t>Count = N. No held MAR row created.</t>
+          <t>detail.error_code="ADMIN_TIME_TOO_EARLY".</t>
         </is>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>API</t>
         </is>
       </c>
       <c r="G60" s="34" t="inlineStr">
@@ -17344,27 +17344,59 @@
       <c r="L60" s="34" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="32" t="inlineStr">
-        <is>
-          <t>TC-5.11 - POST /mar-records with administered_time Within Valid 2-Hour Window Before scheduled_time Returns 201; DB Confirms Correct administered_time | MARRecord</t>
-        </is>
-      </c>
-      <c r="B61" s="36" t="n"/>
-      <c r="C61" s="36" t="n"/>
-      <c r="D61" s="36" t="n"/>
-      <c r="E61" s="36" t="n"/>
-      <c r="F61" s="36" t="n"/>
-      <c r="G61" s="36" t="n"/>
-      <c r="H61" s="36" t="n"/>
-      <c r="I61" s="36" t="n"/>
-      <c r="J61" s="36" t="n"/>
-      <c r="K61" s="37" t="n"/>
-      <c r="L61" s="32" t="n"/>
+      <c r="A61" s="34" t="inlineStr">
+        <is>
+          <t>TC-5.10 Step 4</t>
+        </is>
+      </c>
+      <c r="B61" s="34" t="inlineStr">
+        <is>
+          <t>MARRecord</t>
+        </is>
+      </c>
+      <c r="C61" s="34" t="inlineStr">
+        <is>
+          <t>5.10</t>
+        </is>
+      </c>
+      <c r="D61" s="34" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE tenant_id='tenant-aaa-001'. Assert count = N (unchanged).</t>
+        </is>
+      </c>
+      <c r="E61" s="34" t="inlineStr">
+        <is>
+          <t>Count = N. No row created.</t>
+        </is>
+      </c>
+      <c r="F61" s="34" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G61" s="34" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H61" s="34" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I61" s="34" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J61" s="34" t="n"/>
+      <c r="K61" s="34" t="n"/>
+      <c r="L61" s="34" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="33" t="inlineStr">
-        <is>
-          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Participant P1 exists. scheduled_time="fixture_scheduled_time". Valid window: administered_time &gt;= fixture_scheduled_time minus timedelta(hours=2).</t>
+      <c r="A62" s="32" t="inlineStr">
+        <is>
+          <t>TC-5.11 - POST /mar-records with administered_by Referencing Non-Nurse Role User Returns 403; DB Confirms No Row Created | MARRecord</t>
         </is>
       </c>
       <c r="B62" s="36" t="n"/>
@@ -17377,62 +17409,30 @@
       <c r="I62" s="36" t="n"/>
       <c r="J62" s="36" t="n"/>
       <c r="K62" s="37" t="n"/>
-      <c r="L62" s="33" t="n"/>
+      <c r="L62" s="32" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="34" t="inlineStr">
-        <is>
-          <t>TC-5.11 Step 1</t>
-        </is>
-      </c>
-      <c r="B63" s="34" t="inlineStr">
-        <is>
-          <t>MARRecord</t>
-        </is>
-      </c>
-      <c r="C63" s="34" t="inlineStr">
-        <is>
-          <t>5.11</t>
-        </is>
-      </c>
-      <c r="D63" s="34" t="inlineStr">
-        <is>
-          <t>Send POST /mar-records with administered_time=fixture_administered_time (1h30m before scheduled_time, within 2h window) and status=administered.</t>
-        </is>
-      </c>
-      <c r="E63" s="34" t="inlineStr">
-        <is>
-          <t>HTTP 201 Created. Response contains mar_id.</t>
-        </is>
-      </c>
-      <c r="F63" s="34" t="inlineStr">
-        <is>
-          <t>API</t>
-        </is>
-      </c>
-      <c r="G63" s="34" t="inlineStr">
-        <is>
-          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
-        </is>
-      </c>
-      <c r="H63" s="34" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I63" s="34" t="inlineStr">
-        <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="J63" s="34" t="n"/>
-      <c r="K63" s="34" t="n"/>
-      <c r="L63" s="34" t="n"/>
+      <c r="A63" s="33" t="inlineStr">
+        <is>
+          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Participant P1 exists. scheduled_time="fixture_scheduled_time". Valid window: administered_time &gt;= fixture_scheduled_time minus timedelta(hours=2).</t>
+        </is>
+      </c>
+      <c r="B63" s="36" t="n"/>
+      <c r="C63" s="36" t="n"/>
+      <c r="D63" s="36" t="n"/>
+      <c r="E63" s="36" t="n"/>
+      <c r="F63" s="36" t="n"/>
+      <c r="G63" s="36" t="n"/>
+      <c r="H63" s="36" t="n"/>
+      <c r="I63" s="36" t="n"/>
+      <c r="J63" s="36" t="n"/>
+      <c r="K63" s="37" t="n"/>
+      <c r="L63" s="33" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="34" t="inlineStr">
         <is>
-          <t>TC-5.11 Step 2</t>
+          <t>TC-5.11 Step 1</t>
         </is>
       </c>
       <c r="B64" s="34" t="inlineStr">
@@ -17447,12 +17447,12 @@
       </c>
       <c r="D64" s="34" t="inlineStr">
         <is>
-          <t>Assert response HTTP status code equals 201.</t>
+          <t>Send POST /mar-records with administered_time=fixture_administered_time (1h30m before scheduled_time, within 2h window) and status=administered.</t>
         </is>
       </c>
       <c r="E64" s="34" t="inlineStr">
         <is>
-          <t>HTTP 201 Created.</t>
+          <t>HTTP 201 Created. Response contains mar_id.</t>
         </is>
       </c>
       <c r="F64" s="34" t="inlineStr">
@@ -17482,7 +17482,7 @@
     <row r="65">
       <c r="A65" s="34" t="inlineStr">
         <is>
-          <t>TC-5.11 Step 3</t>
+          <t>TC-5.11 Step 2</t>
         </is>
       </c>
       <c r="B65" s="34" t="inlineStr">
@@ -17497,17 +17497,17 @@
       </c>
       <c r="D65" s="34" t="inlineStr">
         <is>
-          <t>Query DB: SELECT administered_time FROM mar_record WHERE mar_id=&lt;returned_mar_id&gt;.</t>
+          <t>Assert response HTTP status code equals 201.</t>
         </is>
       </c>
       <c r="E65" s="34" t="inlineStr">
         <is>
-          <t>administered_time=fixture_administered_time. Correct administered_time persisted.</t>
+          <t>HTTP 201 Created.</t>
         </is>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>API</t>
         </is>
       </c>
       <c r="G65" s="34" t="inlineStr">
@@ -17530,27 +17530,59 @@
       <c r="L65" s="34" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="32" t="inlineStr">
-        <is>
-          <t>TC-5.12 - POST /mar-records with Future administered_time Returns 422 ADMIN_TIME_FUTURE; DB Confirms No Row Created | MARRecord</t>
-        </is>
-      </c>
-      <c r="B66" s="36" t="n"/>
-      <c r="C66" s="36" t="n"/>
-      <c r="D66" s="36" t="n"/>
-      <c r="E66" s="36" t="n"/>
-      <c r="F66" s="36" t="n"/>
-      <c r="G66" s="36" t="n"/>
-      <c r="H66" s="36" t="n"/>
-      <c r="I66" s="36" t="n"/>
-      <c r="J66" s="36" t="n"/>
-      <c r="K66" s="37" t="n"/>
-      <c r="L66" s="32" t="n"/>
+      <c r="A66" s="34" t="inlineStr">
+        <is>
+          <t>TC-5.11 Step 3</t>
+        </is>
+      </c>
+      <c r="B66" s="34" t="inlineStr">
+        <is>
+          <t>MARRecord</t>
+        </is>
+      </c>
+      <c r="C66" s="34" t="inlineStr">
+        <is>
+          <t>5.11</t>
+        </is>
+      </c>
+      <c r="D66" s="34" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT administered_time FROM mar_record WHERE mar_id=&lt;returned_mar_id&gt;.</t>
+        </is>
+      </c>
+      <c r="E66" s="34" t="inlineStr">
+        <is>
+          <t>administered_time=fixture_administered_time. Correct administered_time persisted.</t>
+        </is>
+      </c>
+      <c r="F66" s="34" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G66" s="34" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H66" s="34" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I66" s="34" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J66" s="34" t="n"/>
+      <c r="K66" s="34" t="n"/>
+      <c r="L66" s="34" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="33" t="inlineStr">
-        <is>
-          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. All timestamps are fixture-computed at runtime. No hardcoded values. Initial MAR count captured as N.</t>
+      <c r="A67" s="32" t="inlineStr">
+        <is>
+          <t>TC-5.12 - POST /mar-records with administered_by Referencing Non-Existent user_id Returns 403 or 422; DB Confirms No Row Created | MARRecord</t>
         </is>
       </c>
       <c r="B67" s="36" t="n"/>
@@ -17563,62 +17595,30 @@
       <c r="I67" s="36" t="n"/>
       <c r="J67" s="36" t="n"/>
       <c r="K67" s="37" t="n"/>
-      <c r="L67" s="33" t="n"/>
+      <c r="L67" s="32" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="34" t="inlineStr">
-        <is>
-          <t>TC-5.12 Step 1</t>
-        </is>
-      </c>
-      <c r="B68" s="34" t="inlineStr">
-        <is>
-          <t>MARRecord</t>
-        </is>
-      </c>
-      <c r="C68" s="34" t="inlineStr">
-        <is>
-          <t>5.12</t>
-        </is>
-      </c>
-      <c r="D68" s="34" t="inlineStr">
-        <is>
-          <t>Send POST /mar-records with administered_time set to a future timestamp (fixture_administered_time_future = datetime.now(UTC) + timedelta(hours=1)) and status=administered.</t>
-        </is>
-      </c>
-      <c r="E68" s="34" t="inlineStr">
-        <is>
-          <t>HTTP 422 Unprocessable Entity. error_code="ADMIN_TIME_FUTURE".</t>
-        </is>
-      </c>
-      <c r="F68" s="34" t="inlineStr">
-        <is>
-          <t>API</t>
-        </is>
-      </c>
-      <c r="G68" s="34" t="inlineStr">
-        <is>
-          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
-        </is>
-      </c>
-      <c r="H68" s="34" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I68" s="34" t="inlineStr">
-        <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="J68" s="34" t="n"/>
-      <c r="K68" s="34" t="n"/>
-      <c r="L68" s="34" t="n"/>
+      <c r="A68" s="33" t="inlineStr">
+        <is>
+          <t>Preconditions: A controlled-substance mar_record exists in tenant-aaa-001 (mar_id known, is_controlled_substance=true). care_coordinator (X-User-Id: user-cc-001, X-Session-Id: sess-tc56) authenticated.</t>
+        </is>
+      </c>
+      <c r="B68" s="36" t="n"/>
+      <c r="C68" s="36" t="n"/>
+      <c r="D68" s="36" t="n"/>
+      <c r="E68" s="36" t="n"/>
+      <c r="F68" s="36" t="n"/>
+      <c r="G68" s="36" t="n"/>
+      <c r="H68" s="36" t="n"/>
+      <c r="I68" s="36" t="n"/>
+      <c r="J68" s="36" t="n"/>
+      <c r="K68" s="37" t="n"/>
+      <c r="L68" s="33" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="34" t="inlineStr">
         <is>
-          <t>TC-5.12 Step 2</t>
+          <t>TC-5.12 Step 1</t>
         </is>
       </c>
       <c r="B69" s="34" t="inlineStr">
@@ -17633,12 +17633,12 @@
       </c>
       <c r="D69" s="34" t="inlineStr">
         <is>
-          <t>Assert response HTTP status code equals 422.</t>
+          <t>Send GET /mar-records/&lt;mar_id&gt; with care_coordinator headers (unauthorized for controlled-substance access).</t>
         </is>
       </c>
       <c r="E69" s="34" t="inlineStr">
         <is>
-          <t>HTTP 422.</t>
+          <t>HTTP 403 Forbidden.</t>
         </is>
       </c>
       <c r="F69" s="34" t="inlineStr">
@@ -17648,7 +17648,7 @@
       </c>
       <c r="G69" s="34" t="inlineStr">
         <is>
-          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+          <t>HIPAA §164.312(a)(2)(iv); 42 CFR Part 2; CMS Medicaid/Medicare</t>
         </is>
       </c>
       <c r="H69" s="34" t="inlineStr">
@@ -17668,7 +17668,7 @@
     <row r="70">
       <c r="A70" s="34" t="inlineStr">
         <is>
-          <t>TC-5.12 Step 3</t>
+          <t>TC-5.12 Step 2</t>
         </is>
       </c>
       <c r="B70" s="34" t="inlineStr">
@@ -17683,22 +17683,22 @@
       </c>
       <c r="D70" s="34" t="inlineStr">
         <is>
-          <t>Assert detail.error_code = "ADMIN_TIME_FUTURE".</t>
+          <t>Query DB: SELECT * FROM audit_log WHERE resource_id=&lt;mar_id&gt; AND event_type='ACCESS_DENIED'. Assert row exists. No time.sleep() before query.</t>
         </is>
       </c>
       <c r="E70" s="34" t="inlineStr">
         <is>
-          <t>detail.error_code="ADMIN_TIME_FUTURE".</t>
+          <t>ACCESS_DENIED audit event row found for this resource.</t>
         </is>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="G70" s="34" t="inlineStr">
         <is>
-          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+          <t>HIPAA §164.312(b); 42 CFR Part 2</t>
         </is>
       </c>
       <c r="H70" s="34" t="inlineStr">
@@ -17718,7 +17718,7 @@
     <row r="71">
       <c r="A71" s="34" t="inlineStr">
         <is>
-          <t>TC-5.12 Step 4</t>
+          <t>TC-5.12 Step 3</t>
         </is>
       </c>
       <c r="B71" s="34" t="inlineStr">
@@ -17733,12 +17733,12 @@
       </c>
       <c r="D71" s="34" t="inlineStr">
         <is>
-          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE tenant_id='tenant-aaa-001'. Assert count = N (unchanged).</t>
+          <t>Assert all 11 mandatory fields non-null on the ACCESS_DENIED row: event_id, event_type, timestamp, user_id, tenant_id, resource_type, resource_id, action, data_affected, session_id, ip_address.</t>
         </is>
       </c>
       <c r="E71" s="34" t="inlineStr">
         <is>
-          <t>Count = N. No row created.</t>
+          <t>All 11 mandatory audit fields are non-null.</t>
         </is>
       </c>
       <c r="F71" s="34" t="inlineStr">
@@ -17748,7 +17748,7 @@
       </c>
       <c r="G71" s="34" t="inlineStr">
         <is>
-          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+          <t>HIPAA §164.312(b); 42 CFR Part 2</t>
         </is>
       </c>
       <c r="H71" s="34" t="inlineStr">
@@ -17766,27 +17766,59 @@
       <c r="L71" s="34" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="32" t="inlineStr">
-        <is>
-          <t>TC-5.13 - POST /mar-records with administered_time More Than 2 Hours Before scheduled_time Returns 422 ADMIN_TIME_TOO_EARLY; DB Confirms No Row Created | MARRecord</t>
-        </is>
-      </c>
-      <c r="B72" s="36" t="n"/>
-      <c r="C72" s="36" t="n"/>
-      <c r="D72" s="36" t="n"/>
-      <c r="E72" s="36" t="n"/>
-      <c r="F72" s="36" t="n"/>
-      <c r="G72" s="36" t="n"/>
-      <c r="H72" s="36" t="n"/>
-      <c r="I72" s="36" t="n"/>
-      <c r="J72" s="36" t="n"/>
-      <c r="K72" s="37" t="n"/>
-      <c r="L72" s="32" t="n"/>
+      <c r="A72" s="34" t="inlineStr">
+        <is>
+          <t>TC-5.12 Step 4</t>
+        </is>
+      </c>
+      <c r="B72" s="34" t="inlineStr">
+        <is>
+          <t>MARRecord</t>
+        </is>
+      </c>
+      <c r="C72" s="34" t="inlineStr">
+        <is>
+          <t>5.12</t>
+        </is>
+      </c>
+      <c r="D72" s="34" t="inlineStr">
+        <is>
+          <t>Assert data_affected contains no raw PHI values (no medication_name, participant_id, administered_time literals).</t>
+        </is>
+      </c>
+      <c r="E72" s="34" t="inlineStr">
+        <is>
+          <t>data_affected contains no raw PHI.</t>
+        </is>
+      </c>
+      <c r="F72" s="34" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G72" s="34" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(b); 42 CFR Part 2</t>
+        </is>
+      </c>
+      <c r="H72" s="34" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I72" s="34" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J72" s="34" t="n"/>
+      <c r="K72" s="34" t="n"/>
+      <c r="L72" s="34" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="33" t="inlineStr">
-        <is>
-          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. scheduled_time="fixture_scheduled_time". 2h window boundary: fixture_scheduled_time minus timedelta(hours=2). Initial MAR count captured as N.</t>
+      <c r="A73" s="32" t="inlineStr">
+        <is>
+          <t>TC-5.13 - POST /mar-records by care_coordinator Returns 403 RBAC_DENIED; DB Confirms No Row Created | MARRecord</t>
         </is>
       </c>
       <c r="B73" s="36" t="n"/>
@@ -17799,62 +17831,30 @@
       <c r="I73" s="36" t="n"/>
       <c r="J73" s="36" t="n"/>
       <c r="K73" s="37" t="n"/>
-      <c r="L73" s="33" t="n"/>
+      <c r="L73" s="32" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="34" t="inlineStr">
-        <is>
-          <t>TC-5.13 Step 1</t>
-        </is>
-      </c>
-      <c r="B74" s="34" t="inlineStr">
-        <is>
-          <t>MARRecord</t>
-        </is>
-      </c>
-      <c r="C74" s="34" t="inlineStr">
-        <is>
-          <t>5.13</t>
-        </is>
-      </c>
-      <c r="D74" s="34" t="inlineStr">
-        <is>
-          <t>Send POST /mar-records with administered_time=fixture_administered_time_too_early (3 hours before scheduled_time, outside 2h window) and status=administered.</t>
-        </is>
-      </c>
-      <c r="E74" s="34" t="inlineStr">
-        <is>
-          <t>HTTP 422 Unprocessable Entity. error_code="ADMIN_TIME_TOO_EARLY".</t>
-        </is>
-      </c>
-      <c r="F74" s="34" t="inlineStr">
-        <is>
-          <t>API</t>
-        </is>
-      </c>
-      <c r="G74" s="34" t="inlineStr">
-        <is>
-          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
-        </is>
-      </c>
-      <c r="H74" s="34" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I74" s="34" t="inlineStr">
-        <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="J74" s="34" t="n"/>
-      <c r="K74" s="34" t="n"/>
-      <c r="L74" s="34" t="n"/>
+      <c r="A74" s="33" t="inlineStr">
+        <is>
+          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Three distinct scheduled_times (fixture_scheduled_time_oral, 09:00:00, 10:00:00) used to avoid duplicate-event conflicts.</t>
+        </is>
+      </c>
+      <c r="B74" s="36" t="n"/>
+      <c r="C74" s="36" t="n"/>
+      <c r="D74" s="36" t="n"/>
+      <c r="E74" s="36" t="n"/>
+      <c r="F74" s="36" t="n"/>
+      <c r="G74" s="36" t="n"/>
+      <c r="H74" s="36" t="n"/>
+      <c r="I74" s="36" t="n"/>
+      <c r="J74" s="36" t="n"/>
+      <c r="K74" s="37" t="n"/>
+      <c r="L74" s="33" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="34" t="inlineStr">
         <is>
-          <t>TC-5.13 Step 2</t>
+          <t>TC-5.13 Step 1</t>
         </is>
       </c>
       <c r="B75" s="34" t="inlineStr">
@@ -17869,12 +17869,12 @@
       </c>
       <c r="D75" s="34" t="inlineStr">
         <is>
-          <t>Assert response HTTP status code equals 422.</t>
+          <t>Send POST /mar-records with route="oral", scheduled_time="fixture_scheduled_time_oral", all other fields valid.</t>
         </is>
       </c>
       <c r="E75" s="34" t="inlineStr">
         <is>
-          <t>HTTP 422.</t>
+          <t>HTTP 201 Created.</t>
         </is>
       </c>
       <c r="F75" s="34" t="inlineStr">
@@ -17889,7 +17889,7 @@
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I75" s="34" t="inlineStr">
@@ -17904,7 +17904,7 @@
     <row r="76">
       <c r="A76" s="34" t="inlineStr">
         <is>
-          <t>TC-5.13 Step 3</t>
+          <t>TC-5.13 Step 2</t>
         </is>
       </c>
       <c r="B76" s="34" t="inlineStr">
@@ -17919,12 +17919,12 @@
       </c>
       <c r="D76" s="34" t="inlineStr">
         <is>
-          <t>Assert detail.error_code = "ADMIN_TIME_TOO_EARLY".</t>
+          <t>Send POST /mar-records with route="injection", scheduled_time="fixture_scheduled_time_injection", all other fields valid.</t>
         </is>
       </c>
       <c r="E76" s="34" t="inlineStr">
         <is>
-          <t>detail.error_code="ADMIN_TIME_TOO_EARLY".</t>
+          <t>HTTP 201 Created.</t>
         </is>
       </c>
       <c r="F76" s="34" t="inlineStr">
@@ -17939,7 +17939,7 @@
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I76" s="34" t="inlineStr">
@@ -17954,7 +17954,7 @@
     <row r="77">
       <c r="A77" s="34" t="inlineStr">
         <is>
-          <t>TC-5.13 Step 4</t>
+          <t>TC-5.13 Step 3</t>
         </is>
       </c>
       <c r="B77" s="34" t="inlineStr">
@@ -17969,17 +17969,17 @@
       </c>
       <c r="D77" s="34" t="inlineStr">
         <is>
-          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE tenant_id='tenant-aaa-001'. Assert count = N (unchanged).</t>
+          <t>Send POST /mar-records with route="topical", scheduled_time="fixture_scheduled_time_topical", all other fields valid.</t>
         </is>
       </c>
       <c r="E77" s="34" t="inlineStr">
         <is>
-          <t>Count = N. No row created.</t>
+          <t>HTTP 201 Created.</t>
         </is>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>API</t>
         </is>
       </c>
       <c r="G77" s="34" t="inlineStr">
@@ -17989,7 +17989,7 @@
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I77" s="34" t="inlineStr">
@@ -18002,27 +18002,59 @@
       <c r="L77" s="34" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="32" t="inlineStr">
-        <is>
-          <t>TC-5.14 - POST /mar-records with route=oral Returns 201; route=injection Returns 201; route=topical Returns 201; DB Confirms Row Created in Each Case | MARRecord</t>
-        </is>
-      </c>
-      <c r="B78" s="36" t="n"/>
-      <c r="C78" s="36" t="n"/>
-      <c r="D78" s="36" t="n"/>
-      <c r="E78" s="36" t="n"/>
-      <c r="F78" s="36" t="n"/>
-      <c r="G78" s="36" t="n"/>
-      <c r="H78" s="36" t="n"/>
-      <c r="I78" s="36" t="n"/>
-      <c r="J78" s="36" t="n"/>
-      <c r="K78" s="37" t="n"/>
-      <c r="L78" s="32" t="n"/>
+      <c r="A78" s="34" t="inlineStr">
+        <is>
+          <t>TC-5.13 Step 4</t>
+        </is>
+      </c>
+      <c r="B78" s="34" t="inlineStr">
+        <is>
+          <t>MARRecord</t>
+        </is>
+      </c>
+      <c r="C78" s="34" t="inlineStr">
+        <is>
+          <t>5.13</t>
+        </is>
+      </c>
+      <c r="D78" s="34" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE tenant_id='tenant-aaa-001' AND route IN ('oral','injection','topical') AND scheduled_time IN ('fixture_scheduled_time_oral','fixture_scheduled_time_injection','fixture_scheduled_time_topical'). Assert count &gt;= 3.</t>
+        </is>
+      </c>
+      <c r="E78" s="34" t="inlineStr">
+        <is>
+          <t>Count &gt;= 3. All three rows persisted with correct route values.</t>
+        </is>
+      </c>
+      <c r="F78" s="34" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G78" s="34" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H78" s="34" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I78" s="34" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J78" s="34" t="n"/>
+      <c r="K78" s="34" t="n"/>
+      <c r="L78" s="34" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="33" t="inlineStr">
-        <is>
-          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Three distinct scheduled_times (fixture_scheduled_time_oral, 09:00:00, 10:00:00) used to avoid duplicate-event conflicts.</t>
+      <c r="A79" s="32" t="inlineStr">
+        <is>
+          <t>TC-5.14 - PATCH on MARRecord with status=administered Returns 422 MAR_ADMINISTERED_IMMUTABLE for Any Field Change; DB Confirms version Unchanged | MARRecord</t>
         </is>
       </c>
       <c r="B79" s="36" t="n"/>
@@ -18035,62 +18067,30 @@
       <c r="I79" s="36" t="n"/>
       <c r="J79" s="36" t="n"/>
       <c r="K79" s="37" t="n"/>
-      <c r="L79" s="33" t="n"/>
+      <c r="L79" s="32" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="34" t="inlineStr">
-        <is>
-          <t>TC-5.14 Step 1</t>
-        </is>
-      </c>
-      <c r="B80" s="34" t="inlineStr">
-        <is>
-          <t>MARRecord</t>
-        </is>
-      </c>
-      <c r="C80" s="34" t="inlineStr">
-        <is>
-          <t>5.14</t>
-        </is>
-      </c>
-      <c r="D80" s="34" t="inlineStr">
-        <is>
-          <t>Send POST /mar-records with route="oral", scheduled_time="fixture_scheduled_time_oral", all other fields valid.</t>
-        </is>
-      </c>
-      <c r="E80" s="34" t="inlineStr">
-        <is>
-          <t>HTTP 201 Created.</t>
-        </is>
-      </c>
-      <c r="F80" s="34" t="inlineStr">
-        <is>
-          <t>API</t>
-        </is>
-      </c>
-      <c r="G80" s="34" t="inlineStr">
-        <is>
-          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
-        </is>
-      </c>
-      <c r="H80" s="34" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I80" s="34" t="inlineStr">
-        <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="J80" s="34" t="n"/>
-      <c r="K80" s="34" t="n"/>
-      <c r="L80" s="34" t="n"/>
+      <c r="A80" s="33" t="inlineStr">
+        <is>
+          <t>Preconditions: A mar_record with status=administered, version=1, notes=null exists in tenant-aaa-001. nurse_medication_aide authenticated.</t>
+        </is>
+      </c>
+      <c r="B80" s="36" t="n"/>
+      <c r="C80" s="36" t="n"/>
+      <c r="D80" s="36" t="n"/>
+      <c r="E80" s="36" t="n"/>
+      <c r="F80" s="36" t="n"/>
+      <c r="G80" s="36" t="n"/>
+      <c r="H80" s="36" t="n"/>
+      <c r="I80" s="36" t="n"/>
+      <c r="J80" s="36" t="n"/>
+      <c r="K80" s="37" t="n"/>
+      <c r="L80" s="33" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="34" t="inlineStr">
         <is>
-          <t>TC-5.14 Step 2</t>
+          <t>TC-5.14 Step 1</t>
         </is>
       </c>
       <c r="B81" s="34" t="inlineStr">
@@ -18105,17 +18105,17 @@
       </c>
       <c r="D81" s="34" t="inlineStr">
         <is>
-          <t>Send POST /mar-records with route="injection", scheduled_time="fixture_scheduled_time_injection", all other fields valid.</t>
+          <t>Query DB: SELECT status, version, notes FROM mar_record WHERE mar_id=&lt;mar_id&gt;. Confirm status='administered', version=1.</t>
         </is>
       </c>
       <c r="E81" s="34" t="inlineStr">
         <is>
-          <t>HTTP 201 Created.</t>
+          <t>status='administered', version=1, notes=null confirmed.</t>
         </is>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="G81" s="34" t="inlineStr">
@@ -18125,7 +18125,7 @@
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I81" s="34" t="inlineStr">
@@ -18140,7 +18140,7 @@
     <row r="82">
       <c r="A82" s="34" t="inlineStr">
         <is>
-          <t>TC-5.14 Step 3</t>
+          <t>TC-5.14 Step 2</t>
         </is>
       </c>
       <c r="B82" s="34" t="inlineStr">
@@ -18155,12 +18155,12 @@
       </c>
       <c r="D82" s="34" t="inlineStr">
         <is>
-          <t>Send POST /mar-records with route="topical", scheduled_time="fixture_scheduled_time_topical", all other fields valid.</t>
+          <t>Send PATCH /mar-records/&lt;mar_id&gt; with {"notes": "post-admin update"} and nurse_medication_aide headers.</t>
         </is>
       </c>
       <c r="E82" s="34" t="inlineStr">
         <is>
-          <t>HTTP 201 Created.</t>
+          <t>HTTP 422 Unprocessable Entity. Administered records are immutable.</t>
         </is>
       </c>
       <c r="F82" s="34" t="inlineStr">
@@ -18175,7 +18175,7 @@
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I82" s="34" t="inlineStr">
@@ -18190,7 +18190,7 @@
     <row r="83">
       <c r="A83" s="34" t="inlineStr">
         <is>
-          <t>TC-5.14 Step 4</t>
+          <t>TC-5.14 Step 3</t>
         </is>
       </c>
       <c r="B83" s="34" t="inlineStr">
@@ -18205,17 +18205,17 @@
       </c>
       <c r="D83" s="34" t="inlineStr">
         <is>
-          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE tenant_id='tenant-aaa-001' AND route IN ('oral','injection','topical') AND scheduled_time IN ('fixture_scheduled_time_oral','fixture_scheduled_time_injection','fixture_scheduled_time_topical'). Assert count &gt;= 3.</t>
+          <t>Assert response HTTP status code equals 422.</t>
         </is>
       </c>
       <c r="E83" s="34" t="inlineStr">
         <is>
-          <t>Count &gt;= 3. All three rows persisted with correct route values.</t>
+          <t>HTTP 422.</t>
         </is>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>API</t>
         </is>
       </c>
       <c r="G83" s="34" t="inlineStr">
@@ -18225,7 +18225,7 @@
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I83" s="34" t="inlineStr">
@@ -18238,27 +18238,59 @@
       <c r="L83" s="34" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="32" t="inlineStr">
-        <is>
-          <t>TC-5.15 - POST /mar-records with Invalid route Returns 400; POST with null route Returns 400; DB Confirms No Row Created in Either Case | MARRecord</t>
-        </is>
-      </c>
-      <c r="B84" s="36" t="n"/>
-      <c r="C84" s="36" t="n"/>
-      <c r="D84" s="36" t="n"/>
-      <c r="E84" s="36" t="n"/>
-      <c r="F84" s="36" t="n"/>
-      <c r="G84" s="36" t="n"/>
-      <c r="H84" s="36" t="n"/>
-      <c r="I84" s="36" t="n"/>
-      <c r="J84" s="36" t="n"/>
-      <c r="K84" s="37" t="n"/>
-      <c r="L84" s="32" t="n"/>
+      <c r="A84" s="34" t="inlineStr">
+        <is>
+          <t>TC-5.14 Step 4</t>
+        </is>
+      </c>
+      <c r="B84" s="34" t="inlineStr">
+        <is>
+          <t>MARRecord</t>
+        </is>
+      </c>
+      <c r="C84" s="34" t="inlineStr">
+        <is>
+          <t>5.14</t>
+        </is>
+      </c>
+      <c r="D84" s="34" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT status, version, notes FROM mar_record WHERE mar_id=&lt;mar_id&gt;. Assert all fields identical to pre-PATCH state.</t>
+        </is>
+      </c>
+      <c r="E84" s="34" t="inlineStr">
+        <is>
+          <t>status='administered', version=1, notes=null. All fields unchanged.</t>
+        </is>
+      </c>
+      <c r="F84" s="34" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G84" s="34" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H84" s="34" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I84" s="34" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J84" s="34" t="n"/>
+      <c r="K84" s="34" t="n"/>
+      <c r="L84" s="34" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="33" t="inlineStr">
-        <is>
-          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Initial MAR count captured as N.</t>
+      <c r="A85" s="32" t="inlineStr">
+        <is>
+          <t>TC-5.15 - PATCH Administered MAR Immutability Check Fires Before Version Check; 422 MAR_ADMINISTERED_IMMUTABLE Even with Stale version Supplied | MARRecord</t>
         </is>
       </c>
       <c r="B85" s="36" t="n"/>
@@ -18271,62 +18303,30 @@
       <c r="I85" s="36" t="n"/>
       <c r="J85" s="36" t="n"/>
       <c r="K85" s="37" t="n"/>
-      <c r="L85" s="33" t="n"/>
+      <c r="L85" s="32" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="34" t="inlineStr">
-        <is>
-          <t>TC-5.15 Step 1</t>
-        </is>
-      </c>
-      <c r="B86" s="34" t="inlineStr">
-        <is>
-          <t>MARRecord</t>
-        </is>
-      </c>
-      <c r="C86" s="34" t="inlineStr">
-        <is>
-          <t>5.15</t>
-        </is>
-      </c>
-      <c r="D86" s="34" t="inlineStr">
-        <is>
-          <t>Send POST /mar-records with route="intravenous" (invalid enum value). All other fields valid.</t>
-        </is>
-      </c>
-      <c r="E86" s="34" t="inlineStr">
-        <is>
-          <t>HTTP 400 Bad Request. Invalid route value rejected.</t>
-        </is>
-      </c>
-      <c r="F86" s="34" t="inlineStr">
-        <is>
-          <t>API</t>
-        </is>
-      </c>
-      <c r="G86" s="34" t="inlineStr">
-        <is>
-          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
-        </is>
-      </c>
-      <c r="H86" s="34" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I86" s="34" t="inlineStr">
-        <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="J86" s="34" t="n"/>
-      <c r="K86" s="34" t="n"/>
-      <c r="L86" s="34" t="n"/>
+      <c r="A86" s="33" t="inlineStr">
+        <is>
+          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Initial MAR count captured as N.</t>
+        </is>
+      </c>
+      <c r="B86" s="36" t="n"/>
+      <c r="C86" s="36" t="n"/>
+      <c r="D86" s="36" t="n"/>
+      <c r="E86" s="36" t="n"/>
+      <c r="F86" s="36" t="n"/>
+      <c r="G86" s="36" t="n"/>
+      <c r="H86" s="36" t="n"/>
+      <c r="I86" s="36" t="n"/>
+      <c r="J86" s="36" t="n"/>
+      <c r="K86" s="37" t="n"/>
+      <c r="L86" s="33" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="34" t="inlineStr">
         <is>
-          <t>TC-5.15 Step 2</t>
+          <t>TC-5.15 Step 1</t>
         </is>
       </c>
       <c r="B87" s="34" t="inlineStr">
@@ -18341,12 +18341,12 @@
       </c>
       <c r="D87" s="34" t="inlineStr">
         <is>
-          <t>Send POST /mar-records with route=null. All other fields valid.</t>
+          <t>Send POST /mar-records with route="intravenous" (invalid enum value). All other fields valid.</t>
         </is>
       </c>
       <c r="E87" s="34" t="inlineStr">
         <is>
-          <t>HTTP 400 Bad Request. Null route rejected.</t>
+          <t>HTTP 400 Bad Request. Invalid route value rejected.</t>
         </is>
       </c>
       <c r="F87" s="34" t="inlineStr">
@@ -18376,7 +18376,7 @@
     <row r="88">
       <c r="A88" s="34" t="inlineStr">
         <is>
-          <t>TC-5.15 Step 3</t>
+          <t>TC-5.15 Step 2</t>
         </is>
       </c>
       <c r="B88" s="34" t="inlineStr">
@@ -18391,17 +18391,17 @@
       </c>
       <c r="D88" s="34" t="inlineStr">
         <is>
-          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE tenant_id='tenant-aaa-001'. Assert count = N (unchanged).</t>
+          <t>Send POST /mar-records with route=null. All other fields valid.</t>
         </is>
       </c>
       <c r="E88" s="34" t="inlineStr">
         <is>
-          <t>Count = N. No rows created by either invalid attempt.</t>
+          <t>HTTP 400 Bad Request. Null route rejected.</t>
         </is>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>API</t>
         </is>
       </c>
       <c r="G88" s="34" t="inlineStr">
@@ -18424,27 +18424,59 @@
       <c r="L88" s="34" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="32" t="inlineStr">
-        <is>
-          <t>TC-5.16 - PATCH on MARRecord with status=administered Returns 422 for Any Field Change; DB Confirms All Fields Unchanged After Rejected Attempt | MARRecord</t>
-        </is>
-      </c>
-      <c r="B89" s="36" t="n"/>
-      <c r="C89" s="36" t="n"/>
-      <c r="D89" s="36" t="n"/>
-      <c r="E89" s="36" t="n"/>
-      <c r="F89" s="36" t="n"/>
-      <c r="G89" s="36" t="n"/>
-      <c r="H89" s="36" t="n"/>
-      <c r="I89" s="36" t="n"/>
-      <c r="J89" s="36" t="n"/>
-      <c r="K89" s="37" t="n"/>
-      <c r="L89" s="32" t="n"/>
+      <c r="A89" s="34" t="inlineStr">
+        <is>
+          <t>TC-5.15 Step 3</t>
+        </is>
+      </c>
+      <c r="B89" s="34" t="inlineStr">
+        <is>
+          <t>MARRecord</t>
+        </is>
+      </c>
+      <c r="C89" s="34" t="inlineStr">
+        <is>
+          <t>5.15</t>
+        </is>
+      </c>
+      <c r="D89" s="34" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE tenant_id='tenant-aaa-001'. Assert count = N (unchanged).</t>
+        </is>
+      </c>
+      <c r="E89" s="34" t="inlineStr">
+        <is>
+          <t>Count = N. No rows created by either invalid attempt.</t>
+        </is>
+      </c>
+      <c r="F89" s="34" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G89" s="34" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H89" s="34" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I89" s="34" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J89" s="34" t="n"/>
+      <c r="K89" s="34" t="n"/>
+      <c r="L89" s="34" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="33" t="inlineStr">
-        <is>
-          <t>Preconditions: A mar_record with status=administered, version=1, notes=null exists in tenant-aaa-001. nurse_medication_aide authenticated.</t>
+      <c r="A90" s="32" t="inlineStr">
+        <is>
+          <t>TC-5.16 - PATCH /mar-records/&lt;id&gt; notes on Missed MAR Returns 200; DB Confirms notes Updated and version Incremented | MARRecord</t>
         </is>
       </c>
       <c r="B90" s="36" t="n"/>
@@ -18457,62 +18489,30 @@
       <c r="I90" s="36" t="n"/>
       <c r="J90" s="36" t="n"/>
       <c r="K90" s="37" t="n"/>
-      <c r="L90" s="33" t="n"/>
+      <c r="L90" s="32" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="34" t="inlineStr">
-        <is>
-          <t>TC-5.16 Step 1</t>
-        </is>
-      </c>
-      <c r="B91" s="34" t="inlineStr">
-        <is>
-          <t>MARRecord</t>
-        </is>
-      </c>
-      <c r="C91" s="34" t="inlineStr">
-        <is>
-          <t>5.16</t>
-        </is>
-      </c>
-      <c r="D91" s="34" t="inlineStr">
-        <is>
-          <t>Query DB: SELECT status, version, notes FROM mar_record WHERE mar_id=&lt;mar_id&gt;. Confirm status='administered', version=1.</t>
-        </is>
-      </c>
-      <c r="E91" s="34" t="inlineStr">
-        <is>
-          <t>status='administered', version=1, notes=null confirmed.</t>
-        </is>
-      </c>
-      <c r="F91" s="34" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="G91" s="34" t="inlineStr">
-        <is>
-          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
-        </is>
-      </c>
-      <c r="H91" s="34" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I91" s="34" t="inlineStr">
-        <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="J91" s="34" t="n"/>
-      <c r="K91" s="34" t="n"/>
-      <c r="L91" s="34" t="n"/>
+      <c r="A91" s="33" t="inlineStr">
+        <is>
+          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Participant P1 exists. scheduled_time="fixture_scheduled_time".</t>
+        </is>
+      </c>
+      <c r="B91" s="36" t="n"/>
+      <c r="C91" s="36" t="n"/>
+      <c r="D91" s="36" t="n"/>
+      <c r="E91" s="36" t="n"/>
+      <c r="F91" s="36" t="n"/>
+      <c r="G91" s="36" t="n"/>
+      <c r="H91" s="36" t="n"/>
+      <c r="I91" s="36" t="n"/>
+      <c r="J91" s="36" t="n"/>
+      <c r="K91" s="37" t="n"/>
+      <c r="L91" s="33" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="34" t="inlineStr">
         <is>
-          <t>TC-5.16 Step 2</t>
+          <t>TC-5.16 Step 1</t>
         </is>
       </c>
       <c r="B92" s="34" t="inlineStr">
@@ -18527,12 +18527,12 @@
       </c>
       <c r="D92" s="34" t="inlineStr">
         <is>
-          <t>Send PATCH /mar-records/&lt;mar_id&gt; with {"notes": "post-admin update"} and nurse_medication_aide headers.</t>
+          <t>Send POST /mar-records with status=administered and administered_time=fixture_scheduled_time (equal to scheduled_time, within valid window). Body includes all required fields.</t>
         </is>
       </c>
       <c r="E92" s="34" t="inlineStr">
         <is>
-          <t>HTTP 422 Unprocessable Entity. Administered records are immutable.</t>
+          <t>HTTP 201 Created. Response contains mar_id.</t>
         </is>
       </c>
       <c r="F92" s="34" t="inlineStr">
@@ -18562,7 +18562,7 @@
     <row r="93">
       <c r="A93" s="34" t="inlineStr">
         <is>
-          <t>TC-5.16 Step 3</t>
+          <t>TC-5.16 Step 2</t>
         </is>
       </c>
       <c r="B93" s="34" t="inlineStr">
@@ -18577,12 +18577,12 @@
       </c>
       <c r="D93" s="34" t="inlineStr">
         <is>
-          <t>Assert response HTTP status code equals 422.</t>
+          <t>Assert response HTTP status code equals 201.</t>
         </is>
       </c>
       <c r="E93" s="34" t="inlineStr">
         <is>
-          <t>HTTP 422.</t>
+          <t>HTTP 201 Created.</t>
         </is>
       </c>
       <c r="F93" s="34" t="inlineStr">
@@ -18612,7 +18612,7 @@
     <row r="94">
       <c r="A94" s="34" t="inlineStr">
         <is>
-          <t>TC-5.16 Step 4</t>
+          <t>TC-5.16 Step 3</t>
         </is>
       </c>
       <c r="B94" s="34" t="inlineStr">
@@ -18627,12 +18627,12 @@
       </c>
       <c r="D94" s="34" t="inlineStr">
         <is>
-          <t>Query DB: SELECT status, version, notes FROM mar_record WHERE mar_id=&lt;mar_id&gt;. Assert all fields identical to pre-PATCH state.</t>
+          <t>Query DB: SELECT status, administered_time FROM mar_record WHERE mar_id=&lt;returned_mar_id&gt;.</t>
         </is>
       </c>
       <c r="E94" s="34" t="inlineStr">
         <is>
-          <t>status='administered', version=1, notes=null. All fields unchanged.</t>
+          <t>status='administered'. administered_time is non-null and matches fixture_scheduled_time.</t>
         </is>
       </c>
       <c r="F94" s="34" t="inlineStr">
@@ -18662,7 +18662,7 @@
     <row r="95">
       <c r="A95" s="32" t="inlineStr">
         <is>
-          <t>TC-5.17 - Correction POST with Valid 20-Char notes and original_mar_id Returns 201; DB Confirms Correction Row Created and All Fields of Original Row Unchanged via Direct DB Query | MARRecord</t>
+          <t>TC-5.17 - Correction POST Without original_mar_id Returns 422 MAR_CORRECTION_MISSING_ORIGINAL; DB Confirms No Correction Row Created | MARRecord</t>
         </is>
       </c>
       <c r="B95" s="36" t="n"/>
@@ -18680,7 +18680,7 @@
     <row r="96">
       <c r="A96" s="33" t="inlineStr">
         <is>
-          <t>Preconditions: A mar_record (original_id known, status=scheduled, version=1) exists in tenant-aaa-001. nurse_medication_aide authenticated.</t>
+          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Initial correction count in tenant = 0.</t>
         </is>
       </c>
       <c r="B96" s="36" t="n"/>
@@ -18713,17 +18713,17 @@
       </c>
       <c r="D97" s="34" t="inlineStr">
         <is>
-          <t>Query DB: SELECT mar_id, status, notes, version FROM mar_record WHERE mar_id=&lt;original_id&gt;. Capture all field values.</t>
+          <t>Send POST /mar-records with is_correction=true but no original_mar_id field. notes="Correction: missing original reference" (&gt;= 20 chars). All other required fields valid.</t>
         </is>
       </c>
       <c r="E97" s="34" t="inlineStr">
         <is>
-          <t>Original row confirmed: status='scheduled', version=1.</t>
+          <t>HTTP 422 Unprocessable Entity. original_mar_id is required for correction records.</t>
         </is>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>API</t>
         </is>
       </c>
       <c r="G97" s="34" t="inlineStr">
@@ -18733,7 +18733,7 @@
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I97" s="34" t="inlineStr">
@@ -18763,12 +18763,12 @@
       </c>
       <c r="D98" s="34" t="inlineStr">
         <is>
-          <t>Send POST /mar-records with is_correction=true, original_mar_id=&lt;original_id&gt;, notes="Correction: dose adjusted per updated prescription" (&gt;= 20 chars). All other required fields valid.</t>
+          <t>Assert response HTTP status code equals 422.</t>
         </is>
       </c>
       <c r="E98" s="34" t="inlineStr">
         <is>
-          <t>HTTP 201 Created. New mar_id returned (distinct from original_id).</t>
+          <t>HTTP 422.</t>
         </is>
       </c>
       <c r="F98" s="34" t="inlineStr">
@@ -18783,7 +18783,7 @@
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I98" s="34" t="inlineStr">
@@ -18813,12 +18813,12 @@
       </c>
       <c r="D99" s="34" t="inlineStr">
         <is>
-          <t>Query DB: SELECT is_correction, original_mar_id FROM mar_record WHERE mar_id=&lt;new_mar_id&gt;.</t>
+          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE is_correction=true AND tenant_id='tenant-aaa-001'. Assert count = 0.</t>
         </is>
       </c>
       <c r="E99" s="34" t="inlineStr">
         <is>
-          <t>is_correction=true. original_mar_id=&lt;original_id&gt;. Correction row correctly linked.</t>
+          <t>Count = 0. No correction row created.</t>
         </is>
       </c>
       <c r="F99" s="34" t="inlineStr">
@@ -18833,7 +18833,7 @@
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I99" s="34" t="inlineStr">
@@ -18846,59 +18846,27 @@
       <c r="L99" s="34" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="34" t="inlineStr">
-        <is>
-          <t>TC-5.17 Step 4</t>
-        </is>
-      </c>
-      <c r="B100" s="34" t="inlineStr">
-        <is>
-          <t>MARRecord</t>
-        </is>
-      </c>
-      <c r="C100" s="34" t="inlineStr">
-        <is>
-          <t>5.17</t>
-        </is>
-      </c>
-      <c r="D100" s="34" t="inlineStr">
-        <is>
-          <t>Query DB: SELECT status, notes, version FROM mar_record WHERE mar_id=&lt;original_id&gt;. Assert all values identical to those captured in Step 1.</t>
-        </is>
-      </c>
-      <c r="E100" s="34" t="inlineStr">
-        <is>
-          <t>All fields of original row unchanged. status, notes, version match captured values exactly.</t>
-        </is>
-      </c>
-      <c r="F100" s="34" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="G100" s="34" t="inlineStr">
-        <is>
-          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
-        </is>
-      </c>
-      <c r="H100" s="34" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I100" s="34" t="inlineStr">
-        <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="J100" s="34" t="n"/>
-      <c r="K100" s="34" t="n"/>
-      <c r="L100" s="34" t="n"/>
+      <c r="A100" s="32" t="inlineStr">
+        <is>
+          <t>TC-5.18 - Correction POST Without 20-Character notes Returns 422 MAR_CORRECTION_NOTES_TOO_SHORT; DB Confirms No Correction Row Created | MARRecord</t>
+        </is>
+      </c>
+      <c r="B100" s="36" t="n"/>
+      <c r="C100" s="36" t="n"/>
+      <c r="D100" s="36" t="n"/>
+      <c r="E100" s="36" t="n"/>
+      <c r="F100" s="36" t="n"/>
+      <c r="G100" s="36" t="n"/>
+      <c r="H100" s="36" t="n"/>
+      <c r="I100" s="36" t="n"/>
+      <c r="J100" s="36" t="n"/>
+      <c r="K100" s="37" t="n"/>
+      <c r="L100" s="32" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="32" t="inlineStr">
-        <is>
-          <t>TC-5.18 - Correction POST Without 20-Character notes Returns 422; DB Confirms No Correction Row Created | MARRecord</t>
+      <c r="A101" s="33" t="inlineStr">
+        <is>
+          <t>Preconditions: A mar_record exists in tenant-aaa-001 (original_id known). nurse_medication_aide authenticated. Initial correction count for original_id = 0.</t>
         </is>
       </c>
       <c r="B101" s="36" t="n"/>
@@ -18911,30 +18879,62 @@
       <c r="I101" s="36" t="n"/>
       <c r="J101" s="36" t="n"/>
       <c r="K101" s="37" t="n"/>
-      <c r="L101" s="32" t="n"/>
+      <c r="L101" s="33" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="33" t="inlineStr">
-        <is>
-          <t>Preconditions: A mar_record exists in tenant-aaa-001 (original_id known). nurse_medication_aide authenticated. Initial correction count for original_id = 0.</t>
-        </is>
-      </c>
-      <c r="B102" s="36" t="n"/>
-      <c r="C102" s="36" t="n"/>
-      <c r="D102" s="36" t="n"/>
-      <c r="E102" s="36" t="n"/>
-      <c r="F102" s="36" t="n"/>
-      <c r="G102" s="36" t="n"/>
-      <c r="H102" s="36" t="n"/>
-      <c r="I102" s="36" t="n"/>
-      <c r="J102" s="36" t="n"/>
-      <c r="K102" s="37" t="n"/>
-      <c r="L102" s="33" t="n"/>
+      <c r="A102" s="34" t="inlineStr">
+        <is>
+          <t>TC-5.18 Step 1</t>
+        </is>
+      </c>
+      <c r="B102" s="34" t="inlineStr">
+        <is>
+          <t>MARRecord</t>
+        </is>
+      </c>
+      <c r="C102" s="34" t="inlineStr">
+        <is>
+          <t>5.18</t>
+        </is>
+      </c>
+      <c r="D102" s="34" t="inlineStr">
+        <is>
+          <t>Send POST /mar-records with is_correction=true, original_mar_id=&lt;original_id&gt;, notes="Short" (fewer than 20 characters).</t>
+        </is>
+      </c>
+      <c r="E102" s="34" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity. notes too short for a correction record.</t>
+        </is>
+      </c>
+      <c r="F102" s="34" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G102" s="34" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H102" s="34" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I102" s="34" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J102" s="34" t="n"/>
+      <c r="K102" s="34" t="n"/>
+      <c r="L102" s="34" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="34" t="inlineStr">
         <is>
-          <t>TC-5.18 Step 1</t>
+          <t>TC-5.18 Step 2</t>
         </is>
       </c>
       <c r="B103" s="34" t="inlineStr">
@@ -18949,12 +18949,12 @@
       </c>
       <c r="D103" s="34" t="inlineStr">
         <is>
-          <t>Send POST /mar-records with is_correction=true, original_mar_id=&lt;original_id&gt;, notes="Short" (fewer than 20 characters).</t>
+          <t>Assert response HTTP status code equals 422.</t>
         </is>
       </c>
       <c r="E103" s="34" t="inlineStr">
         <is>
-          <t>HTTP 422 Unprocessable Entity. notes too short for a correction record.</t>
+          <t>HTTP 422.</t>
         </is>
       </c>
       <c r="F103" s="34" t="inlineStr">
@@ -18984,7 +18984,7 @@
     <row r="104">
       <c r="A104" s="34" t="inlineStr">
         <is>
-          <t>TC-5.18 Step 2</t>
+          <t>TC-5.18 Step 3</t>
         </is>
       </c>
       <c r="B104" s="34" t="inlineStr">
@@ -18999,17 +18999,17 @@
       </c>
       <c r="D104" s="34" t="inlineStr">
         <is>
-          <t>Assert response HTTP status code equals 422.</t>
+          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE is_correction=true AND original_mar_id=&lt;original_id&gt;. Assert count = 0.</t>
         </is>
       </c>
       <c r="E104" s="34" t="inlineStr">
         <is>
-          <t>HTTP 422.</t>
+          <t>Count = 0. No correction row created.</t>
         </is>
       </c>
       <c r="F104" s="34" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="G104" s="34" t="inlineStr">
@@ -19032,59 +19032,27 @@
       <c r="L104" s="34" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="34" t="inlineStr">
-        <is>
-          <t>TC-5.18 Step 3</t>
-        </is>
-      </c>
-      <c r="B105" s="34" t="inlineStr">
-        <is>
-          <t>MARRecord</t>
-        </is>
-      </c>
-      <c r="C105" s="34" t="inlineStr">
-        <is>
-          <t>5.18</t>
-        </is>
-      </c>
-      <c r="D105" s="34" t="inlineStr">
-        <is>
-          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE is_correction=true AND original_mar_id=&lt;original_id&gt;. Assert count = 0.</t>
-        </is>
-      </c>
-      <c r="E105" s="34" t="inlineStr">
-        <is>
-          <t>Count = 0. No correction row created.</t>
-        </is>
-      </c>
-      <c r="F105" s="34" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="G105" s="34" t="inlineStr">
-        <is>
-          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
-        </is>
-      </c>
-      <c r="H105" s="34" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I105" s="34" t="inlineStr">
-        <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="J105" s="34" t="n"/>
-      <c r="K105" s="34" t="n"/>
-      <c r="L105" s="34" t="n"/>
+      <c r="A105" s="32" t="inlineStr">
+        <is>
+          <t>TC-5.19 - Correction POST with Valid original_mar_id and 20-Char notes Returns 201; DB Confirms is_correction=True and original_mar_id Set | MARRecord</t>
+        </is>
+      </c>
+      <c r="B105" s="36" t="n"/>
+      <c r="C105" s="36" t="n"/>
+      <c r="D105" s="36" t="n"/>
+      <c r="E105" s="36" t="n"/>
+      <c r="F105" s="36" t="n"/>
+      <c r="G105" s="36" t="n"/>
+      <c r="H105" s="36" t="n"/>
+      <c r="I105" s="36" t="n"/>
+      <c r="J105" s="36" t="n"/>
+      <c r="K105" s="37" t="n"/>
+      <c r="L105" s="32" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="32" t="inlineStr">
-        <is>
-          <t>TC-5.19 - Correction POST Without original_mar_id Returns 422; DB Confirms No Correction Row Created | MARRecord</t>
+      <c r="A106" s="33" t="inlineStr">
+        <is>
+          <t>Preconditions: A mar_record (original_id known, status=scheduled, version=1) exists in tenant-aaa-001. nurse_medication_aide authenticated.</t>
         </is>
       </c>
       <c r="B106" s="36" t="n"/>
@@ -19097,30 +19065,62 @@
       <c r="I106" s="36" t="n"/>
       <c r="J106" s="36" t="n"/>
       <c r="K106" s="37" t="n"/>
-      <c r="L106" s="32" t="n"/>
+      <c r="L106" s="33" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="33" t="inlineStr">
-        <is>
-          <t>Preconditions: nurse_medication_aide authenticated in tenant-aaa-001. Initial correction count in tenant = 0.</t>
-        </is>
-      </c>
-      <c r="B107" s="36" t="n"/>
-      <c r="C107" s="36" t="n"/>
-      <c r="D107" s="36" t="n"/>
-      <c r="E107" s="36" t="n"/>
-      <c r="F107" s="36" t="n"/>
-      <c r="G107" s="36" t="n"/>
-      <c r="H107" s="36" t="n"/>
-      <c r="I107" s="36" t="n"/>
-      <c r="J107" s="36" t="n"/>
-      <c r="K107" s="37" t="n"/>
-      <c r="L107" s="33" t="n"/>
+      <c r="A107" s="34" t="inlineStr">
+        <is>
+          <t>TC-5.19 Step 1</t>
+        </is>
+      </c>
+      <c r="B107" s="34" t="inlineStr">
+        <is>
+          <t>MARRecord</t>
+        </is>
+      </c>
+      <c r="C107" s="34" t="inlineStr">
+        <is>
+          <t>5.19</t>
+        </is>
+      </c>
+      <c r="D107" s="34" t="inlineStr">
+        <is>
+          <t>Query DB: SELECT mar_id, status, notes, version FROM mar_record WHERE mar_id=&lt;original_id&gt;. Capture all field values.</t>
+        </is>
+      </c>
+      <c r="E107" s="34" t="inlineStr">
+        <is>
+          <t>Original row confirmed: status='scheduled', version=1.</t>
+        </is>
+      </c>
+      <c r="F107" s="34" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G107" s="34" t="inlineStr">
+        <is>
+          <t>CMS Medicaid/Medicare; State Adult Day Care Licensing</t>
+        </is>
+      </c>
+      <c r="H107" s="34" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I107" s="34" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J107" s="34" t="n"/>
+      <c r="K107" s="34" t="n"/>
+      <c r="L107" s="34" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="34" t="inlineStr">
         <is>
-          <t>TC-5.19 Step 1</t>
+          <t>TC-5.19 Step 2</t>
         </is>
       </c>
       <c r="B108" s="34" t="inlineStr">
@@ -19135,12 +19135,12 @@
       </c>
       <c r="D108" s="34" t="inlineStr">
         <is>
-          <t>Send POST /mar-records with is_correction=true but no original_mar_id field. notes="Correction: missing original reference" (&gt;= 20 chars). All other required fields valid.</t>
+          <t>Send POST /mar-records with is_correction=true, original_mar_id=&lt;original_id&gt;, notes="Correction: dose adjusted per updated prescription" (&gt;= 20 chars). All other required fields valid.</t>
         </is>
       </c>
       <c r="E108" s="34" t="inlineStr">
         <is>
-          <t>HTTP 422 Unprocessable Entity. original_mar_id is required for correction records.</t>
+          <t>HTTP 201 Created. New mar_id returned (distinct from original_id).</t>
         </is>
       </c>
       <c r="F108" s="34" t="inlineStr">
@@ -19155,7 +19155,7 @@
       </c>
       <c r="H108" s="34" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I108" s="34" t="inlineStr">
@@ -19170,7 +19170,7 @@
     <row r="109">
       <c r="A109" s="34" t="inlineStr">
         <is>
-          <t>TC-5.19 Step 2</t>
+          <t>TC-5.19 Step 3</t>
         </is>
       </c>
       <c r="B109" s="34" t="inlineStr">
@@ -19185,17 +19185,17 @@
       </c>
       <c r="D109" s="34" t="inlineStr">
         <is>
-          <t>Assert response HTTP status code equals 422.</t>
+          <t>Query DB: SELECT is_correction, original_mar_id FROM mar_record WHERE mar_id=&lt;new_mar_id&gt;.</t>
         </is>
       </c>
       <c r="E109" s="34" t="inlineStr">
         <is>
-          <t>HTTP 422.</t>
+          <t>is_correction=true. original_mar_id=&lt;original_id&gt;. Correction row correctly linked.</t>
         </is>
       </c>
       <c r="F109" s="34" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="G109" s="34" t="inlineStr">
@@ -19205,7 +19205,7 @@
       </c>
       <c r="H109" s="34" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I109" s="34" t="inlineStr">
@@ -19220,7 +19220,7 @@
     <row r="110">
       <c r="A110" s="34" t="inlineStr">
         <is>
-          <t>TC-5.19 Step 3</t>
+          <t>TC-5.19 Step 4</t>
         </is>
       </c>
       <c r="B110" s="34" t="inlineStr">
@@ -19235,12 +19235,12 @@
       </c>
       <c r="D110" s="34" t="inlineStr">
         <is>
-          <t>Query DB: SELECT COUNT(*) FROM mar_record WHERE is_correction=true AND tenant_id='tenant-aaa-001'. Assert count = 0.</t>
+          <t>Query DB: SELECT status, notes, version FROM mar_record WHERE mar_id=&lt;original_id&gt;. Assert all values identical to those captured in Step 1.</t>
         </is>
       </c>
       <c r="E110" s="34" t="inlineStr">
         <is>
-          <t>Count = 0. No correction row created.</t>
+          <t>All fields of original row unchanged. status, notes, version match captured values exactly.</t>
         </is>
       </c>
       <c r="F110" s="34" t="inlineStr">
@@ -19255,7 +19255,7 @@
       </c>
       <c r="H110" s="34" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I110" s="34" t="inlineStr">
@@ -19270,7 +19270,7 @@
     <row r="111">
       <c r="A111" s="32" t="inlineStr">
         <is>
-          <t>TC-5.20 - PATCH Non-Administered MARRecord with Correct version Returns 200; DB Confirms version Incremented | MARRecord</t>
+          <t>TC-5.20 - PATCH /mar-records/&lt;id&gt; status Transition on Missed MAR Returns 200; DB Confirms status Changed and version Incremented | MARRecord</t>
         </is>
       </c>
       <c r="B111" s="36" t="n"/>
@@ -19506,7 +19506,7 @@
     <row r="117">
       <c r="A117" s="32" t="inlineStr">
         <is>
-          <t>TC-5.21 - PATCH with Stale version Returns 409 MAR_VERSION_CONFLICT; DB version Unchanged; PATCH Administered MARRecord Returns 422 Before Version Check; DB version Unchanged | MARRecord</t>
+          <t>TC-5.21 - PATCH with Stale version Returns 409 MAR_VERSION_CONFLICT; DB version Unchanged | MARRecord</t>
         </is>
       </c>
       <c r="B117" s="36" t="n"/>
@@ -19791,46 +19791,46 @@
     </row>
   </sheetData>
   <mergeCells count="42">
+    <mergeCell ref="A34:K34"/>
     <mergeCell ref="A30:K30"/>
     <mergeCell ref="A15:K15"/>
     <mergeCell ref="A73:K73"/>
     <mergeCell ref="A51:K51"/>
-    <mergeCell ref="A107:K107"/>
-    <mergeCell ref="A36:K36"/>
+    <mergeCell ref="A45:K45"/>
     <mergeCell ref="A79:K79"/>
-    <mergeCell ref="A61:K61"/>
-    <mergeCell ref="A78:K78"/>
     <mergeCell ref="A111:K111"/>
     <mergeCell ref="A41:K41"/>
     <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A90:K90"/>
     <mergeCell ref="A46:K46"/>
-    <mergeCell ref="A84:K84"/>
-    <mergeCell ref="A90:K90"/>
-    <mergeCell ref="A66:K66"/>
+    <mergeCell ref="A80:K80"/>
     <mergeCell ref="A118:K118"/>
     <mergeCell ref="A56:K56"/>
-    <mergeCell ref="A89:K89"/>
+    <mergeCell ref="A74:K74"/>
+    <mergeCell ref="A105:K105"/>
+    <mergeCell ref="A50:K50"/>
+    <mergeCell ref="A101:K101"/>
+    <mergeCell ref="A21:K21"/>
     <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A21:K21"/>
-    <mergeCell ref="A101:K101"/>
+    <mergeCell ref="A86:K86"/>
+    <mergeCell ref="A95:K95"/>
     <mergeCell ref="A57:K57"/>
-    <mergeCell ref="A95:K95"/>
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A47:K47"/>
-    <mergeCell ref="A42:K42"/>
     <mergeCell ref="A85:K85"/>
     <mergeCell ref="A106:K106"/>
     <mergeCell ref="A22:K22"/>
+    <mergeCell ref="A91:K91"/>
     <mergeCell ref="A35:K35"/>
     <mergeCell ref="A62:K62"/>
+    <mergeCell ref="A100:K100"/>
     <mergeCell ref="A96:K96"/>
-    <mergeCell ref="A72:K72"/>
     <mergeCell ref="A29:K29"/>
     <mergeCell ref="A112:K112"/>
-    <mergeCell ref="A52:K52"/>
+    <mergeCell ref="A63:K63"/>
     <mergeCell ref="A10:K10"/>
     <mergeCell ref="A117:K117"/>
-    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="A68:K68"/>
+    <mergeCell ref="A40:K40"/>
     <mergeCell ref="A9:K9"/>
     <mergeCell ref="A67:K67"/>
   </mergeCells>
@@ -22101,12 +22101,12 @@
       </c>
       <c r="D58" s="34" t="inlineStr">
         <is>
-          <t>Query DB: SELECT COUNT(*) FROM audit_log WHERE resource_id=&lt;id&gt; AND event_type='ESCALATION_ALERT'. Assert count &gt;= 1.</t>
+          <t>Query DB: SELECT event_id, event_type, timestamp, user_id, tenant_id, resource_type, resource_id, action, data_affected, session_id, outcome FROM audit_log WHERE resource_id=incident_id AND event_type='ESCALATION_ALERT'. Assert all 11 mandatory fields are non-null on the returned row. Assert data_affected contains no raw PHI values.</t>
         </is>
       </c>
       <c r="E58" s="34" t="inlineStr">
         <is>
-          <t>ESCALATION_ALERT audit event row created by job.</t>
+          <t>All 11 mandatory audit fields non-null. data_affected contains no raw PHI. ESCALATION_ALERT event correctly structured per HIPAA audit requirements.</t>
         </is>
       </c>
       <c r="F58" s="34" t="inlineStr">

</xml_diff>

<commit_message>
phase 1 complete: groups 7-9 written and passing, DBSchema TC added, docs updated, CI gate expanded to 44 tests
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_cases/test_cases_phase1.xlsx
+++ b/test_cases/test_cases_phase1.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AuditLog" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RBACSweep" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TenantIsolation" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DBSchema" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -76,7 +77,7 @@
       <patternFill patternType="solid"/>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -291,11 +292,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -396,6 +406,18 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4154,6 +4176,802 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16.8" customWidth="1" min="1" max="1"/>
+    <col width="20.4" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="9.6" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="15.6" customWidth="1" min="10" max="10"/>
+    <col width="10.8" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="45" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B1" s="45" t="inlineStr">
+        <is>
+          <t>Requirement Group</t>
+        </is>
+      </c>
+      <c r="C1" s="45" t="inlineStr">
+        <is>
+          <t>REQ_ID</t>
+        </is>
+      </c>
+      <c r="D1" s="45" t="inlineStr">
+        <is>
+          <t>Step Description</t>
+        </is>
+      </c>
+      <c r="E1" s="45" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="F1" s="45" t="inlineStr">
+        <is>
+          <t>Layer</t>
+        </is>
+      </c>
+      <c r="G1" s="45" t="inlineStr">
+        <is>
+          <t>Regulatory Reference</t>
+        </is>
+      </c>
+      <c r="H1" s="45" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="I1" s="45" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="45" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="K1" s="45" t="inlineStr">
+        <is>
+          <t>Pass/Fail</t>
+        </is>
+      </c>
+      <c r="L1" s="45" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="46" t="inlineStr">
+        <is>
+          <t>TC-10.1 - UNIQUE Index on (tenant_id, medicaid_id) Present on Participant Table</t>
+        </is>
+      </c>
+      <c r="B2" s="36" t="n"/>
+      <c r="C2" s="36" t="n"/>
+      <c r="D2" s="36" t="n"/>
+      <c r="E2" s="36" t="n"/>
+      <c r="F2" s="36" t="n"/>
+      <c r="G2" s="36" t="n"/>
+      <c r="H2" s="36" t="n"/>
+      <c r="I2" s="36" t="n"/>
+      <c r="J2" s="36" t="n"/>
+      <c r="K2" s="37" t="n"/>
+      <c r="L2" s="46" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="47" t="inlineStr">
+        <is>
+          <t>Preconditions: SQLite in-memory DB created from Base.metadata. schema_conn fixture available.</t>
+        </is>
+      </c>
+      <c r="B3" s="36" t="n"/>
+      <c r="C3" s="36" t="n"/>
+      <c r="D3" s="36" t="n"/>
+      <c r="E3" s="36" t="n"/>
+      <c r="F3" s="36" t="n"/>
+      <c r="G3" s="36" t="n"/>
+      <c r="H3" s="36" t="n"/>
+      <c r="I3" s="36" t="n"/>
+      <c r="J3" s="36" t="n"/>
+      <c r="K3" s="37" t="n"/>
+      <c r="L3" s="47" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="48" t="inlineStr">
+        <is>
+          <t>TC-10.1 Step 1</t>
+        </is>
+      </c>
+      <c r="B4" s="48" t="inlineStr">
+        <is>
+          <t>DBSchema</t>
+        </is>
+      </c>
+      <c r="C4" s="48" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="D4" s="48" t="inlineStr">
+        <is>
+          <t>Run PRAGMA index_list on participant table. Assert UNIQUE index exists on columns (tenant_id, medicaid_id).</t>
+        </is>
+      </c>
+      <c r="E4" s="48" t="inlineStr">
+        <is>
+          <t>UNIQUE index on (tenant_id, medicaid_id) confirmed present.</t>
+        </is>
+      </c>
+      <c r="F4" s="48" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G4" s="48" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(c); CMS data integrity</t>
+        </is>
+      </c>
+      <c r="H4" s="48" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I4" s="48" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J4" s="48" t="n"/>
+      <c r="K4" s="48" t="n"/>
+      <c r="L4" s="48" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="46" t="inlineStr">
+        <is>
+          <t>TC-10.2 - UNIQUE Index on (tenant_id, email) and PRIMARY KEY on user_id Present on User Table</t>
+        </is>
+      </c>
+      <c r="B5" s="36" t="n"/>
+      <c r="C5" s="36" t="n"/>
+      <c r="D5" s="36" t="n"/>
+      <c r="E5" s="36" t="n"/>
+      <c r="F5" s="36" t="n"/>
+      <c r="G5" s="36" t="n"/>
+      <c r="H5" s="36" t="n"/>
+      <c r="I5" s="36" t="n"/>
+      <c r="J5" s="36" t="n"/>
+      <c r="K5" s="37" t="n"/>
+      <c r="L5" s="46" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="47" t="inlineStr">
+        <is>
+          <t>Preconditions: SQLite in-memory DB created from Base.metadata. schema_conn fixture available.</t>
+        </is>
+      </c>
+      <c r="B6" s="36" t="n"/>
+      <c r="C6" s="36" t="n"/>
+      <c r="D6" s="36" t="n"/>
+      <c r="E6" s="36" t="n"/>
+      <c r="F6" s="36" t="n"/>
+      <c r="G6" s="36" t="n"/>
+      <c r="H6" s="36" t="n"/>
+      <c r="I6" s="36" t="n"/>
+      <c r="J6" s="36" t="n"/>
+      <c r="K6" s="37" t="n"/>
+      <c r="L6" s="47" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="48" t="inlineStr">
+        <is>
+          <t>TC-10.2 Step 1</t>
+        </is>
+      </c>
+      <c r="B7" s="48" t="inlineStr">
+        <is>
+          <t>DBSchema</t>
+        </is>
+      </c>
+      <c r="C7" s="48" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="D7" s="48" t="inlineStr">
+        <is>
+          <t>Run PRAGMA index_list on user table. Assert UNIQUE index on (tenant_id, email). Assert user_id column exists.</t>
+        </is>
+      </c>
+      <c r="E7" s="48" t="inlineStr">
+        <is>
+          <t>UNIQUE index on (tenant_id, email) and user_id column confirmed present.</t>
+        </is>
+      </c>
+      <c r="F7" s="48" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G7" s="48" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(c); CMS data integrity</t>
+        </is>
+      </c>
+      <c r="H7" s="48" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I7" s="48" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J7" s="48" t="n"/>
+      <c r="K7" s="48" t="n"/>
+      <c r="L7" s="48" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="46" t="inlineStr">
+        <is>
+          <t>TC-10.3 - UNIQUE Index on (tenant_id, participant_id, date_of_service) Present on Attendance Table</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="n"/>
+      <c r="C8" s="36" t="n"/>
+      <c r="D8" s="36" t="n"/>
+      <c r="E8" s="36" t="n"/>
+      <c r="F8" s="36" t="n"/>
+      <c r="G8" s="36" t="n"/>
+      <c r="H8" s="36" t="n"/>
+      <c r="I8" s="36" t="n"/>
+      <c r="J8" s="36" t="n"/>
+      <c r="K8" s="37" t="n"/>
+      <c r="L8" s="46" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="47" t="inlineStr">
+        <is>
+          <t>Preconditions: SQLite in-memory DB created from Base.metadata. schema_conn fixture available.</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="n"/>
+      <c r="C9" s="36" t="n"/>
+      <c r="D9" s="36" t="n"/>
+      <c r="E9" s="36" t="n"/>
+      <c r="F9" s="36" t="n"/>
+      <c r="G9" s="36" t="n"/>
+      <c r="H9" s="36" t="n"/>
+      <c r="I9" s="36" t="n"/>
+      <c r="J9" s="36" t="n"/>
+      <c r="K9" s="37" t="n"/>
+      <c r="L9" s="47" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="48" t="inlineStr">
+        <is>
+          <t>TC-10.3 Step 1</t>
+        </is>
+      </c>
+      <c r="B10" s="48" t="inlineStr">
+        <is>
+          <t>DBSchema</t>
+        </is>
+      </c>
+      <c r="C10" s="48" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="D10" s="48" t="inlineStr">
+        <is>
+          <t>Run PRAGMA index_list on attendance table. Assert UNIQUE index on (tenant_id, participant_id, date_of_service).</t>
+        </is>
+      </c>
+      <c r="E10" s="48" t="inlineStr">
+        <is>
+          <t>UNIQUE index on (tenant_id, participant_id, date_of_service) confirmed present.</t>
+        </is>
+      </c>
+      <c r="F10" s="48" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G10" s="48" t="inlineStr">
+        <is>
+          <t>CMS billing integrity; HIPAA §164.312(c)</t>
+        </is>
+      </c>
+      <c r="H10" s="48" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I10" s="48" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J10" s="48" t="n"/>
+      <c r="K10" s="48" t="n"/>
+      <c r="L10" s="48" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="46" t="inlineStr">
+        <is>
+          <t>TC-10.4 - UNIQUE Index on claim_reference_number and Composite Billing Key Present on Claim Table</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="n"/>
+      <c r="C11" s="36" t="n"/>
+      <c r="D11" s="36" t="n"/>
+      <c r="E11" s="36" t="n"/>
+      <c r="F11" s="36" t="n"/>
+      <c r="G11" s="36" t="n"/>
+      <c r="H11" s="36" t="n"/>
+      <c r="I11" s="36" t="n"/>
+      <c r="J11" s="36" t="n"/>
+      <c r="K11" s="37" t="n"/>
+      <c r="L11" s="46" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="47" t="inlineStr">
+        <is>
+          <t>Preconditions: SQLite in-memory DB created from Base.metadata. schema_conn fixture available.</t>
+        </is>
+      </c>
+      <c r="B12" s="36" t="n"/>
+      <c r="C12" s="36" t="n"/>
+      <c r="D12" s="36" t="n"/>
+      <c r="E12" s="36" t="n"/>
+      <c r="F12" s="36" t="n"/>
+      <c r="G12" s="36" t="n"/>
+      <c r="H12" s="36" t="n"/>
+      <c r="I12" s="36" t="n"/>
+      <c r="J12" s="36" t="n"/>
+      <c r="K12" s="37" t="n"/>
+      <c r="L12" s="47" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="48" t="inlineStr">
+        <is>
+          <t>TC-10.4 Step 1</t>
+        </is>
+      </c>
+      <c r="B13" s="48" t="inlineStr">
+        <is>
+          <t>DBSchema</t>
+        </is>
+      </c>
+      <c r="C13" s="48" t="inlineStr">
+        <is>
+          <t>10.4</t>
+        </is>
+      </c>
+      <c r="D13" s="48" t="inlineStr">
+        <is>
+          <t>Run PRAGMA index_list on claim table. Assert UNIQUE index on claim_reference_number. Assert composite UNIQUE index on (tenant_id, participant_id, date_of_service_start, procedure_code, payer_type).</t>
+        </is>
+      </c>
+      <c r="E13" s="48" t="inlineStr">
+        <is>
+          <t>Both UNIQUE indexes confirmed present.</t>
+        </is>
+      </c>
+      <c r="F13" s="48" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G13" s="48" t="inlineStr">
+        <is>
+          <t>CMS billing integrity; HIPAA §164.312(c)</t>
+        </is>
+      </c>
+      <c r="H13" s="48" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I13" s="48" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J13" s="48" t="n"/>
+      <c r="K13" s="48" t="n"/>
+      <c r="L13" s="48" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="46" t="inlineStr">
+        <is>
+          <t>TC-10.5 - UNIQUE Index on (tenant_id, participant_id, medication_name, scheduled_time) Present on MAR Record Table</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="n"/>
+      <c r="C14" s="36" t="n"/>
+      <c r="D14" s="36" t="n"/>
+      <c r="E14" s="36" t="n"/>
+      <c r="F14" s="36" t="n"/>
+      <c r="G14" s="36" t="n"/>
+      <c r="H14" s="36" t="n"/>
+      <c r="I14" s="36" t="n"/>
+      <c r="J14" s="36" t="n"/>
+      <c r="K14" s="37" t="n"/>
+      <c r="L14" s="46" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="47" t="inlineStr">
+        <is>
+          <t>Preconditions: SQLite in-memory DB created from Base.metadata. schema_conn fixture available.</t>
+        </is>
+      </c>
+      <c r="B15" s="36" t="n"/>
+      <c r="C15" s="36" t="n"/>
+      <c r="D15" s="36" t="n"/>
+      <c r="E15" s="36" t="n"/>
+      <c r="F15" s="36" t="n"/>
+      <c r="G15" s="36" t="n"/>
+      <c r="H15" s="36" t="n"/>
+      <c r="I15" s="36" t="n"/>
+      <c r="J15" s="36" t="n"/>
+      <c r="K15" s="37" t="n"/>
+      <c r="L15" s="47" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="48" t="inlineStr">
+        <is>
+          <t>TC-10.5 Step 1</t>
+        </is>
+      </c>
+      <c r="B16" s="48" t="inlineStr">
+        <is>
+          <t>DBSchema</t>
+        </is>
+      </c>
+      <c r="C16" s="48" t="inlineStr">
+        <is>
+          <t>10.5</t>
+        </is>
+      </c>
+      <c r="D16" s="48" t="inlineStr">
+        <is>
+          <t>Run PRAGMA index_list on mar_record table. Assert UNIQUE index on (tenant_id, participant_id, medication_name, scheduled_time).</t>
+        </is>
+      </c>
+      <c r="E16" s="48" t="inlineStr">
+        <is>
+          <t>UNIQUE index on (tenant_id, participant_id, medication_name, scheduled_time) confirmed present.</t>
+        </is>
+      </c>
+      <c r="F16" s="48" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G16" s="48" t="inlineStr">
+        <is>
+          <t>42 CFR Part 2; HIPAA §164.312(c)</t>
+        </is>
+      </c>
+      <c r="H16" s="48" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I16" s="48" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J16" s="48" t="n"/>
+      <c r="K16" s="48" t="n"/>
+      <c r="L16" s="48" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="46" t="inlineStr">
+        <is>
+          <t>TC-10.6 - NOT NULL Constraints Confirmed on All Mandatory Fields for All Six Entities</t>
+        </is>
+      </c>
+      <c r="B17" s="36" t="n"/>
+      <c r="C17" s="36" t="n"/>
+      <c r="D17" s="36" t="n"/>
+      <c r="E17" s="36" t="n"/>
+      <c r="F17" s="36" t="n"/>
+      <c r="G17" s="36" t="n"/>
+      <c r="H17" s="36" t="n"/>
+      <c r="I17" s="36" t="n"/>
+      <c r="J17" s="36" t="n"/>
+      <c r="K17" s="37" t="n"/>
+      <c r="L17" s="46" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="47" t="inlineStr">
+        <is>
+          <t>Preconditions: SQLite in-memory DB created from Base.metadata. schema_conn fixture available.</t>
+        </is>
+      </c>
+      <c r="B18" s="36" t="n"/>
+      <c r="C18" s="36" t="n"/>
+      <c r="D18" s="36" t="n"/>
+      <c r="E18" s="36" t="n"/>
+      <c r="F18" s="36" t="n"/>
+      <c r="G18" s="36" t="n"/>
+      <c r="H18" s="36" t="n"/>
+      <c r="I18" s="36" t="n"/>
+      <c r="J18" s="36" t="n"/>
+      <c r="K18" s="37" t="n"/>
+      <c r="L18" s="47" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="48" t="inlineStr">
+        <is>
+          <t>TC-10.6 Step 1</t>
+        </is>
+      </c>
+      <c r="B19" s="48" t="inlineStr">
+        <is>
+          <t>DBSchema</t>
+        </is>
+      </c>
+      <c r="C19" s="48" t="inlineStr">
+        <is>
+          <t>10.6</t>
+        </is>
+      </c>
+      <c r="D19" s="48" t="inlineStr">
+        <is>
+          <t>Run PRAGMA table_info on all six entity tables. Assert NOT NULL on all mandatory fields per entity.</t>
+        </is>
+      </c>
+      <c r="E19" s="48" t="inlineStr">
+        <is>
+          <t>NOT NULL confirmed on all mandatory fields for all six entities.</t>
+        </is>
+      </c>
+      <c r="F19" s="48" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G19" s="48" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(c); CMS data integrity</t>
+        </is>
+      </c>
+      <c r="H19" s="48" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I19" s="48" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J19" s="48" t="n"/>
+      <c r="K19" s="48" t="n"/>
+      <c r="L19" s="48" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="46" t="inlineStr">
+        <is>
+          <t>TC-10.7 - version Column of INTEGER Type Present on All Six Entity Tables</t>
+        </is>
+      </c>
+      <c r="B20" s="36" t="n"/>
+      <c r="C20" s="36" t="n"/>
+      <c r="D20" s="36" t="n"/>
+      <c r="E20" s="36" t="n"/>
+      <c r="F20" s="36" t="n"/>
+      <c r="G20" s="36" t="n"/>
+      <c r="H20" s="36" t="n"/>
+      <c r="I20" s="36" t="n"/>
+      <c r="J20" s="36" t="n"/>
+      <c r="K20" s="37" t="n"/>
+      <c r="L20" s="46" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="47" t="inlineStr">
+        <is>
+          <t>Preconditions: SQLite in-memory DB created from Base.metadata. schema_conn fixture available.</t>
+        </is>
+      </c>
+      <c r="B21" s="36" t="n"/>
+      <c r="C21" s="36" t="n"/>
+      <c r="D21" s="36" t="n"/>
+      <c r="E21" s="36" t="n"/>
+      <c r="F21" s="36" t="n"/>
+      <c r="G21" s="36" t="n"/>
+      <c r="H21" s="36" t="n"/>
+      <c r="I21" s="36" t="n"/>
+      <c r="J21" s="36" t="n"/>
+      <c r="K21" s="37" t="n"/>
+      <c r="L21" s="47" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="48" t="inlineStr">
+        <is>
+          <t>TC-10.7 Step 1</t>
+        </is>
+      </c>
+      <c r="B22" s="48" t="inlineStr">
+        <is>
+          <t>DBSchema</t>
+        </is>
+      </c>
+      <c r="C22" s="48" t="inlineStr">
+        <is>
+          <t>10.7</t>
+        </is>
+      </c>
+      <c r="D22" s="48" t="inlineStr">
+        <is>
+          <t>Run PRAGMA table_info on all six entity tables. Assert version column exists with INTEGER type.</t>
+        </is>
+      </c>
+      <c r="E22" s="48" t="inlineStr">
+        <is>
+          <t>version column of INTEGER type confirmed on all six entity tables.</t>
+        </is>
+      </c>
+      <c r="F22" s="48" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G22" s="48" t="inlineStr">
+        <is>
+          <t>HIPAA §164.312(b); data integrity</t>
+        </is>
+      </c>
+      <c r="H22" s="48" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I22" s="48" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J22" s="48" t="n"/>
+      <c r="K22" s="48" t="n"/>
+      <c r="L22" s="48" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="46" t="inlineStr">
+        <is>
+          <t>TC-10.8 - is_deleted Defaults False on Participant and User Tables; No Row Has NULL is_deleted</t>
+        </is>
+      </c>
+      <c r="B23" s="36" t="n"/>
+      <c r="C23" s="36" t="n"/>
+      <c r="D23" s="36" t="n"/>
+      <c r="E23" s="36" t="n"/>
+      <c r="F23" s="36" t="n"/>
+      <c r="G23" s="36" t="n"/>
+      <c r="H23" s="36" t="n"/>
+      <c r="I23" s="36" t="n"/>
+      <c r="J23" s="36" t="n"/>
+      <c r="K23" s="37" t="n"/>
+      <c r="L23" s="46" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="47" t="inlineStr">
+        <is>
+          <t>Preconditions: SQLite in-memory DB created from Base.metadata. schema_conn fixture available.</t>
+        </is>
+      </c>
+      <c r="B24" s="36" t="n"/>
+      <c r="C24" s="36" t="n"/>
+      <c r="D24" s="36" t="n"/>
+      <c r="E24" s="36" t="n"/>
+      <c r="F24" s="36" t="n"/>
+      <c r="G24" s="36" t="n"/>
+      <c r="H24" s="36" t="n"/>
+      <c r="I24" s="36" t="n"/>
+      <c r="J24" s="36" t="n"/>
+      <c r="K24" s="37" t="n"/>
+      <c r="L24" s="47" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="48" t="inlineStr">
+        <is>
+          <t>TC-10.8 Step 1</t>
+        </is>
+      </c>
+      <c r="B25" s="48" t="inlineStr">
+        <is>
+          <t>DBSchema</t>
+        </is>
+      </c>
+      <c r="C25" s="48" t="inlineStr">
+        <is>
+          <t>10.8</t>
+        </is>
+      </c>
+      <c r="D25" s="48" t="inlineStr">
+        <is>
+          <t>Run PRAGMA table_info on participant and user tables. Assert is_deleted column has DEFAULT 0 or false. Assert SELECT COUNT(*) WHERE is_deleted IS NULL = 0.</t>
+        </is>
+      </c>
+      <c r="E25" s="48" t="inlineStr">
+        <is>
+          <t>is_deleted column has DEFAULT false on participant; no row has NULL is_deleted.</t>
+        </is>
+      </c>
+      <c r="F25" s="48" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="G25" s="48" t="inlineStr">
+        <is>
+          <t>HIPAA §164.530(j) record retention</t>
+        </is>
+      </c>
+      <c r="H25" s="48" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I25" s="48" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J25" s="48" t="n"/>
+      <c r="K25" s="48" t="n"/>
+      <c r="L25" s="48" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="A6:K6"/>
+    <mergeCell ref="A12:K12"/>
+    <mergeCell ref="A18:K18"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A20:K20"/>
+    <mergeCell ref="A21:K21"/>
+    <mergeCell ref="A23:K23"/>
+    <mergeCell ref="A15:K15"/>
+    <mergeCell ref="A24:K24"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A11:K11"/>
+    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="A9:K9"/>
+    <mergeCell ref="A8:K8"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>